<commit_message>
chore: sneaker release update [2026-09-14 12:06 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated September 13, 2026  ·  11:17 UTC</t>
+          <t>Generated September 14, 2026  ·  12:06 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46290</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46354</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46280</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>46280</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E13" s="40" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>46281</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         <v>46282</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E15" s="40" t="inlineStr">
         <is>
@@ -1927,19 +1927,19 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C16" s="31" t="n">
         <v>46283</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -1950,11 +1950,11 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>250</v>
-      </c>
-      <c r="H16" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>180</v>
+      </c>
+      <c r="H16" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
@@ -2171,7 +2171,7 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>9/13 – 9/19</t>
+          <t>9/14 – 9/20</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
@@ -2192,7 +2192,7 @@
       </c>
       <c r="B30" s="35" t="inlineStr">
         <is>
-          <t>9/20 – 9/26</t>
+          <t>9/21 – 9/27</t>
         </is>
       </c>
       <c r="C30" s="35" t="n">
@@ -2213,14 +2213,14 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>9/27 – 10/3</t>
+          <t>9/28 – 10/4</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D31" s="39" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>5.8</v>
@@ -2234,7 +2234,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>10/4 – 10/10</t>
+          <t>10/5 – 10/11</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2255,7 +2255,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>10/11 – 10/17</t>
+          <t>10/12 – 10/18</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2276,17 +2276,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>10/18 – 10/24</t>
+          <t>10/19 – 10/25</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D34" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.1</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2297,17 +2297,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>10/25 – 10/31</t>
+          <t>10/26 – 11/1</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2318,7 +2318,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>11/1 – 11/7</t>
+          <t>11/2 – 11/8</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2339,17 +2339,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>11/8 – 11/14</t>
+          <t>11/9 – 11/15</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
         <v>8</v>
       </c>
       <c r="D37" s="39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>5.6</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2360,17 +2360,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>11/15 – 11/21</t>
+          <t>11/16 – 11/22</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D38" s="40" t="n">
         <v>7</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2381,7 +2381,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>11/22 – 11/28</t>
+          <t>11/23 – 11/29</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>11/29 – 12/5</t>
+          <t>11/30 – 12/6</t>
         </is>
       </c>
       <c r="C40" s="35" t="n">
@@ -2423,7 +2423,7 @@
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>12/6 – 12/12</t>
+          <t>12/7 – 12/13</t>
         </is>
       </c>
       <c r="C41" s="30" t="n">
@@ -2718,7 +2718,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 13, 2026  ·  11:17 UTC</t>
+          <t>Generated September 14, 2026  ·  12:06 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2988,26 +2988,26 @@
         <v>46283</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D12" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -3016,7 +3016,7 @@
         <v>46283</v>
       </c>
       <c r="B13" s="41" t="n">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C13" s="40" t="inlineStr">
         <is>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Laser”</t>
+          <t>JAIDE x Air Jordan 11 Low “Fiberglass”</t>
         </is>
       </c>
     </row>
@@ -3044,11 +3044,11 @@
         <v>46283</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C14" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D14" s="34" t="inlineStr">
@@ -3058,12 +3058,12 @@
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>PSG x Nike KD 6</t>
         </is>
       </c>
     </row>
@@ -3072,7 +3072,7 @@
         <v>46283</v>
       </c>
       <c r="B15" s="41" t="n">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="C15" s="40" t="inlineStr">
         <is>
@@ -3091,7 +3091,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 11 Low “Fiberglass”</t>
+          <t>APB x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -3100,16 +3100,16 @@
         <v>46283</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>135</v>
+        <v>145</v>
       </c>
       <c r="C16" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D16" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3119,7 +3119,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>PSG x Nike KD 6</t>
+          <t>Nike A’Two “Dawn Staley”</t>
         </is>
       </c>
     </row>
@@ -3128,11 +3128,11 @@
         <v>46283</v>
       </c>
       <c r="B17" s="41" t="n">
-        <v>200</v>
-      </c>
-      <c r="C17" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>65</v>
+      </c>
+      <c r="C17" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D17" s="42" t="inlineStr">
@@ -3142,12 +3142,12 @@
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>APB x Air Jordan 11 Low</t>
+          <t>K-Pop Demon Hunters x Vans Fall 2026 Collection</t>
         </is>
       </c>
     </row>
@@ -3156,11 +3156,11 @@
         <v>46283</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -3175,7 +3175,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike A’Two “Dawn Staley”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -3184,11 +3184,11 @@
         <v>46283</v>
       </c>
       <c r="B19" s="41" t="n">
-        <v>65</v>
-      </c>
-      <c r="C19" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>210</v>
+      </c>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="42" t="inlineStr">
@@ -3198,12 +3198,12 @@
       </c>
       <c r="E19" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>K-Pop Demon Hunters x Vans Fall 2026 Collection</t>
+          <t>Nike LeBron 23 “Laser”</t>
         </is>
       </c>
     </row>
@@ -3772,26 +3772,26 @@
         <v>46291</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>160</v>
+        <v>180</v>
       </c>
       <c r="C40" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Bad Bunny x adidas Badbo 1.0 “Night Navy”</t>
+          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3800,7 @@
         <v>46291</v>
       </c>
       <c r="B41" s="41" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="C41" s="40" t="inlineStr">
         <is>
@@ -3819,7 +3819,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
     </row>
@@ -3827,17 +3827,15 @@
       <c r="A42" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B42" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C42" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B42" s="33" t="inlineStr"/>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -3847,7 +3845,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 “Light British Tan”</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
     </row>
@@ -3855,17 +3853,15 @@
       <c r="A43" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B43" s="41" t="n">
-        <v>180</v>
-      </c>
-      <c r="C43" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D43" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B43" s="41" t="inlineStr"/>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D43" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E43" s="35" t="inlineStr">
@@ -3875,7 +3871,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -3884,16 +3880,16 @@
         <v>46291</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="C44" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D44" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E44" s="30" t="inlineStr">
@@ -3903,7 +3899,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
+          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
         </is>
       </c>
     </row>
@@ -3911,15 +3907,17 @@
       <c r="A45" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B45" s="41" t="inlineStr"/>
-      <c r="C45" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B45" s="41" t="n">
+        <v>200</v>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
@@ -3929,7 +3927,7 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low Pack</t>
+          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3935,9 @@
       <c r="A46" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B46" s="33" t="inlineStr"/>
+      <c r="B46" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3950,12 +3950,12 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Air Jordan 4014 “Ferrari”</t>
         </is>
       </c>
     </row>
@@ -3963,27 +3963,25 @@
       <c r="A47" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B47" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C47" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D47" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B47" s="41" t="inlineStr"/>
+      <c r="C47" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D47" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
+          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
         </is>
       </c>
     </row>
@@ -3992,26 +3990,26 @@
         <v>46291</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C48" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D48" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>155</v>
+      </c>
+      <c r="C48" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
+          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
         </is>
       </c>
     </row>
@@ -4020,26 +4018,26 @@
         <v>46291</v>
       </c>
       <c r="B49" s="41" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D49" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D49" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4014 “Ferrari”</t>
+          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
         </is>
       </c>
     </row>
@@ -4047,10 +4045,12 @@
       <c r="A50" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B50" s="33" t="inlineStr"/>
-      <c r="C50" s="55" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B50" s="33" t="n">
+        <v>210</v>
+      </c>
+      <c r="C50" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4060,12 +4060,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
+          <t>Nike Kobe 3 Protro “Orca” 2026</t>
         </is>
       </c>
     </row>
@@ -4076,24 +4076,24 @@
       <c r="B51" s="41" t="n">
         <v>155</v>
       </c>
-      <c r="C51" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D51" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C51" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D51" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
+          <t>NOCTA x Nike KD 19</t>
         </is>
       </c>
     </row>
@@ -4102,26 +4102,26 @@
         <v>46291</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C52" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D52" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C52" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
+          <t>Bad Bunny x adidas Badbo 1.0 “Night Navy”</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4130,7 @@
         <v>46291</v>
       </c>
       <c r="B53" s="41" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
@@ -4149,7 +4149,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
         <v>46291</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="C54" s="48" t="inlineStr">
         <is>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>NOCTA x Nike KD 19</t>
+          <t>Nike SB P-Rod 1 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -4517,19 +4517,19 @@
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="B67" s="41" t="n">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C67" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D67" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D67" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E67" s="35" t="inlineStr">
@@ -4539,7 +4539,7 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Air Jordan 4 “Light Army”</t>
         </is>
       </c>
     </row>
@@ -4548,16 +4548,16 @@
         <v>46298</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C68" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -4567,43 +4567,45 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 Low “Black Ostrich”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="B69" s="41" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C69" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D69" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D69" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
+          <t>Air Jordan 14 Low “Black Ostrich”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B70" s="33" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="B70" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C70" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -4616,12 +4618,12 @@
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
         </is>
       </c>
     </row>
@@ -4629,12 +4631,10 @@
       <c r="A71" s="36" t="n">
         <v>46303</v>
       </c>
-      <c r="B71" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C71" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B71" s="41" t="inlineStr"/>
+      <c r="C71" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4644,25 +4644,25 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Marshmallow”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C72" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C72" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D72" s="43" t="inlineStr">
@@ -4672,12 +4672,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
+          <t>Vans Old Skool 36 Pearlized “Marshmallow”</t>
         </is>
       </c>
     </row>
@@ -4686,11 +4686,11 @@
         <v>46304</v>
       </c>
       <c r="B73" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C73" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C73" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D73" s="42" t="inlineStr">
@@ -4700,25 +4700,25 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
+          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C74" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C74" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4728,25 +4728,25 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Royal” 2026</t>
+          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="36" t="n">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="B75" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C75" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>180</v>
+      </c>
+      <c r="C75" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4761,7 +4761,7 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunrise”</t>
+          <t>Air Jordan 1 High OG “Royal” 2026</t>
         </is>
       </c>
     </row>
@@ -4772,42 +4772,42 @@
       <c r="B76" s="33" t="n">
         <v>125</v>
       </c>
-      <c r="C76" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D76" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C76" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Jordan Tatum 5 “Sunrise”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="36" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="B77" s="41" t="n">
-        <v>250</v>
+        <v>125</v>
       </c>
       <c r="C77" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D77" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D77" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E77" s="35" t="inlineStr">
@@ -4817,7 +4817,7 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
@@ -4826,7 +4826,7 @@
         <v>46311</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C78" s="39" t="inlineStr">
         <is>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Mummy”</t>
+          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -4873,7 +4873,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Phantom”</t>
+          <t>Nike Air Foamposite One “Mummy”</t>
         </is>
       </c>
     </row>
@@ -4882,7 +4882,7 @@
         <v>46311</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C80" s="39" t="inlineStr">
         <is>
@@ -4901,16 +4901,16 @@
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Nike Air Foamposite One “Phantom”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B81" s="41" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="C81" s="40" t="inlineStr">
         <is>
@@ -4924,12 +4924,12 @@
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -4938,7 +4938,7 @@
         <v>46312</v>
       </c>
       <c r="B82" s="33" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C82" s="39" t="inlineStr">
         <is>
@@ -4957,18 +4957,20 @@
       </c>
       <c r="F82" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Fireside”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="83" ht="15" customHeight="1">
       <c r="A83" s="36" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B83" s="41" t="inlineStr"/>
-      <c r="C83" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>46312</v>
+      </c>
+      <c r="B83" s="41" t="n">
+        <v>215</v>
+      </c>
+      <c r="C83" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D83" s="42" t="inlineStr">
@@ -4978,25 +4980,23 @@
       </c>
       <c r="E83" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>SZA x Vans VANSZA Collection</t>
+          <t>Air Jordan 12 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46319</v>
-      </c>
-      <c r="B84" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C84" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46317</v>
+      </c>
+      <c r="B84" s="33" t="inlineStr"/>
+      <c r="C84" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -5006,12 +5006,12 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>SZA x Vans VANSZA Collection</t>
         </is>
       </c>
     </row>
@@ -5020,11 +5020,11 @@
         <v>46319</v>
       </c>
       <c r="B85" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C85" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C85" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D85" s="42" t="inlineStr">
@@ -5039,7 +5039,7 @@
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Nike Ja 4 “Radar”</t>
         </is>
       </c>
     </row>
@@ -5048,11 +5048,11 @@
         <v>46319</v>
       </c>
       <c r="B86" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C86" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C86" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D86" s="43" t="inlineStr">
@@ -5062,12 +5062,12 @@
       </c>
       <c r="E86" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Radar”</t>
+          <t>Vans Old Skool 36 Pearlized “Red”</t>
         </is>
       </c>
     </row>
@@ -5076,26 +5076,26 @@
         <v>46319</v>
       </c>
       <c r="B87" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C87" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D87" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C87" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D87" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E87" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Red”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -5104,11 +5104,11 @@
         <v>46319</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C88" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C88" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D88" s="34" t="inlineStr">
@@ -5123,7 +5123,7 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
         </is>
       </c>
     </row>
@@ -5132,16 +5132,16 @@
         <v>46319</v>
       </c>
       <c r="B89" s="41" t="n">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="C89" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5151,7 +5151,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -5160,11 +5160,11 @@
         <v>46319</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C90" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C90" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D90" s="43" t="inlineStr">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -5188,7 +5188,7 @@
         <v>46319</v>
       </c>
       <c r="B91" s="41" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
@@ -5202,21 +5202,21 @@
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B92" s="33" t="n">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="C92" s="39" t="inlineStr">
         <is>
@@ -5230,40 +5230,40 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46325</v>
+        <v>46320</v>
       </c>
       <c r="B93" s="41" t="n">
-        <v>180</v>
-      </c>
-      <c r="C93" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D93" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C93" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D93" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 4 High “University Red”</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
@@ -5300,16 +5300,16 @@
         <v>46325</v>
       </c>
       <c r="B95" s="41" t="n">
-        <v>155</v>
+        <v>180</v>
       </c>
       <c r="C95" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D95" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D95" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5319,20 +5319,20 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Halloween”</t>
+          <t>Nike Ja 4 High “University Red”</t>
         </is>
       </c>
     </row>
     <row r="96" ht="15" customHeight="1">
       <c r="A96" s="31" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C96" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C96" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D96" s="43" t="inlineStr">
@@ -5342,40 +5342,40 @@
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Forest Green”</t>
+          <t>Nike Book 2 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="97" ht="15" customHeight="1">
       <c r="A97" s="36" t="n">
-        <v>46329</v>
+        <v>46326</v>
       </c>
       <c r="B97" s="41" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C97" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D97" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D97" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
+          <t>Air Jordan 14 “Forest Green”</t>
         </is>
       </c>
     </row>
@@ -5391,9 +5391,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D98" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D98" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E98" s="30" t="inlineStr">
@@ -5403,20 +5403,20 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
+          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
         </is>
       </c>
     </row>
     <row r="99" ht="15" customHeight="1">
       <c r="A99" s="36" t="n">
-        <v>46331</v>
+        <v>46329</v>
       </c>
       <c r="B99" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C99" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>240</v>
+      </c>
+      <c r="C99" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D99" s="42" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Victor Wembanyama x Nike GT Cut 4 “Statue of Liberty”</t>
+          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
         </is>
       </c>
     </row>
@@ -5459,16 +5459,16 @@
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Victor Wembanyama x Nike GT Cut 4 “State of Liberty”</t>
+          <t>Victor Wembanyama x Nike GT Cut 4 “Statue of Liberty”</t>
         </is>
       </c>
     </row>
     <row r="101" ht="15" customHeight="1">
       <c r="A101" s="36" t="n">
-        <v>46332</v>
+        <v>46331</v>
       </c>
       <c r="B101" s="41" t="n">
-        <v>145</v>
+        <v>210</v>
       </c>
       <c r="C101" s="53" t="inlineStr">
         <is>
@@ -5487,20 +5487,20 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Desert Night”</t>
+          <t>Victor Wembanyama x Nike GT Cut 4 “State of Liberty”</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="31" t="n">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C102" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C102" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D102" s="43" t="inlineStr">
@@ -5510,12 +5510,12 @@
       </c>
       <c r="E102" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Nike Book 2 “Desert Night”</t>
         </is>
       </c>
     </row>
@@ -5524,16 +5524,16 @@
         <v>46333</v>
       </c>
       <c r="B103" s="41" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C103" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D103" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D103" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E103" s="35" t="inlineStr">
@@ -5543,25 +5543,25 @@
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
     <row r="104" ht="15" customHeight="1">
       <c r="A104" s="31" t="n">
-        <v>46337</v>
+        <v>46333</v>
       </c>
       <c r="B104" s="33" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C104" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D104" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D104" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E104" s="30" t="inlineStr">
@@ -5571,7 +5571,7 @@
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Lapis”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -5580,7 +5580,7 @@
         <v>46337</v>
       </c>
       <c r="B105" s="41" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C105" s="40" t="inlineStr">
         <is>
@@ -5594,30 +5594,30 @@
       </c>
       <c r="E105" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F105" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Lapis”</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" s="31" t="n">
-        <v>46338</v>
+        <v>46337</v>
       </c>
       <c r="B106" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C106" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D106" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C106" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D106" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E106" s="30" t="inlineStr">
@@ -5627,7 +5627,7 @@
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Varsity Royal” 2026</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -5636,26 +5636,26 @@
         <v>46338</v>
       </c>
       <c r="B107" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C107" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D107" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>170</v>
+      </c>
+      <c r="C107" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D107" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E107" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F107" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Lime Pop”</t>
+          <t>Nike Air Bakin “Varsity Royal” 2026</t>
         </is>
       </c>
     </row>
@@ -5664,11 +5664,11 @@
         <v>46338</v>
       </c>
       <c r="B108" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C108" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C108" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D108" s="43" t="inlineStr">
@@ -5678,40 +5678,40 @@
       </c>
       <c r="E108" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F108" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Varsity Royal”</t>
+          <t>Vans Old Skool 36 Pearlized “Lime Pop”</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="36" t="n">
-        <v>46340</v>
+        <v>46338</v>
       </c>
       <c r="B109" s="41" t="n">
-        <v>255</v>
-      </c>
-      <c r="C109" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D109" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C109" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D109" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E109" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F109" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Nike Air Bakin “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -5720,11 +5720,11 @@
         <v>46340</v>
       </c>
       <c r="B110" s="33" t="n">
-        <v>240</v>
-      </c>
-      <c r="C110" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>255</v>
+      </c>
+      <c r="C110" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D110" s="34" t="inlineStr">
@@ -5739,7 +5739,7 @@
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -5748,11 +5748,11 @@
         <v>46340</v>
       </c>
       <c r="B111" s="41" t="n">
-        <v>220</v>
-      </c>
-      <c r="C111" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>240</v>
+      </c>
+      <c r="C111" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D111" s="38" t="inlineStr">
@@ -5767,7 +5767,7 @@
       </c>
       <c r="F111" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Light Army”</t>
+          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
         </is>
       </c>
     </row>
@@ -5907,7 +5907,7 @@
       </c>
       <c r="F116" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 Be “Legendary”</t>
+          <t>Nike Book 2 “Be Legendary”</t>
         </is>
       </c>
     </row>
@@ -5944,7 +5944,7 @@
         <v>46347</v>
       </c>
       <c r="B118" s="33" t="n">
-        <v>165</v>
+        <v>125</v>
       </c>
       <c r="C118" s="39" t="inlineStr">
         <is>
@@ -5958,12 +5958,12 @@
       </c>
       <c r="E118" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F118" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5972,11 +5972,11 @@
         <v>46347</v>
       </c>
       <c r="B119" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C119" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C119" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D119" s="42" t="inlineStr">
@@ -5991,7 +5991,7 @@
       </c>
       <c r="F119" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -6000,16 +6000,16 @@
         <v>46347</v>
       </c>
       <c r="B120" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C120" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D120" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C120" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D120" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E120" s="30" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="F120" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -6028,26 +6028,26 @@
         <v>46347</v>
       </c>
       <c r="B121" s="41" t="n">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C121" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D121" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D121" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E121" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F121" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -6056,7 +6056,7 @@
         <v>46347</v>
       </c>
       <c r="B122" s="33" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="C122" s="39" t="inlineStr">
         <is>
@@ -6070,12 +6070,12 @@
       </c>
       <c r="E122" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F122" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -6084,7 +6084,7 @@
         <v>46347</v>
       </c>
       <c r="B123" s="41" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="C123" s="40" t="inlineStr">
         <is>
@@ -6098,12 +6098,12 @@
       </c>
       <c r="E123" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F123" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -6112,7 +6112,7 @@
         <v>46353</v>
       </c>
       <c r="B124" s="33" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C124" s="39" t="inlineStr">
         <is>
@@ -6126,12 +6126,12 @@
       </c>
       <c r="E124" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F124" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -6140,11 +6140,11 @@
         <v>46353</v>
       </c>
       <c r="B125" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C125" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>240</v>
+      </c>
+      <c r="C125" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D125" s="42" t="inlineStr">
@@ -6154,25 +6154,25 @@
       </c>
       <c r="E125" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F125" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Black”</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" s="31" t="n">
-        <v>46354</v>
+        <v>46353</v>
       </c>
       <c r="B126" s="33" t="n">
-        <v>190</v>
-      </c>
-      <c r="C126" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C126" s="55" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D126" s="43" t="inlineStr">
@@ -6182,12 +6182,12 @@
       </c>
       <c r="E126" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F126" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Vans Old Skool 36 Pearlized “Black”</t>
         </is>
       </c>
     </row>
@@ -6251,12 +6251,10 @@
       <c r="A129" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B129" s="41" t="n">
-        <v>230</v>
-      </c>
-      <c r="C129" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B129" s="41" t="inlineStr"/>
+      <c r="C129" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D129" s="42" t="inlineStr">
@@ -6266,12 +6264,12 @@
       </c>
       <c r="E129" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F129" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike KD 6 “Aunt Pearl” 2026</t>
         </is>
       </c>
     </row>
@@ -6279,15 +6277,17 @@
       <c r="A130" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B130" s="33" t="inlineStr"/>
-      <c r="C130" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D130" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B130" s="33" t="n">
+        <v>130</v>
+      </c>
+      <c r="C130" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D130" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E130" s="30" t="inlineStr">
@@ -6297,7 +6297,7 @@
       </c>
       <c r="F130" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Aunt Pearl” 2026</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -6305,12 +6305,10 @@
       <c r="A131" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B131" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C131" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B131" s="41" t="inlineStr"/>
+      <c r="C131" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D131" s="38" t="inlineStr">
@@ -6320,12 +6318,12 @@
       </c>
       <c r="E131" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F131" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6333,25 +6331,27 @@
       <c r="A132" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B132" s="33" t="inlineStr"/>
-      <c r="C132" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D132" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B132" s="33" t="n">
+        <v>190</v>
+      </c>
+      <c r="C132" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D132" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E132" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F132" s="30" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -6443,9 +6443,7 @@
       <c r="A136" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B136" s="33" t="n">
-        <v>150</v>
-      </c>
+      <c r="B136" s="33" t="inlineStr"/>
       <c r="C136" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6463,7 +6461,7 @@
       </c>
       <c r="F136" s="30" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -6471,7 +6469,9 @@
       <c r="A137" s="36" t="n">
         <v>46367</v>
       </c>
-      <c r="B137" s="41" t="inlineStr"/>
+      <c r="B137" s="41" t="n">
+        <v>150</v>
+      </c>
       <c r="C137" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="F137" s="35" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6591,7 +6591,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 13, 2026  ·  11:17 UTC</t>
+          <t>Generated September 14, 2026  ·  12:06 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6749,26 +6749,26 @@
         <v>46283</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>250</v>
+        <v>180</v>
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -6777,7 +6777,7 @@
         <v>46283</v>
       </c>
       <c r="B9" s="41" t="n">
-        <v>210</v>
+        <v>205</v>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
@@ -6791,12 +6791,12 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 “Laser”</t>
+          <t>JAIDE x Air Jordan 11 Low “Fiberglass”</t>
         </is>
       </c>
     </row>
@@ -6805,16 +6805,16 @@
         <v>46283</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D10" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>APB x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -6833,7 +6833,7 @@
         <v>46283</v>
       </c>
       <c r="B11" s="41" t="n">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
@@ -6847,12 +6847,12 @@
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 11 Low “Fiberglass”</t>
+          <t>Nike Air Foamposite Pro “Green Camo” 2026</t>
         </is>
       </c>
     </row>
@@ -6861,7 +6861,7 @@
         <v>46283</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
@@ -6875,12 +6875,12 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>APB x Air Jordan 11 Low</t>
+          <t>Nike LeBron 23 “Laser”</t>
         </is>
       </c>
     </row>
@@ -7085,7 +7085,7 @@
         <v>46291</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
@@ -7104,7 +7104,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
     </row>
@@ -7112,9 +7112,7 @@
       <c r="A21" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B21" s="41" t="n">
-        <v>140</v>
-      </c>
+      <c r="B21" s="41" t="inlineStr"/>
       <c r="C21" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7132,7 +7130,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
     </row>
@@ -7158,7 +7156,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low Pack</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -7166,15 +7164,17 @@
       <c r="A23" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B23" s="41" t="inlineStr"/>
+      <c r="B23" s="41" t="n">
+        <v>210</v>
+      </c>
       <c r="C23" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -7184,7 +7184,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
         </is>
       </c>
     </row>
@@ -7193,26 +7193,26 @@
         <v>46291</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D24" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
+          <t>Air Jordan 4014 “Ferrari”</t>
         </is>
       </c>
     </row>
@@ -7221,7 +7221,7 @@
         <v>46291</v>
       </c>
       <c r="B25" s="41" t="n">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="C25" s="40" t="inlineStr">
         <is>
@@ -7240,7 +7240,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4014 “Ferrari”</t>
+          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
         </is>
       </c>
     </row>
@@ -7249,26 +7249,26 @@
         <v>46291</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C26" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
+          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
         </is>
       </c>
     </row>
@@ -7277,16 +7277,16 @@
         <v>46291</v>
       </c>
       <c r="B27" s="41" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="C27" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -7296,7 +7296,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
+          <t>Nike Kobe 3 Protro “Orca” 2026</t>
         </is>
       </c>
     </row>
@@ -7305,7 +7305,7 @@
         <v>46291</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -7324,7 +7324,7 @@
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
     </row>
@@ -7496,19 +7496,19 @@
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="36" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="B35" s="41" t="n">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C35" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D35" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D35" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E35" s="35" t="inlineStr">
@@ -7518,7 +7518,7 @@
       </c>
       <c r="F35" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Air Jordan 4 “Light Army”</t>
         </is>
       </c>
     </row>
@@ -7527,16 +7527,16 @@
         <v>46298</v>
       </c>
       <c r="B36" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C36" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D36" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D36" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E36" s="30" t="inlineStr">
@@ -7546,43 +7546,45 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 Low “Black Ostrich”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
       <c r="A37" s="36" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="B37" s="41" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C37" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D37" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E37" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F37" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
+          <t>Air Jordan 14 Low “Black Ostrich”</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46303</v>
-      </c>
-      <c r="B38" s="33" t="inlineStr"/>
+        <v>46300</v>
+      </c>
+      <c r="B38" s="33" t="n">
+        <v>200</v>
+      </c>
       <c r="C38" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7595,22 +7597,20 @@
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
       <c r="A39" s="36" t="n">
-        <v>46305</v>
-      </c>
-      <c r="B39" s="41" t="n">
-        <v>180</v>
-      </c>
+        <v>46303</v>
+      </c>
+      <c r="B39" s="41" t="inlineStr"/>
       <c r="C39" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -7628,53 +7628,53 @@
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Royal” 2026</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>125</v>
+        <v>180</v>
       </c>
       <c r="C40" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D40" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Air Jordan 1 High OG “Royal” 2026</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="36" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="B41" s="41" t="n">
-        <v>250</v>
+        <v>125</v>
       </c>
       <c r="C41" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -7684,7 +7684,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
@@ -7693,7 +7693,7 @@
         <v>46311</v>
       </c>
       <c r="B42" s="33" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C42" s="39" t="inlineStr">
         <is>
@@ -7712,7 +7712,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Mummy”</t>
+          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -7740,7 +7740,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Phantom”</t>
+          <t>Nike Air Foamposite One “Mummy”</t>
         </is>
       </c>
     </row>
@@ -7749,7 +7749,7 @@
         <v>46311</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C44" s="39" t="inlineStr">
         <is>
@@ -7768,16 +7768,16 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Nike Air Foamposite One “Phantom”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="36" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B45" s="41" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="C45" s="40" t="inlineStr">
         <is>
@@ -7791,12 +7791,12 @@
       </c>
       <c r="E45" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -7805,7 +7805,7 @@
         <v>46312</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
@@ -7824,16 +7824,16 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Fireside”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="36" t="n">
-        <v>46319</v>
+        <v>46312</v>
       </c>
       <c r="B47" s="41" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="C47" s="40" t="inlineStr">
         <is>
@@ -7852,7 +7852,7 @@
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Air Jordan 12 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -7861,16 +7861,16 @@
         <v>46319</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D48" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
@@ -7880,7 +7880,7 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -7889,16 +7889,16 @@
         <v>46319</v>
       </c>
       <c r="B49" s="41" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D49" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D49" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
@@ -7908,7 +7908,7 @@
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -7917,7 +7917,7 @@
         <v>46319</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C50" s="39" t="inlineStr">
         <is>
@@ -7931,21 +7931,21 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B51" s="41" t="n">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="C51" s="40" t="inlineStr">
         <is>
@@ -7959,21 +7959,21 @@
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46326</v>
+        <v>46320</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C52" s="39" t="inlineStr">
         <is>
@@ -7992,35 +7992,35 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Forest Green”</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="36" t="n">
-        <v>46329</v>
+        <v>46326</v>
       </c>
       <c r="B53" s="41" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D53" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
+          <t>Air Jordan 14 “Forest Green”</t>
         </is>
       </c>
     </row>
@@ -8036,9 +8036,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
@@ -8048,16 +8048,16 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
+          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46333</v>
+        <v>46329</v>
       </c>
       <c r="B55" s="41" t="n">
-        <v>215</v>
+        <v>240</v>
       </c>
       <c r="C55" s="40" t="inlineStr">
         <is>
@@ -8071,12 +8071,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
         </is>
       </c>
     </row>
@@ -8085,16 +8085,16 @@
         <v>46333</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C56" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D56" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -8104,25 +8104,25 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
     <row r="57" ht="15" customHeight="1">
       <c r="A57" s="36" t="n">
-        <v>46337</v>
+        <v>46333</v>
       </c>
       <c r="B57" s="41" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C57" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D57" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D57" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E57" s="35" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Lapis”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -8141,7 +8141,7 @@
         <v>46337</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C58" s="39" t="inlineStr">
         <is>
@@ -8155,40 +8155,40 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Lapis”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46340</v>
+        <v>46337</v>
       </c>
       <c r="B59" s="41" t="n">
-        <v>255</v>
+        <v>200</v>
       </c>
       <c r="C59" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D59" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -8197,7 +8197,7 @@
         <v>46340</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>220</v>
+        <v>255</v>
       </c>
       <c r="C60" s="39" t="inlineStr">
         <is>
@@ -8216,7 +8216,7 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Light Army”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -8281,7 +8281,7 @@
         <v>46347</v>
       </c>
       <c r="B63" s="41" t="n">
-        <v>165</v>
+        <v>125</v>
       </c>
       <c r="C63" s="40" t="inlineStr">
         <is>
@@ -8295,12 +8295,12 @@
       </c>
       <c r="E63" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -8309,16 +8309,16 @@
         <v>46347</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>125</v>
+        <v>230</v>
       </c>
       <c r="C64" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D64" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D64" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
@@ -8328,7 +8328,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -8337,26 +8337,26 @@
         <v>46347</v>
       </c>
       <c r="B65" s="41" t="n">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C65" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D65" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D65" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -8365,7 +8365,7 @@
         <v>46347</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="C66" s="39" t="inlineStr">
         <is>
@@ -8379,12 +8379,12 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -8393,7 +8393,7 @@
         <v>46347</v>
       </c>
       <c r="B67" s="41" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="C67" s="40" t="inlineStr">
         <is>
@@ -8407,12 +8407,12 @@
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -8421,7 +8421,7 @@
         <v>46353</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C68" s="39" t="inlineStr">
         <is>
@@ -8435,21 +8435,21 @@
       </c>
       <c r="E68" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46354</v>
+        <v>46353</v>
       </c>
       <c r="B69" s="41" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C69" s="40" t="inlineStr">
         <is>
@@ -8468,7 +8468,7 @@
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -8505,26 +8505,26 @@
         <v>46354</v>
       </c>
       <c r="B71" s="41" t="n">
-        <v>230</v>
+        <v>130</v>
       </c>
       <c r="C71" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D71" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D71" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -8532,12 +8532,10 @@
       <c r="A72" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B72" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C72" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B72" s="33" t="inlineStr"/>
+      <c r="C72" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D72" s="34" t="inlineStr">
@@ -8547,12 +8545,12 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -8560,25 +8558,27 @@
       <c r="A73" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B73" s="41" t="inlineStr"/>
-      <c r="C73" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D73" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B73" s="41" t="n">
+        <v>190</v>
+      </c>
+      <c r="C73" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D73" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -8614,9 +8614,7 @@
       <c r="A75" s="36" t="n">
         <v>46367</v>
       </c>
-      <c r="B75" s="41" t="n">
-        <v>150</v>
-      </c>
+      <c r="B75" s="41" t="inlineStr"/>
       <c r="C75" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8634,7 +8632,7 @@
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -8642,7 +8640,9 @@
       <c r="A76" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B76" s="33" t="inlineStr"/>
+      <c r="B76" s="33" t="n">
+        <v>150</v>
+      </c>
       <c r="C76" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8660,7 +8660,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-09-21 12:15 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$140</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated September 20, 2026  ·  10:51 UTC</t>
+          <t>Generated September 21, 2026  ·  12:15 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1621,7 +1621,7 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
@@ -1629,7 +1629,7 @@
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
@@ -1737,7 +1737,7 @@
         <v>46290</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46354</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46295</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>46290</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E13" s="40" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1871,7 +1871,7 @@
         <v>46291</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="H14" s="43" t="inlineStr">
         <is>
@@ -1893,19 +1893,19 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C15" s="36" t="n">
         <v>46291</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E15" s="40" t="inlineStr">
         <is>
@@ -1916,18 +1916,18 @@
         <v>7</v>
       </c>
       <c r="G15" s="41" t="n">
-        <v>255</v>
-      </c>
-      <c r="H15" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="H15" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>46291</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -1949,9 +1949,7 @@
       <c r="F16" s="30" t="n">
         <v>7</v>
       </c>
-      <c r="G16" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="G16" s="30" t="inlineStr"/>
       <c r="H16" s="43" t="inlineStr">
         <is>
           <t>Online + Retail</t>
@@ -2012,7 +2010,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2028,7 +2026,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2046,7 +2044,7 @@
         </is>
       </c>
       <c r="E21" s="35" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G21" s="47" t="inlineStr">
         <is>
@@ -2191,7 +2189,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>9/20 – 9/26</t>
+          <t>9/21 – 9/27</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2212,7 +2210,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>9/27 – 10/3</t>
+          <t>9/28 – 10/4</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2233,7 +2231,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>10/4 – 10/10</t>
+          <t>10/5 – 10/11</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2254,7 +2252,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>10/11 – 10/17</t>
+          <t>10/12 – 10/18</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2275,17 +2273,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>10/18 – 10/24</t>
+          <t>10/19 – 10/25</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D35" s="39" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2296,17 +2294,17 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>10/25 – 10/31</t>
+          <t>10/26 – 11/1</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D36" s="40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" s="35" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2317,7 +2315,7 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>11/1 – 11/7</t>
+          <t>11/2 – 11/8</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
@@ -2338,17 +2336,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>11/8 – 11/14</t>
+          <t>11/9 – 11/15</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D38" s="40" t="n">
         <v>4</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2359,17 +2357,17 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>11/15 – 11/21</t>
+          <t>11/16 – 11/22</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D39" s="39" t="n">
         <v>8</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2380,7 +2378,7 @@
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>11/22 – 11/28</t>
+          <t>11/23 – 11/29</t>
         </is>
       </c>
       <c r="C40" s="35" t="n">
@@ -2401,17 +2399,17 @@
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>11/29 – 12/5</t>
+          <t>11/30 – 12/6</t>
         </is>
       </c>
       <c r="C41" s="30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D41" s="39" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E41" s="30" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2422,7 +2420,7 @@
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>12/6 – 12/12</t>
+          <t>12/7 – 12/13</t>
         </is>
       </c>
       <c r="C42" s="35" t="n">
@@ -2443,7 +2441,7 @@
       </c>
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>12/13 – 12/19</t>
+          <t>12/14 – 12/20</t>
         </is>
       </c>
       <c r="C43" s="30" t="n">
@@ -2551,7 +2549,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2567,7 +2565,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2593,7 +2591,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2643,7 +2641,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5">
@@ -2732,7 +2730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F140"/>
+  <dimension ref="A1:F141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2758,7 +2756,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 20, 2026  ·  10:51 UTC</t>
+          <t>Generated September 21, 2026  ·  12:15 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -3000,26 +2998,26 @@
         <v>46290</v>
       </c>
       <c r="B11" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C11" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D11" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>225</v>
+      </c>
+      <c r="C11" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D11" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Jaws” (Deep Water)</t>
+          <t>J Balvin x Air Jordan 4 “Lemonade”</t>
         </is>
       </c>
     </row>
@@ -3028,16 +3026,16 @@
         <v>46290</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>225</v>
-      </c>
-      <c r="C12" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D12" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>205</v>
+      </c>
+      <c r="C12" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
@@ -3047,7 +3045,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>J Balvin x Air Jordan 4 “Lemonade”</t>
+          <t>Air Jordan 5 “Sunset” 2026</t>
         </is>
       </c>
     </row>
@@ -3056,11 +3054,11 @@
         <v>46290</v>
       </c>
       <c r="B13" s="41" t="n">
-        <v>205</v>
-      </c>
-      <c r="C13" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>120</v>
+      </c>
+      <c r="C13" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D13" s="42" t="inlineStr">
@@ -3070,12 +3068,12 @@
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Sunset” 2026</t>
+          <t>Billionaire Boys Club x Reebok Club C 85</t>
         </is>
       </c>
     </row>
@@ -3084,11 +3082,11 @@
         <v>46290</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C14" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>140</v>
+      </c>
+      <c r="C14" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D14" s="43" t="inlineStr">
@@ -3098,12 +3096,12 @@
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Billionaire Boys Club x Reebok Club C 85</t>
+          <t>Nike Ja 4 “Jaws” (Deep Water)</t>
         </is>
       </c>
     </row>
@@ -3196,26 +3194,26 @@
         <v>46291</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="C18" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D18" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D18" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>NOCTA x Nike KD 19</t>
+          <t>Bad Bunny x adidas Badbo 1.0 “Puerto Rican Night”</t>
         </is>
       </c>
     </row>
@@ -3224,7 +3222,7 @@
         <v>46291</v>
       </c>
       <c r="B19" s="41" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C19" s="40" t="inlineStr">
         <is>
@@ -3243,7 +3241,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
     </row>
@@ -3252,11 +3250,11 @@
         <v>46291</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>255</v>
-      </c>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>125</v>
+      </c>
+      <c r="C20" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D20" s="34" t="inlineStr">
@@ -3266,12 +3264,12 @@
       </c>
       <c r="E20" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14</t>
+          <t>Nike SB P-Rod 1 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -3280,11 +3278,11 @@
         <v>46291</v>
       </c>
       <c r="B21" s="41" t="n">
-        <v>160</v>
-      </c>
-      <c r="C21" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>140</v>
+      </c>
+      <c r="C21" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D21" s="42" t="inlineStr">
@@ -3294,12 +3292,12 @@
       </c>
       <c r="E21" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Bad Bunny x adidas Badbo 1.0 “Puerto Rican Night”</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
     </row>
@@ -3308,16 +3306,16 @@
         <v>46291</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C22" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D22" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>180</v>
+      </c>
+      <c r="C22" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D22" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3327,7 +3325,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
         </is>
       </c>
     </row>
@@ -3335,17 +3333,15 @@
       <c r="A23" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B23" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C23" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D23" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B23" s="41" t="inlineStr"/>
+      <c r="C23" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D23" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
@@ -3355,7 +3351,7 @@
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 “Light British Tan”</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
     </row>
@@ -3364,26 +3360,26 @@
         <v>46291</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D24" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D24" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -3392,11 +3388,11 @@
         <v>46291</v>
       </c>
       <c r="B25" s="41" t="n">
-        <v>180</v>
-      </c>
-      <c r="C25" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>210</v>
+      </c>
+      <c r="C25" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D25" s="38" t="inlineStr">
@@ -3411,7 +3407,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
+          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
         </is>
       </c>
     </row>
@@ -3419,15 +3415,17 @@
       <c r="A26" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B26" s="33" t="inlineStr"/>
-      <c r="C26" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D26" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B26" s="33" t="n">
+        <v>200</v>
+      </c>
+      <c r="C26" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D26" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
@@ -3437,7 +3435,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low Pack</t>
+          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
         </is>
       </c>
     </row>
@@ -3446,16 +3444,16 @@
         <v>46291</v>
       </c>
       <c r="B27" s="41" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C27" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D27" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -3465,7 +3463,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 4014 “Ferrari”</t>
         </is>
       </c>
     </row>
@@ -3474,26 +3472,26 @@
         <v>46291</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D28" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
+          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
         </is>
       </c>
     </row>
@@ -3502,11 +3500,11 @@
         <v>46291</v>
       </c>
       <c r="B29" s="41" t="n">
-        <v>200</v>
-      </c>
-      <c r="C29" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C29" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D29" s="38" t="inlineStr">
@@ -3521,7 +3519,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
+          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
         </is>
       </c>
     </row>
@@ -3529,12 +3527,10 @@
       <c r="A30" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B30" s="33" t="n">
-        <v>200</v>
-      </c>
-      <c r="C30" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B30" s="33" t="inlineStr"/>
+      <c r="C30" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D30" s="43" t="inlineStr">
@@ -3544,12 +3540,12 @@
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4014 “Ferrari”</t>
+          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
         </is>
       </c>
     </row>
@@ -3560,24 +3556,24 @@
       <c r="B31" s="41" t="n">
         <v>155</v>
       </c>
-      <c r="C31" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C31" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D31" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
+          <t>NOCTA x Nike KD 19</t>
         </is>
       </c>
     </row>
@@ -3586,16 +3582,16 @@
         <v>46291</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>150</v>
+        <v>210</v>
       </c>
       <c r="C32" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D32" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
@@ -3605,7 +3601,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
+          <t>Nike Kobe 3 Protro “Orca” 2026</t>
         </is>
       </c>
     </row>
@@ -3613,25 +3609,27 @@
       <c r="A33" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B33" s="41" t="inlineStr"/>
-      <c r="C33" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D33" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B33" s="41" t="n">
+        <v>255</v>
+      </c>
+      <c r="C33" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D33" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
+          <t>Mowalola x Air Jordan 14</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3804,7 @@
         <v>46295</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="C40" s="39" t="inlineStr">
         <is>
@@ -3825,7 +3823,7 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 1000.3 “Pure Platinum”</t>
+          <t>Union LA x Nike Dunk Low “Bamboo”</t>
         </is>
       </c>
     </row>
@@ -3834,7 +3832,7 @@
         <v>46295</v>
       </c>
       <c r="B41" s="41" t="n">
-        <v>125</v>
+        <v>210</v>
       </c>
       <c r="C41" s="40" t="inlineStr">
         <is>
@@ -3848,12 +3846,12 @@
       </c>
       <c r="E41" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Leopard”</t>
+          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -3861,15 +3859,17 @@
       <c r="A42" s="31" t="n">
         <v>46295</v>
       </c>
-      <c r="B42" s="33" t="inlineStr"/>
+      <c r="B42" s="33" t="n">
+        <v>180</v>
+      </c>
       <c r="C42" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D42" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D42" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Black Rat”</t>
+          <t>Nike Air Max 1000.3 “Pure Platinum”</t>
         </is>
       </c>
     </row>
@@ -3888,16 +3888,16 @@
         <v>46295</v>
       </c>
       <c r="B43" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C43" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D43" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>125</v>
+      </c>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D43" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E43" s="35" t="inlineStr">
@@ -3907,7 +3907,7 @@
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>MoMA x Nike Air Rift 2 Pack</t>
+          <t>Nike Air Force 1 Low “Leopard”</t>
         </is>
       </c>
     </row>
@@ -3915,9 +3915,7 @@
       <c r="A44" s="31" t="n">
         <v>46295</v>
       </c>
-      <c r="B44" s="33" t="n">
-        <v>155</v>
-      </c>
+      <c r="B44" s="33" t="inlineStr"/>
       <c r="C44" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3935,7 +3933,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Nike Air Force 1 Low “Black Rat”</t>
         </is>
       </c>
     </row>
@@ -3944,16 +3942,16 @@
         <v>46295</v>
       </c>
       <c r="B45" s="41" t="n">
-        <v>200</v>
+        <v>130</v>
       </c>
       <c r="C45" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
@@ -3963,7 +3961,7 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 “UCLA”</t>
+          <t>MoMA x Nike Air Rift 2 Pack</t>
         </is>
       </c>
     </row>
@@ -3972,16 +3970,16 @@
         <v>46295</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>135</v>
+        <v>155</v>
       </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D46" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D46" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E46" s="30" t="inlineStr">
@@ -3991,7 +3989,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Union LA x Nike Dunk Low “Bamboo”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -4000,11 +3998,11 @@
         <v>46295</v>
       </c>
       <c r="B47" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C47" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C47" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D47" s="42" t="inlineStr">
@@ -4014,12 +4012,12 @@
       </c>
       <c r="E47" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
+          <t>Nike Zoom Huarache 2K4 “UCLA”</t>
         </is>
       </c>
     </row>
@@ -4140,16 +4138,16 @@
         <v>46298</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C52" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D52" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
@@ -4159,7 +4157,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 Low “Black Ostrich”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -4168,16 +4166,16 @@
         <v>46298</v>
       </c>
       <c r="B53" s="41" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D53" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
@@ -4187,7 +4185,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Air Jordan 14 Low “Black Ostrich”</t>
         </is>
       </c>
     </row>
@@ -4394,24 +4392,24 @@
       <c r="B61" s="41" t="n">
         <v>125</v>
       </c>
-      <c r="C61" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D61" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Jordan Tatum 5 “Sunrise”</t>
         </is>
       </c>
     </row>
@@ -4422,24 +4420,24 @@
       <c r="B62" s="33" t="n">
         <v>125</v>
       </c>
-      <c r="C62" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C62" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D62" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunrise”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
@@ -4698,7 +4696,7 @@
         <v>46319</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C72" s="39" t="inlineStr">
         <is>
@@ -4717,7 +4715,7 @@
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -4740,12 +4738,12 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4754,11 +4752,11 @@
         <v>46319</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C74" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C74" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4768,12 +4766,12 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Nike Ja 4 “Radar”</t>
         </is>
       </c>
     </row>
@@ -4782,11 +4780,11 @@
         <v>46319</v>
       </c>
       <c r="B75" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C75" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C75" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4796,12 +4794,12 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Radar”</t>
+          <t>Vans Old Skool 36 Pearlized “Red”</t>
         </is>
       </c>
     </row>
@@ -4810,26 +4808,26 @@
         <v>46319</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C76" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D76" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C76" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D76" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Red”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -4838,11 +4836,11 @@
         <v>46319</v>
       </c>
       <c r="B77" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="C77" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D77" s="38" t="inlineStr">
@@ -4857,7 +4855,7 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
         </is>
       </c>
     </row>
@@ -4866,16 +4864,16 @@
         <v>46319</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="C78" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D78" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D78" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
@@ -4885,7 +4883,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4894,11 +4892,11 @@
         <v>46319</v>
       </c>
       <c r="B79" s="41" t="n">
-        <v>145</v>
-      </c>
-      <c r="C79" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C79" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4913,7 +4911,7 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -5174,16 +5172,16 @@
         <v>46333</v>
       </c>
       <c r="B89" s="41" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C89" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D89" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5193,7 +5191,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
@@ -5202,16 +5200,16 @@
         <v>46333</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>215</v>
+        <v>245</v>
       </c>
       <c r="C90" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D90" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D90" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5221,7 +5219,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Air Jordan 17 Low “Black Pack”</t>
         </is>
       </c>
     </row>
@@ -5230,7 +5228,7 @@
         <v>46333</v>
       </c>
       <c r="B91" s="41" t="n">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
@@ -5249,7 +5247,7 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 17 Low “Black Pack”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -5286,7 +5284,7 @@
         <v>46337</v>
       </c>
       <c r="B93" s="41" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C93" s="40" t="inlineStr">
         <is>
@@ -5300,12 +5298,12 @@
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -5314,7 +5312,7 @@
         <v>46337</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C94" s="39" t="inlineStr">
         <is>
@@ -5328,12 +5326,12 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Light British Tan”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -5734,7 +5732,7 @@
         <v>46347</v>
       </c>
       <c r="B109" s="41" t="n">
-        <v>215</v>
+        <v>165</v>
       </c>
       <c r="C109" s="40" t="inlineStr">
         <is>
@@ -5753,7 +5751,7 @@
       </c>
       <c r="F109" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -5762,7 +5760,7 @@
         <v>46347</v>
       </c>
       <c r="B110" s="33" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C110" s="39" t="inlineStr">
         <is>
@@ -5781,7 +5779,7 @@
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5789,10 +5787,12 @@
       <c r="A111" s="36" t="n">
         <v>46347</v>
       </c>
-      <c r="B111" s="41" t="inlineStr"/>
-      <c r="C111" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B111" s="41" t="n">
+        <v>140</v>
+      </c>
+      <c r="C111" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D111" s="42" t="inlineStr">
@@ -5802,12 +5802,12 @@
       </c>
       <c r="E111" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F111" s="35" t="inlineStr">
         <is>
-          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -5816,26 +5816,26 @@
         <v>46347</v>
       </c>
       <c r="B112" s="33" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="C112" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D112" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D112" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E112" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F112" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -5844,7 +5844,7 @@
         <v>46347</v>
       </c>
       <c r="B113" s="41" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="C113" s="40" t="inlineStr">
         <is>
@@ -5858,12 +5858,12 @@
       </c>
       <c r="E113" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F113" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -5874,9 +5874,9 @@
       <c r="B114" s="33" t="n">
         <v>140</v>
       </c>
-      <c r="C114" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C114" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D114" s="43" t="inlineStr">
@@ -5891,7 +5891,7 @@
       </c>
       <c r="F114" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -5899,27 +5899,25 @@
       <c r="A115" s="36" t="n">
         <v>46347</v>
       </c>
-      <c r="B115" s="41" t="n">
-        <v>230</v>
-      </c>
-      <c r="C115" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D115" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B115" s="41" t="inlineStr"/>
+      <c r="C115" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D115" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E115" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F115" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
         </is>
       </c>
     </row>
@@ -5928,7 +5926,7 @@
         <v>46353</v>
       </c>
       <c r="B116" s="33" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C116" s="39" t="inlineStr">
         <is>
@@ -5942,12 +5940,12 @@
       </c>
       <c r="E116" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F116" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -5956,7 +5954,7 @@
         <v>46353</v>
       </c>
       <c r="B117" s="41" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C117" s="40" t="inlineStr">
         <is>
@@ -5970,12 +5968,12 @@
       </c>
       <c r="E117" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F117" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -6011,10 +6009,12 @@
       <c r="A119" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B119" s="41" t="inlineStr"/>
-      <c r="C119" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B119" s="41" t="n">
+        <v>190</v>
+      </c>
+      <c r="C119" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D119" s="42" t="inlineStr">
@@ -6029,7 +6029,7 @@
       </c>
       <c r="F119" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Aunt Pearl” 2026</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -6037,25 +6037,27 @@
       <c r="A120" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B120" s="33" t="inlineStr"/>
-      <c r="C120" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D120" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B120" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="C120" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D120" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E120" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F120" s="30" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Caitlin 1 “Warning Code”</t>
         </is>
       </c>
     </row>
@@ -6063,9 +6065,7 @@
       <c r="A121" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B121" s="41" t="n">
-        <v>190</v>
-      </c>
+      <c r="B121" s="41" t="inlineStr"/>
       <c r="C121" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="F121" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -6092,16 +6092,16 @@
         <v>46354</v>
       </c>
       <c r="B122" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C122" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D122" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>120</v>
+      </c>
+      <c r="C122" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D122" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E122" s="30" t="inlineStr">
@@ -6111,7 +6111,7 @@
       </c>
       <c r="F122" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Warning Code”</t>
+          <t>Instant Skateboards x Nike SB Air Force 1</t>
         </is>
       </c>
     </row>
@@ -6119,15 +6119,17 @@
       <c r="A123" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B123" s="41" t="inlineStr"/>
+      <c r="B123" s="41" t="n">
+        <v>130</v>
+      </c>
       <c r="C123" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D123" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D123" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E123" s="35" t="inlineStr">
@@ -6137,7 +6139,7 @@
       </c>
       <c r="F123" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -6145,17 +6147,15 @@
       <c r="A124" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B124" s="33" t="n">
-        <v>120</v>
-      </c>
-      <c r="C124" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D124" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B124" s="33" t="inlineStr"/>
+      <c r="C124" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D124" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E124" s="30" t="inlineStr">
@@ -6165,7 +6165,7 @@
       </c>
       <c r="F124" s="30" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1</t>
+          <t>Nike KD 6 “Aunt Pearl” 2026</t>
         </is>
       </c>
     </row>
@@ -6173,12 +6173,10 @@
       <c r="A125" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B125" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C125" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B125" s="41" t="inlineStr"/>
+      <c r="C125" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D125" s="38" t="inlineStr">
@@ -6188,25 +6186,25 @@
       </c>
       <c r="E125" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F125" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" s="31" t="n">
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="B126" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C126" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C126" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D126" s="43" t="inlineStr">
@@ -6221,35 +6219,35 @@
       </c>
       <c r="F126" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Black/White”</t>
+          <t>Nike LeBron 24 “Chosen 1s”</t>
         </is>
       </c>
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="A127" s="36" t="n">
-        <v>46361</v>
+        <v>46359</v>
       </c>
       <c r="B127" s="41" t="n">
-        <v>300</v>
+        <v>170</v>
       </c>
       <c r="C127" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D127" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+      <c r="D127" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E127" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F127" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
+          <t>Nike Air Bakin “Black/White”</t>
         </is>
       </c>
     </row>
@@ -6347,9 +6345,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D131" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D131" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E131" s="35" t="inlineStr">
@@ -6359,35 +6357,35 @@
       </c>
       <c r="F131" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish</t>
+          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
         </is>
       </c>
     </row>
     <row r="132" ht="15" customHeight="1">
       <c r="A132" s="31" t="n">
-        <v>46367</v>
+        <v>46361</v>
       </c>
       <c r="B132" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C132" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D132" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>300</v>
+      </c>
+      <c r="C132" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D132" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E132" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F132" s="30" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Pharrell x adidas Adistar Jellyfish</t>
         </is>
       </c>
     </row>
@@ -6450,35 +6448,35 @@
         <v>46367</v>
       </c>
       <c r="B135" s="41" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C135" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D135" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D135" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E135" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F135" s="35" t="inlineStr">
         <is>
-          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="136" ht="15" customHeight="1">
       <c r="A136" s="31" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="B136" s="33" t="n">
-        <v>235</v>
+        <v>190</v>
       </c>
       <c r="C136" s="39" t="inlineStr">
         <is>
@@ -6492,25 +6490,25 @@
       </c>
       <c r="E136" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F136" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customHeight="1">
       <c r="A137" s="36" t="n">
-        <v>46375</v>
+        <v>46368</v>
       </c>
       <c r="B137" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C137" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>235</v>
+      </c>
+      <c r="C137" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D137" s="42" t="inlineStr">
@@ -6520,12 +6518,12 @@
       </c>
       <c r="E137" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F137" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Triple Black”</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
@@ -6613,8 +6611,36 @@
         </is>
       </c>
     </row>
+    <row r="141" ht="15" customHeight="1">
+      <c r="A141" s="36" t="n">
+        <v>46375</v>
+      </c>
+      <c r="B141" s="41" t="n">
+        <v>210</v>
+      </c>
+      <c r="C141" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D141" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E141" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F141" s="35" t="inlineStr">
+        <is>
+          <t>Nike GT Future “Triple Black”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F140"/>
+  <autoFilter ref="A3:F141"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -6629,7 +6655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F74"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6655,7 +6681,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 20, 2026  ·  10:51 UTC</t>
+          <t>Generated September 21, 2026  ·  12:15 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6757,7 +6783,7 @@
         <v>46291</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>210</v>
+        <v>200</v>
       </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
@@ -6776,7 +6802,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
     </row>
@@ -6785,26 +6811,26 @@
         <v>46291</v>
       </c>
       <c r="B7" s="41" t="n">
-        <v>255</v>
+        <v>140</v>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D7" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
     </row>
@@ -6812,9 +6838,7 @@
       <c r="A8" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B8" s="33" t="n">
-        <v>200</v>
-      </c>
+      <c r="B8" s="33" t="inlineStr"/>
       <c r="C8" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6832,7 +6856,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
     </row>
@@ -6841,26 +6865,26 @@
         <v>46291</v>
       </c>
       <c r="B9" s="41" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C9" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D9" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -6868,15 +6892,17 @@
       <c r="A10" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B10" s="33" t="inlineStr"/>
+      <c r="B10" s="33" t="n">
+        <v>210</v>
+      </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D10" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D10" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
@@ -6886,7 +6912,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low Pack</t>
+          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
         </is>
       </c>
     </row>
@@ -6895,16 +6921,16 @@
         <v>46291</v>
       </c>
       <c r="B11" s="41" t="n">
-        <v>180</v>
+        <v>200</v>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D11" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D11" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E11" s="35" t="inlineStr">
@@ -6914,7 +6940,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Air Jordan 4014 “Ferrari”</t>
         </is>
       </c>
     </row>
@@ -6923,26 +6949,26 @@
         <v>46291</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D12" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D12" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
+          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
         </is>
       </c>
     </row>
@@ -6951,26 +6977,26 @@
         <v>46291</v>
       </c>
       <c r="B13" s="41" t="n">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="C13" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4014 “Ferrari”</t>
+          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
         </is>
       </c>
     </row>
@@ -6979,7 +7005,7 @@
         <v>46291</v>
       </c>
       <c r="B14" s="33" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
@@ -6993,12 +7019,12 @@
       </c>
       <c r="E14" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
+          <t>Nike Kobe 3 Protro “Orca” 2026</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7033,7 @@
         <v>46291</v>
       </c>
       <c r="B15" s="41" t="n">
-        <v>150</v>
+        <v>255</v>
       </c>
       <c r="C15" s="40" t="inlineStr">
         <is>
@@ -7021,12 +7047,12 @@
       </c>
       <c r="E15" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
+          <t>Mowalola x Air Jordan 14</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7089,7 @@
         <v>46295</v>
       </c>
       <c r="B17" s="41" t="n">
-        <v>180</v>
+        <v>135</v>
       </c>
       <c r="C17" s="40" t="inlineStr">
         <is>
@@ -7082,7 +7108,7 @@
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 1000.3 “Pure Platinum”</t>
+          <t>Union LA x Nike Dunk Low “Bamboo”</t>
         </is>
       </c>
     </row>
@@ -7091,7 +7117,7 @@
         <v>46295</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>125</v>
+        <v>210</v>
       </c>
       <c r="C18" s="39" t="inlineStr">
         <is>
@@ -7105,12 +7131,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Leopard”</t>
+          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -7118,15 +7144,17 @@
       <c r="A19" s="36" t="n">
         <v>46295</v>
       </c>
-      <c r="B19" s="41" t="inlineStr"/>
+      <c r="B19" s="41" t="n">
+        <v>180</v>
+      </c>
       <c r="C19" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -7136,7 +7164,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Black Rat”</t>
+          <t>Nike Air Max 1000.3 “Pure Platinum”</t>
         </is>
       </c>
     </row>
@@ -7145,7 +7173,7 @@
         <v>46295</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
@@ -7164,7 +7192,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Nike Air Force 1 Low “Leopard”</t>
         </is>
       </c>
     </row>
@@ -7172,17 +7200,15 @@
       <c r="A21" s="36" t="n">
         <v>46295</v>
       </c>
-      <c r="B21" s="41" t="n">
-        <v>135</v>
-      </c>
+      <c r="B21" s="41" t="inlineStr"/>
       <c r="C21" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D21" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D21" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -7192,7 +7218,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Union LA x Nike Dunk Low “Bamboo”</t>
+          <t>Nike Air Force 1 Low “Black Rat”</t>
         </is>
       </c>
     </row>
@@ -7201,7 +7227,7 @@
         <v>46295</v>
       </c>
       <c r="B22" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C22" s="39" t="inlineStr">
         <is>
@@ -7215,12 +7241,12 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -7313,16 +7339,16 @@
         <v>46298</v>
       </c>
       <c r="B26" s="33" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C26" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D26" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
@@ -7332,7 +7358,7 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 Low “Black Ostrich”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -7341,16 +7367,16 @@
         <v>46298</v>
       </c>
       <c r="B27" s="41" t="n">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="C27" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D27" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E27" s="35" t="inlineStr">
@@ -7360,7 +7386,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Air Jordan 14 Low “Black Ostrich”</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7675,7 @@
         <v>46319</v>
       </c>
       <c r="B38" s="33" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C38" s="39" t="inlineStr">
         <is>
@@ -7668,7 +7694,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -7691,12 +7717,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -7705,26 +7731,26 @@
         <v>46319</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C40" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D40" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -7733,16 +7759,16 @@
         <v>46319</v>
       </c>
       <c r="B41" s="41" t="n">
-        <v>150</v>
+        <v>190</v>
       </c>
       <c r="C41" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D41" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E41" s="35" t="inlineStr">
@@ -7752,7 +7778,7 @@
       </c>
       <c r="F41" s="35" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -7817,16 +7843,16 @@
         <v>46333</v>
       </c>
       <c r="B44" s="33" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C44" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D44" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D44" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E44" s="30" t="inlineStr">
@@ -7836,7 +7862,7 @@
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
@@ -7845,16 +7871,16 @@
         <v>46333</v>
       </c>
       <c r="B45" s="41" t="n">
-        <v>215</v>
+        <v>245</v>
       </c>
       <c r="C45" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="35" t="inlineStr">
@@ -7864,7 +7890,7 @@
       </c>
       <c r="F45" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Air Jordan 17 Low “Black Pack”</t>
         </is>
       </c>
     </row>
@@ -7873,7 +7899,7 @@
         <v>46333</v>
       </c>
       <c r="B46" s="33" t="n">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
@@ -7892,7 +7918,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 17 Low “Black Pack”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -7929,7 +7955,7 @@
         <v>46337</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
@@ -7943,12 +7969,12 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -7957,7 +7983,7 @@
         <v>46337</v>
       </c>
       <c r="B49" s="41" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
@@ -7971,12 +7997,12 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Light British Tan”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -8097,7 +8123,7 @@
         <v>46347</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>215</v>
+        <v>165</v>
       </c>
       <c r="C54" s="39" t="inlineStr">
         <is>
@@ -8116,7 +8142,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -8125,7 +8151,7 @@
         <v>46347</v>
       </c>
       <c r="B55" s="41" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C55" s="40" t="inlineStr">
         <is>
@@ -8144,7 +8170,7 @@
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -8153,26 +8179,26 @@
         <v>46347</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="C56" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D56" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -8181,7 +8207,7 @@
         <v>46347</v>
       </c>
       <c r="B57" s="41" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="C57" s="40" t="inlineStr">
         <is>
@@ -8195,12 +8221,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -8209,16 +8235,16 @@
         <v>46347</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="C58" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D58" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
@@ -8228,7 +8254,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -8237,7 +8263,7 @@
         <v>46353</v>
       </c>
       <c r="B59" s="41" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C59" s="40" t="inlineStr">
         <is>
@@ -8251,12 +8277,12 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -8265,7 +8291,7 @@
         <v>46353</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C60" s="39" t="inlineStr">
         <is>
@@ -8279,12 +8305,12 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -8292,25 +8318,27 @@
       <c r="A61" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B61" s="41" t="inlineStr"/>
-      <c r="C61" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D61" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B61" s="41" t="n">
+        <v>190</v>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D61" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E61" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -8318,9 +8346,7 @@
       <c r="A62" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B62" s="33" t="n">
-        <v>190</v>
-      </c>
+      <c r="B62" s="33" t="inlineStr"/>
       <c r="C62" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8338,7 +8364,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -8346,15 +8372,17 @@
       <c r="A63" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B63" s="41" t="inlineStr"/>
+      <c r="B63" s="41" t="n">
+        <v>120</v>
+      </c>
       <c r="C63" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D63" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
@@ -8364,7 +8392,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Instant Skateboards x Nike SB Air Force 1</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8401,7 @@
         <v>46354</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C64" s="39" t="inlineStr">
         <is>
@@ -8392,7 +8420,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -8400,12 +8428,10 @@
       <c r="A65" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B65" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C65" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B65" s="41" t="inlineStr"/>
+      <c r="C65" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D65" s="38" t="inlineStr">
@@ -8415,20 +8441,22 @@
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="66" ht="15" customHeight="1">
       <c r="A66" s="31" t="n">
-        <v>46361</v>
-      </c>
-      <c r="B66" s="33" t="inlineStr"/>
+        <v>46357</v>
+      </c>
+      <c r="B66" s="33" t="n">
+        <v>190</v>
+      </c>
       <c r="C66" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8441,12 +8469,12 @@
       </c>
       <c r="E66" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Nike LeBron 24 “Chosen 1s”</t>
         </is>
       </c>
     </row>
@@ -8454,9 +8482,7 @@
       <c r="A67" s="36" t="n">
         <v>46361</v>
       </c>
-      <c r="B67" s="41" t="n">
-        <v>215</v>
-      </c>
+      <c r="B67" s="41" t="inlineStr"/>
       <c r="C67" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8474,25 +8500,25 @@
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46367</v>
+        <v>46361</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>150</v>
+        <v>215</v>
       </c>
       <c r="C68" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D68" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D68" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -8502,7 +8528,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
@@ -8565,35 +8591,35 @@
         <v>46367</v>
       </c>
       <c r="B71" s="41" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C71" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D71" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D71" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>235</v>
+        <v>190</v>
       </c>
       <c r="C72" s="39" t="inlineStr">
         <is>
@@ -8607,21 +8633,21 @@
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
         </is>
       </c>
     </row>
     <row r="73" ht="15" customHeight="1">
       <c r="A73" s="36" t="n">
-        <v>46375</v>
+        <v>46368</v>
       </c>
       <c r="B73" s="41" t="n">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C73" s="40" t="inlineStr">
         <is>
@@ -8640,7 +8666,7 @@
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
@@ -8649,31 +8675,59 @@
         <v>46375</v>
       </c>
       <c r="B74" s="33" t="n">
+        <v>220</v>
+      </c>
+      <c r="C74" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D74" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E74" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F74" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Pink Thunder”</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="15" customHeight="1">
+      <c r="A75" s="36" t="n">
+        <v>46375</v>
+      </c>
+      <c r="B75" s="41" t="n">
         <v>120</v>
       </c>
-      <c r="C74" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D74" s="34" t="inlineStr">
+      <c r="C75" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D75" s="38" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
       </c>
-      <c r="E74" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F74" s="30" t="inlineStr">
+      <c r="E75" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F75" s="35" t="inlineStr">
         <is>
           <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F74"/>
+  <autoFilter ref="A3:F75"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-09-22 11:09 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$143</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$75</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -679,13 +679,13 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated September 21, 2026  ·  12:15 UTC</t>
+          <t>Generated September 22, 2026  ·  11:09 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1621,11 +1621,11 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
@@ -1634,7 +1634,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$182</t>
+          <t>$181</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46290</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46354</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46295</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>46290</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E13" s="40" t="inlineStr">
         <is>
@@ -1871,7 +1871,7 @@
         <v>46291</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         <v>46291</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E15" s="40" t="inlineStr">
         <is>
@@ -1939,7 +1939,7 @@
         <v>46291</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -2010,7 +2010,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2026,7 +2026,7 @@
         </is>
       </c>
       <c r="H20" s="30" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
@@ -2062,7 +2062,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D22" s="48" t="inlineStr">
         <is>
@@ -2070,7 +2070,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G22" s="49" t="inlineStr">
         <is>
@@ -2096,7 +2096,7 @@
         </is>
       </c>
       <c r="E23" s="35" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -2189,17 +2189,17 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>9/21 – 9/27</t>
+          <t>9/22 – 9/28</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D31" s="39" t="n">
         <v>13</v>
       </c>
       <c r="E31" s="30" t="n">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2210,14 +2210,14 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>9/28 – 10/4</t>
+          <t>9/29 – 10/5</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D32" s="40" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E32" s="35" t="n">
         <v>5.9</v>
@@ -2231,17 +2231,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>10/5 – 10/11</t>
+          <t>10/6 – 10/12</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D33" s="39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>5</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2252,7 +2252,7 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>10/12 – 10/18</t>
+          <t>10/13 – 10/19</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
@@ -2273,7 +2273,7 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>10/19 – 10/25</t>
+          <t>10/20 – 10/26</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
@@ -2294,7 +2294,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>10/26 – 11/1</t>
+          <t>10/27 – 11/2</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2315,17 +2315,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>11/2 – 11/8</t>
+          <t>11/3 – 11/9</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D37" s="39" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E37" s="30" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2336,17 +2336,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>11/9 – 11/15</t>
+          <t>11/10 – 11/16</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D38" s="40" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>5.2</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2357,17 +2357,17 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>11/16 – 11/22</t>
+          <t>11/17 – 11/23</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D39" s="39" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2378,7 +2378,7 @@
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>11/23 – 11/29</t>
+          <t>11/24 – 11/30</t>
         </is>
       </c>
       <c r="C40" s="35" t="n">
@@ -2399,7 +2399,7 @@
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>11/30 – 12/6</t>
+          <t>12/1 – 12/7</t>
         </is>
       </c>
       <c r="C41" s="30" t="n">
@@ -2420,7 +2420,7 @@
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>12/7 – 12/13</t>
+          <t>12/8 – 12/14</t>
         </is>
       </c>
       <c r="C42" s="35" t="n">
@@ -2441,17 +2441,17 @@
       </c>
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>12/14 – 12/20</t>
+          <t>12/15 – 12/21</t>
         </is>
       </c>
       <c r="C43" s="30" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D43" s="39" t="n">
         <v>2</v>
       </c>
       <c r="E43" s="30" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
   </sheetData>
@@ -2549,7 +2549,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -2607,7 +2607,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="4">
@@ -2617,7 +2617,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2625,7 +2625,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2659,7 +2659,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2730,7 +2730,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F141"/>
+  <dimension ref="A1:F143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2756,7 +2756,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 21, 2026  ·  12:15 UTC</t>
+          <t>Generated September 22, 2026  ·  11:09 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2799,10 +2799,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46286</v>
+        <v>46287</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C4" s="48" t="inlineStr">
         <is>
@@ -2821,7 +2821,7 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>PSG x Nike KD 6 "Metallic Silver"</t>
+          <t>Nike GT Future “Varsity Red”</t>
         </is>
       </c>
     </row>
@@ -2830,11 +2830,11 @@
         <v>46287</v>
       </c>
       <c r="B5" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C5" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>110</v>
+      </c>
+      <c r="C5" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D5" s="42" t="inlineStr">
@@ -2844,12 +2844,12 @@
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Varsity Red”</t>
+          <t>Pokémon x adidas Superstar "Pikachu White"</t>
         </is>
       </c>
     </row>
@@ -2916,7 +2916,7 @@
       <c r="B8" s="33" t="n">
         <v>140</v>
       </c>
-      <c r="C8" s="54" t="inlineStr">
+      <c r="C8" s="53" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -2972,7 +2972,7 @@
       <c r="B10" s="33" t="n">
         <v>140</v>
       </c>
-      <c r="C10" s="54" t="inlineStr">
+      <c r="C10" s="53" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -3112,7 +3112,7 @@
       <c r="B15" s="41" t="n">
         <v>140</v>
       </c>
-      <c r="C15" s="53" t="inlineStr">
+      <c r="C15" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3168,7 +3168,7 @@
       <c r="B17" s="41" t="n">
         <v>210</v>
       </c>
-      <c r="C17" s="53" t="inlineStr">
+      <c r="C17" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3194,11 +3194,11 @@
         <v>46291</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>160</v>
-      </c>
-      <c r="C18" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>200</v>
+      </c>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D18" s="43" t="inlineStr">
@@ -3208,12 +3208,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Bad Bunny x adidas Badbo 1.0 “Puerto Rican Night”</t>
+          <t>Nike LeBron 23 Hyper Pink</t>
         </is>
       </c>
     </row>
@@ -3222,16 +3222,16 @@
         <v>46291</v>
       </c>
       <c r="B19" s="41" t="n">
-        <v>200</v>
-      </c>
-      <c r="C19" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D19" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D19" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E19" s="35" t="inlineStr">
@@ -3241,7 +3241,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 23 Hyper Pink</t>
+          <t>Nike SB P-Rod 1 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -3250,16 +3250,16 @@
         <v>46291</v>
       </c>
       <c r="B20" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C20" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D20" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="C20" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D20" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -3269,7 +3269,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 “Light British Tan”</t>
+          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
         </is>
       </c>
     </row>
@@ -3278,16 +3278,16 @@
         <v>46291</v>
       </c>
       <c r="B21" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C21" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D21" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>180</v>
+      </c>
+      <c r="C21" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D21" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E21" s="35" t="inlineStr">
@@ -3297,7 +3297,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Cracked Leather” Pack</t>
+          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
         </is>
       </c>
     </row>
@@ -3305,17 +3305,15 @@
       <c r="A22" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B22" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C22" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D22" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B22" s="33" t="inlineStr"/>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D22" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E22" s="30" t="inlineStr">
@@ -3325,7 +3323,7 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>One Piece x Nike Air Max Plus “Devil Fruits” Collection</t>
+          <t>APB x Nike Dunk Low Pack</t>
         </is>
       </c>
     </row>
@@ -3333,25 +3331,27 @@
       <c r="A23" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B23" s="41" t="inlineStr"/>
+      <c r="B23" s="41" t="n">
+        <v>180</v>
+      </c>
       <c r="C23" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D23" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D23" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E23" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F23" s="35" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low Pack</t>
+          <t>Mowalola x Air Jordan 14 Mule</t>
         </is>
       </c>
     </row>
@@ -3360,7 +3360,7 @@
         <v>46291</v>
       </c>
       <c r="B24" s="33" t="n">
-        <v>180</v>
+        <v>210</v>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
@@ -3374,12 +3374,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14 Mule</t>
+          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
         </is>
       </c>
     </row>
@@ -3388,11 +3388,11 @@
         <v>46291</v>
       </c>
       <c r="B25" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C25" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C25" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D25" s="38" t="inlineStr">
@@ -3407,7 +3407,7 @@
       </c>
       <c r="F25" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 Elite Low Protro “EYBL”</t>
+          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
         </is>
       </c>
     </row>
@@ -3418,24 +3418,24 @@
       <c r="B26" s="33" t="n">
         <v>200</v>
       </c>
-      <c r="C26" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D26" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C26" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D26" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
+          <t>Air Jordan 4014 “Ferrari”</t>
         </is>
       </c>
     </row>
@@ -3444,7 +3444,7 @@
         <v>46291</v>
       </c>
       <c r="B27" s="41" t="n">
-        <v>200</v>
+        <v>155</v>
       </c>
       <c r="C27" s="40" t="inlineStr">
         <is>
@@ -3463,7 +3463,7 @@
       </c>
       <c r="F27" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4014 “Ferrari”</t>
+          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
         </is>
       </c>
     </row>
@@ -3472,26 +3472,26 @@
         <v>46291</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D28" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D28" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Last Dance at the Garden”</t>
+          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
         </is>
       </c>
     </row>
@@ -3499,27 +3499,25 @@
       <c r="A29" s="36" t="n">
         <v>46291</v>
       </c>
-      <c r="B29" s="41" t="n">
-        <v>150</v>
-      </c>
-      <c r="C29" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D29" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B29" s="41" t="inlineStr"/>
+      <c r="C29" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D29" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Victor Victor x Nike Air Force 1 ’01 “Court Purple”</t>
+          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
         </is>
       </c>
     </row>
@@ -3527,25 +3525,27 @@
       <c r="A30" s="31" t="n">
         <v>46291</v>
       </c>
-      <c r="B30" s="33" t="inlineStr"/>
-      <c r="C30" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D30" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B30" s="33" t="n">
+        <v>155</v>
+      </c>
+      <c r="C30" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Pokemon x adidas ZX 8000 “Mewtwo”</t>
+          <t>NOCTA x Nike KD 19</t>
         </is>
       </c>
     </row>
@@ -3554,16 +3554,16 @@
         <v>46291</v>
       </c>
       <c r="B31" s="41" t="n">
-        <v>155</v>
-      </c>
-      <c r="C31" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D31" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>210</v>
+      </c>
+      <c r="C31" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D31" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
@@ -3573,7 +3573,7 @@
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>NOCTA x Nike KD 19</t>
+          <t>Nike Kobe 3 Protro “Orca” 2026</t>
         </is>
       </c>
     </row>
@@ -3582,26 +3582,26 @@
         <v>46291</v>
       </c>
       <c r="B32" s="33" t="n">
-        <v>210</v>
+        <v>255</v>
       </c>
       <c r="C32" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D32" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Protro “Orca” 2026</t>
+          <t>Mowalola x Air Jordan 14</t>
         </is>
       </c>
     </row>
@@ -3610,26 +3610,26 @@
         <v>46291</v>
       </c>
       <c r="B33" s="41" t="n">
-        <v>255</v>
-      </c>
-      <c r="C33" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D33" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>160</v>
+      </c>
+      <c r="C33" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D33" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Mowalola x Air Jordan 14</t>
+          <t>Bad Bunny x adidas Badbo 1.0 “Puerto Rican Night”</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3722,7 @@
       <c r="B37" s="41" t="n">
         <v>170</v>
       </c>
-      <c r="C37" s="53" t="inlineStr">
+      <c r="C37" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3778,7 +3778,7 @@
       <c r="B39" s="41" t="n">
         <v>170</v>
       </c>
-      <c r="C39" s="53" t="inlineStr">
+      <c r="C39" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3944,7 +3944,7 @@
       <c r="B45" s="41" t="n">
         <v>130</v>
       </c>
-      <c r="C45" s="53" t="inlineStr">
+      <c r="C45" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4000,7 +4000,7 @@
       <c r="B47" s="41" t="n">
         <v>200</v>
       </c>
-      <c r="C47" s="53" t="inlineStr">
+      <c r="C47" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4023,29 +4023,29 @@
     </row>
     <row r="48" ht="15" customHeight="1">
       <c r="A48" s="31" t="n">
-        <v>46296</v>
+        <v>46295</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C48" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D48" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>120</v>
+      </c>
+      <c r="C48" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D48" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Howard” 2026</t>
+          <t>Tom Sachs x Nike General Purpose Shoe “Demerits”</t>
         </is>
       </c>
     </row>
@@ -4054,26 +4054,26 @@
         <v>46296</v>
       </c>
       <c r="B49" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C49" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D49" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C49" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D49" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Racer Blue”</t>
+          <t>Air Jordan 1 Low OG “Howard” 2026</t>
         </is>
       </c>
     </row>
@@ -4082,11 +4082,11 @@
         <v>46296</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C50" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C50" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D50" s="43" t="inlineStr">
@@ -4101,53 +4101,53 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe Air Force 1 Low</t>
+          <t>Nike Caitlin 1 “Racer Blue”</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15" customHeight="1">
       <c r="A51" s="36" t="n">
-        <v>46297</v>
+        <v>46296</v>
       </c>
       <c r="B51" s="41" t="n">
-        <v>220</v>
+        <v>125</v>
       </c>
       <c r="C51" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D51" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Light Army”</t>
+          <t>Nike Kobe Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46298</v>
+        <v>46297</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>205</v>
+        <v>220</v>
       </c>
       <c r="C52" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D52" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D52" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E52" s="30" t="inlineStr">
@@ -4157,7 +4157,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Air Jordan 4 “Light Army”</t>
         </is>
       </c>
     </row>
@@ -4166,16 +4166,16 @@
         <v>46298</v>
       </c>
       <c r="B53" s="41" t="n">
-        <v>240</v>
+        <v>205</v>
       </c>
       <c r="C53" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D53" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E53" s="35" t="inlineStr">
@@ -4185,48 +4185,48 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 14 Low “Black Ostrich”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="54" ht="15" customHeight="1">
       <c r="A54" s="31" t="n">
-        <v>46300</v>
+        <v>46298</v>
       </c>
       <c r="B54" s="33" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C54" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D54" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D54" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
+          <t>Air Jordan 14 Low “Black Ostrich”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="36" t="n">
-        <v>46303</v>
+        <v>46300</v>
       </c>
       <c r="B55" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C55" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="42" t="inlineStr">
@@ -4236,25 +4236,25 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Marshmallow”</t>
+          <t>Nike Kobe 10 Low Protro “5 AM Flight”</t>
         </is>
       </c>
     </row>
     <row r="56" ht="15" customHeight="1">
       <c r="A56" s="31" t="n">
-        <v>46304</v>
+        <v>46303</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C56" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C56" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D56" s="43" t="inlineStr">
@@ -4264,12 +4264,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
+          <t>Vans Old Skool 36 Pearlized “Marshmallow”</t>
         </is>
       </c>
     </row>
@@ -4278,11 +4278,11 @@
         <v>46304</v>
       </c>
       <c r="B57" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C57" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>170</v>
+      </c>
+      <c r="C57" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D57" s="42" t="inlineStr">
@@ -4292,12 +4292,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
+          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
         </is>
       </c>
     </row>
@@ -4306,11 +4306,11 @@
         <v>46304</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>220</v>
-      </c>
-      <c r="C58" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D58" s="43" t="inlineStr">
@@ -4320,23 +4320,23 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>New Balance</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Aminé x New Balance 992 “Outdoor School”</t>
+          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
         </is>
       </c>
     </row>
     <row r="59" ht="15" customHeight="1">
       <c r="A59" s="36" t="n">
-        <v>46305</v>
+        <v>46304</v>
       </c>
       <c r="B59" s="41" t="n">
-        <v>135</v>
-      </c>
-      <c r="C59" s="53" t="inlineStr">
+        <v>220</v>
+      </c>
+      <c r="C59" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4348,12 +4348,12 @@
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Texas”</t>
+          <t>Aminé x New Balance 992 “Outdoor School”</t>
         </is>
       </c>
     </row>
@@ -4362,11 +4362,11 @@
         <v>46305</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>180</v>
-      </c>
-      <c r="C60" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>135</v>
+      </c>
+      <c r="C60" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D60" s="43" t="inlineStr">
@@ -4376,25 +4376,25 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Royal” 2026</t>
+          <t>Nike KD 6 “Texas”</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="36" t="n">
-        <v>46310</v>
+        <v>46305</v>
       </c>
       <c r="B61" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C61" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>180</v>
+      </c>
+      <c r="C61" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D61" s="42" t="inlineStr">
@@ -4409,7 +4409,7 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunrise”</t>
+          <t>Air Jordan 1 High OG “Royal” 2026</t>
         </is>
       </c>
     </row>
@@ -4420,42 +4420,42 @@
       <c r="B62" s="33" t="n">
         <v>125</v>
       </c>
-      <c r="C62" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D62" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D62" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Jordan Tatum 5 “Sunrise”</t>
         </is>
       </c>
     </row>
     <row r="63" ht="15" customHeight="1">
       <c r="A63" s="36" t="n">
-        <v>46311</v>
+        <v>46310</v>
       </c>
       <c r="B63" s="41" t="n">
-        <v>240</v>
+        <v>125</v>
       </c>
       <c r="C63" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D63" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D63" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
@@ -4465,7 +4465,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Mummy”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
@@ -4474,7 +4474,7 @@
         <v>46311</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C64" s="39" t="inlineStr">
         <is>
@@ -4493,7 +4493,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>Nike Air Foamposite One “Mummy”</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
         <v>46311</v>
       </c>
       <c r="B65" s="41" t="n">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="C65" s="40" t="inlineStr">
         <is>
@@ -4521,7 +4521,7 @@
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Phantom”</t>
+          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -4530,7 +4530,7 @@
         <v>46311</v>
       </c>
       <c r="B66" s="33" t="n">
-        <v>250</v>
+        <v>240</v>
       </c>
       <c r="C66" s="39" t="inlineStr">
         <is>
@@ -4549,16 +4549,16 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Nike Air Foamposite One “Phantom”</t>
         </is>
       </c>
     </row>
     <row r="67" ht="15" customHeight="1">
       <c r="A67" s="36" t="n">
-        <v>46312</v>
+        <v>46311</v>
       </c>
       <c r="B67" s="41" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
       <c r="C67" s="40" t="inlineStr">
         <is>
@@ -4572,12 +4572,12 @@
       </c>
       <c r="E67" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F67" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
         </is>
       </c>
     </row>
@@ -4586,7 +4586,7 @@
         <v>46312</v>
       </c>
       <c r="B68" s="33" t="n">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="C68" s="39" t="inlineStr">
         <is>
@@ -4605,20 +4605,20 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Fireside”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="69" ht="15" customHeight="1">
       <c r="A69" s="36" t="n">
-        <v>46315</v>
+        <v>46312</v>
       </c>
       <c r="B69" s="41" t="n">
-        <v>160</v>
-      </c>
-      <c r="C69" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>215</v>
+      </c>
+      <c r="C69" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D69" s="42" t="inlineStr">
@@ -4628,21 +4628,23 @@
       </c>
       <c r="E69" s="35" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F69" s="35" t="inlineStr">
         <is>
-          <t>Reebok Angel Reese 1 “Reese’s”</t>
+          <t>Air Jordan 12 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B70" s="33" t="inlineStr"/>
-      <c r="C70" s="54" t="inlineStr">
+        <v>46315</v>
+      </c>
+      <c r="B70" s="33" t="n">
+        <v>160</v>
+      </c>
+      <c r="C70" s="53" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -4654,25 +4656,23 @@
       </c>
       <c r="E70" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>SZA x Vans VANSZA Collection</t>
+          <t>Reebok Angel Reese 1 “Reese’s”</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="36" t="n">
-        <v>46318</v>
-      </c>
-      <c r="B71" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C71" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46317</v>
+      </c>
+      <c r="B71" s="41" t="inlineStr"/>
+      <c r="C71" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D71" s="42" t="inlineStr">
@@ -4682,21 +4682,21 @@
       </c>
       <c r="E71" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F71" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “NYC Rat”</t>
+          <t>SZA x Vans VANSZA Collection</t>
         </is>
       </c>
     </row>
     <row r="72" ht="15" customHeight="1">
       <c r="A72" s="31" t="n">
-        <v>46319</v>
+        <v>46318</v>
       </c>
       <c r="B72" s="33" t="n">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C72" s="39" t="inlineStr">
         <is>
@@ -4715,7 +4715,7 @@
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Nike Air Force 1 Low “NYC Rat”</t>
         </is>
       </c>
     </row>
@@ -4738,12 +4738,12 @@
       </c>
       <c r="E73" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F73" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -4752,11 +4752,11 @@
         <v>46319</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C74" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>125</v>
+      </c>
+      <c r="C74" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D74" s="43" t="inlineStr">
@@ -4766,12 +4766,12 @@
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Radar”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4780,11 +4780,11 @@
         <v>46319</v>
       </c>
       <c r="B75" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C75" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>140</v>
+      </c>
+      <c r="C75" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D75" s="42" t="inlineStr">
@@ -4794,12 +4794,12 @@
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Red”</t>
+          <t>Nike Ja 4 “Radar”</t>
         </is>
       </c>
     </row>
@@ -4808,26 +4808,26 @@
         <v>46319</v>
       </c>
       <c r="B76" s="33" t="n">
-        <v>150</v>
-      </c>
-      <c r="C76" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D76" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C76" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D76" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Vans Old Skool 36 Pearlized “Red”</t>
         </is>
       </c>
     </row>
@@ -4836,11 +4836,11 @@
         <v>46319</v>
       </c>
       <c r="B77" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C77" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>150</v>
+      </c>
+      <c r="C77" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D77" s="38" t="inlineStr">
@@ -4855,7 +4855,7 @@
       </c>
       <c r="F77" s="35" t="inlineStr">
         <is>
-          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -4864,16 +4864,16 @@
         <v>46319</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="C78" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D78" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D78" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E78" s="30" t="inlineStr">
@@ -4883,7 +4883,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
         </is>
       </c>
     </row>
@@ -4892,11 +4892,11 @@
         <v>46319</v>
       </c>
       <c r="B79" s="41" t="n">
-        <v>190</v>
-      </c>
-      <c r="C79" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C79" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D79" s="42" t="inlineStr">
@@ -4911,16 +4911,16 @@
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="80" ht="15" customHeight="1">
       <c r="A80" s="31" t="n">
-        <v>46320</v>
+        <v>46319</v>
       </c>
       <c r="B80" s="33" t="n">
-        <v>205</v>
+        <v>190</v>
       </c>
       <c r="C80" s="39" t="inlineStr">
         <is>
@@ -4934,25 +4934,25 @@
       </c>
       <c r="E80" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F80" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
     <row r="81" ht="15" customHeight="1">
       <c r="A81" s="36" t="n">
-        <v>46325</v>
+        <v>46320</v>
       </c>
       <c r="B81" s="41" t="n">
-        <v>155</v>
-      </c>
-      <c r="C81" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C81" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D81" s="42" t="inlineStr">
@@ -4962,12 +4962,12 @@
       </c>
       <c r="E81" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F81" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
@@ -5006,7 +5006,7 @@
       <c r="B83" s="41" t="n">
         <v>155</v>
       </c>
-      <c r="C83" s="53" t="inlineStr">
+      <c r="C83" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5023,20 +5023,20 @@
       </c>
       <c r="F83" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Halloween”</t>
+          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
         </is>
       </c>
     </row>
     <row r="84" ht="15" customHeight="1">
       <c r="A84" s="31" t="n">
-        <v>46326</v>
+        <v>46325</v>
       </c>
       <c r="B84" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C84" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C84" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D84" s="43" t="inlineStr">
@@ -5046,25 +5046,25 @@
       </c>
       <c r="E84" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F84" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Forest Green”</t>
+          <t>Nike Book 2 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="85" ht="15" customHeight="1">
       <c r="A85" s="36" t="n">
-        <v>46331</v>
+        <v>46326</v>
       </c>
       <c r="B85" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C85" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C85" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D85" s="42" t="inlineStr">
@@ -5074,12 +5074,12 @@
       </c>
       <c r="E85" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F85" s="35" t="inlineStr">
         <is>
-          <t>Victor Wembanyama x Nike GT Cut 4 “Statue of Liberty”</t>
+          <t>Air Jordan 14 “Forest Green”</t>
         </is>
       </c>
     </row>
@@ -5107,7 +5107,7 @@
       </c>
       <c r="F86" s="30" t="inlineStr">
         <is>
-          <t>Victor Wembanyama x Nike GT Cut 4 “State of Liberty”</t>
+          <t>Victor Wembanyama x Nike GT Cut 4 “Statue of Liberty”</t>
         </is>
       </c>
     </row>
@@ -5116,9 +5116,9 @@
         <v>46331</v>
       </c>
       <c r="B87" s="41" t="n">
-        <v>265</v>
-      </c>
-      <c r="C87" s="53" t="inlineStr">
+        <v>210</v>
+      </c>
+      <c r="C87" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5135,16 +5135,16 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max Foamdome “Eggplant”</t>
+          <t>Victor Wembanyama x Nike GT Cut 4 “State of Liberty”</t>
         </is>
       </c>
     </row>
     <row r="88" ht="15" customHeight="1">
       <c r="A88" s="31" t="n">
-        <v>46332</v>
+        <v>46331</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>145</v>
+        <v>265</v>
       </c>
       <c r="C88" s="48" t="inlineStr">
         <is>
@@ -5163,20 +5163,20 @@
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Desert Night”</t>
+          <t>Nike Air Max Foamdome “Eggplant”</t>
         </is>
       </c>
     </row>
     <row r="89" ht="15" customHeight="1">
       <c r="A89" s="36" t="n">
-        <v>46333</v>
+        <v>46332</v>
       </c>
       <c r="B89" s="41" t="n">
-        <v>215</v>
-      </c>
-      <c r="C89" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C89" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D89" s="42" t="inlineStr">
@@ -5186,12 +5186,12 @@
       </c>
       <c r="E89" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Nike Book 2 “Desert Night”</t>
         </is>
       </c>
     </row>
@@ -5200,16 +5200,16 @@
         <v>46333</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="C90" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D90" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D90" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5219,7 +5219,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 17 Low “Black Pack”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5228,7 @@
         <v>46333</v>
       </c>
       <c r="B91" s="41" t="n">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C91" s="40" t="inlineStr">
         <is>
@@ -5247,13 +5247,13 @@
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 17 Low “Black Pack”</t>
         </is>
       </c>
     </row>
     <row r="92" ht="15" customHeight="1">
       <c r="A92" s="31" t="n">
-        <v>46335</v>
+        <v>46333</v>
       </c>
       <c r="B92" s="33" t="n">
         <v>240</v>
@@ -5270,40 +5270,40 @@
       </c>
       <c r="E92" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
     <row r="93" ht="15" customHeight="1">
       <c r="A93" s="36" t="n">
-        <v>46337</v>
+        <v>46335</v>
       </c>
       <c r="B93" s="41" t="n">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C93" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D93" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E93" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F93" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Light British Tan”</t>
+          <t>Nike Air Foamposite Pro “Black Mummy Duck”</t>
         </is>
       </c>
     </row>
@@ -5312,7 +5312,7 @@
         <v>46337</v>
       </c>
       <c r="B94" s="33" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C94" s="39" t="inlineStr">
         <is>
@@ -5326,30 +5326,30 @@
       </c>
       <c r="E94" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F94" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Light British Tan”</t>
         </is>
       </c>
     </row>
     <row r="95" ht="15" customHeight="1">
       <c r="A95" s="36" t="n">
-        <v>46338</v>
+        <v>46337</v>
       </c>
       <c r="B95" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C95" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D95" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C95" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D95" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E95" s="35" t="inlineStr">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="F95" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Varsity Royal” 2026</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -5368,26 +5368,26 @@
         <v>46338</v>
       </c>
       <c r="B96" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C96" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D96" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>170</v>
+      </c>
+      <c r="C96" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D96" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E96" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F96" s="30" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Lime Pop”</t>
+          <t>Nike Air Bakin “Varsity Royal” 2026</t>
         </is>
       </c>
     </row>
@@ -5396,11 +5396,11 @@
         <v>46338</v>
       </c>
       <c r="B97" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C97" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C97" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D97" s="42" t="inlineStr">
@@ -5410,18 +5410,18 @@
       </c>
       <c r="E97" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Varsity Royal”</t>
+          <t>Vans Old Skool 36 Pearlized “Lime Pop”</t>
         </is>
       </c>
     </row>
     <row r="98" ht="15" customHeight="1">
       <c r="A98" s="31" t="n">
-        <v>46339</v>
+        <v>46338</v>
       </c>
       <c r="B98" s="33" t="n">
         <v>170</v>
@@ -5443,7 +5443,7 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 Patent “Black Red”</t>
+          <t>Nike Air Bakin “Varsity Royal”</t>
         </is>
       </c>
     </row>
@@ -5454,7 +5454,7 @@
       <c r="B99" s="41" t="n">
         <v>170</v>
       </c>
-      <c r="C99" s="53" t="inlineStr">
+      <c r="C99" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5471,35 +5471,35 @@
       </c>
       <c r="F99" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2</t>
+          <t>Nike Air Diamond Turf 2 Patent “Black Red”</t>
         </is>
       </c>
     </row>
     <row r="100" ht="15" customHeight="1">
       <c r="A100" s="31" t="n">
-        <v>46340</v>
+        <v>46339</v>
       </c>
       <c r="B100" s="33" t="n">
-        <v>255</v>
-      </c>
-      <c r="C100" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D100" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C100" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D100" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E100" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Nike Air Diamond Turf 2</t>
         </is>
       </c>
     </row>
@@ -5508,11 +5508,11 @@
         <v>46340</v>
       </c>
       <c r="B101" s="41" t="n">
-        <v>240</v>
-      </c>
-      <c r="C101" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>255</v>
+      </c>
+      <c r="C101" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D101" s="38" t="inlineStr">
@@ -5527,16 +5527,16 @@
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
     <row r="102" ht="15" customHeight="1">
       <c r="A102" s="31" t="n">
-        <v>46341</v>
+        <v>46340</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>155</v>
+        <v>240</v>
       </c>
       <c r="C102" s="48" t="inlineStr">
         <is>
@@ -5550,25 +5550,25 @@
       </c>
       <c r="E102" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Playa Society x Nike A’Two</t>
+          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
         </is>
       </c>
     </row>
     <row r="103" ht="15" customHeight="1">
       <c r="A103" s="36" t="n">
-        <v>46342</v>
+        <v>46341</v>
       </c>
       <c r="B103" s="41" t="n">
-        <v>255</v>
-      </c>
-      <c r="C103" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C103" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D103" s="38" t="inlineStr">
@@ -5578,12 +5578,12 @@
       </c>
       <c r="E103" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam Galaxy”</t>
+          <t>Playa Society x Nike A’Two</t>
         </is>
       </c>
     </row>
@@ -5592,35 +5592,35 @@
         <v>46342</v>
       </c>
       <c r="B104" s="33" t="n">
-        <v>230</v>
+        <v>255</v>
       </c>
       <c r="C104" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D104" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D104" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E104" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
+          <t>Air Jordan 11 “Space Jam Galaxy”</t>
         </is>
       </c>
     </row>
     <row r="105" ht="15" customHeight="1">
       <c r="A105" s="36" t="n">
-        <v>46343</v>
+        <v>46342</v>
       </c>
       <c r="B105" s="41" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="C105" s="40" t="inlineStr">
         <is>
@@ -5639,20 +5639,20 @@
       </c>
       <c r="F105" s="35" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Shooting Star”</t>
+          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
         </is>
       </c>
     </row>
     <row r="106" ht="15" customHeight="1">
       <c r="A106" s="31" t="n">
-        <v>46345</v>
+        <v>46343</v>
       </c>
       <c r="B106" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C106" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>200</v>
+      </c>
+      <c r="C106" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D106" s="43" t="inlineStr">
@@ -5662,25 +5662,25 @@
       </c>
       <c r="E106" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Navy”</t>
+          <t>Nike LeBron 24 “Shooting Star”</t>
         </is>
       </c>
     </row>
     <row r="107" ht="15" customHeight="1">
       <c r="A107" s="36" t="n">
-        <v>46346</v>
+        <v>46345</v>
       </c>
       <c r="B107" s="41" t="n">
-        <v>145</v>
-      </c>
-      <c r="C107" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C107" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D107" s="42" t="inlineStr">
@@ -5690,12 +5690,12 @@
       </c>
       <c r="E107" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F107" s="35" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Be Legendary”</t>
+          <t>Vans Old Skool 36 Pearlized “Navy”</t>
         </is>
       </c>
     </row>
@@ -5704,11 +5704,11 @@
         <v>46346</v>
       </c>
       <c r="B108" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C108" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>145</v>
+      </c>
+      <c r="C108" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D108" s="43" t="inlineStr">
@@ -5718,25 +5718,25 @@
       </c>
       <c r="E108" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F108" s="30" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 3 “Lucid Pink”</t>
+          <t>Nike Book 2 “Be Legendary”</t>
         </is>
       </c>
     </row>
     <row r="109" ht="15" customHeight="1">
       <c r="A109" s="36" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="B109" s="41" t="n">
-        <v>165</v>
-      </c>
-      <c r="C109" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C109" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D109" s="42" t="inlineStr">
@@ -5746,12 +5746,12 @@
       </c>
       <c r="E109" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F109" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>adidas Anthony Edwards 3 “Lucid Pink”</t>
         </is>
       </c>
     </row>
@@ -5760,7 +5760,7 @@
         <v>46347</v>
       </c>
       <c r="B110" s="33" t="n">
-        <v>125</v>
+        <v>165</v>
       </c>
       <c r="C110" s="39" t="inlineStr">
         <is>
@@ -5774,12 +5774,12 @@
       </c>
       <c r="E110" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -5788,11 +5788,11 @@
         <v>46347</v>
       </c>
       <c r="B111" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C111" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>125</v>
+      </c>
+      <c r="C111" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D111" s="42" t="inlineStr">
@@ -5807,7 +5807,7 @@
       </c>
       <c r="F111" s="35" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5816,16 +5816,16 @@
         <v>46347</v>
       </c>
       <c r="B112" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C112" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D112" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="C112" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D112" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E112" s="30" t="inlineStr">
@@ -5835,7 +5835,7 @@
       </c>
       <c r="F112" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -5844,26 +5844,26 @@
         <v>46347</v>
       </c>
       <c r="B113" s="41" t="n">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="C113" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D113" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D113" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E113" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F113" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -5872,7 +5872,7 @@
         <v>46347</v>
       </c>
       <c r="B114" s="33" t="n">
-        <v>140</v>
+        <v>215</v>
       </c>
       <c r="C114" s="39" t="inlineStr">
         <is>
@@ -5886,12 +5886,12 @@
       </c>
       <c r="E114" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F114" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -5899,10 +5899,12 @@
       <c r="A115" s="36" t="n">
         <v>46347</v>
       </c>
-      <c r="B115" s="41" t="inlineStr"/>
-      <c r="C115" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B115" s="41" t="n">
+        <v>140</v>
+      </c>
+      <c r="C115" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D115" s="42" t="inlineStr">
@@ -5912,25 +5914,23 @@
       </c>
       <c r="E115" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F115" s="35" t="inlineStr">
         <is>
-          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
     <row r="116" ht="15" customHeight="1">
       <c r="A116" s="31" t="n">
-        <v>46353</v>
-      </c>
-      <c r="B116" s="33" t="n">
-        <v>230</v>
-      </c>
-      <c r="C116" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46347</v>
+      </c>
+      <c r="B116" s="33" t="inlineStr"/>
+      <c r="C116" s="53" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D116" s="43" t="inlineStr">
@@ -5940,12 +5940,12 @@
       </c>
       <c r="E116" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F116" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
         </is>
       </c>
     </row>
@@ -5954,7 +5954,7 @@
         <v>46353</v>
       </c>
       <c r="B117" s="41" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C117" s="40" t="inlineStr">
         <is>
@@ -5968,12 +5968,12 @@
       </c>
       <c r="E117" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F117" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -5982,11 +5982,11 @@
         <v>46353</v>
       </c>
       <c r="B118" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C118" s="54" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>240</v>
+      </c>
+      <c r="C118" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D118" s="43" t="inlineStr">
@@ -5996,25 +5996,25 @@
       </c>
       <c r="E118" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F118" s="30" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Black”</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
     <row r="119" ht="15" customHeight="1">
       <c r="A119" s="36" t="n">
-        <v>46354</v>
+        <v>46353</v>
       </c>
       <c r="B119" s="41" t="n">
-        <v>190</v>
-      </c>
-      <c r="C119" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C119" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D119" s="42" t="inlineStr">
@@ -6024,12 +6024,12 @@
       </c>
       <c r="E119" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F119" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Vans Old Skool 36 Pearlized “Black”</t>
         </is>
       </c>
     </row>
@@ -6197,7 +6197,7 @@
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" s="31" t="n">
-        <v>46357</v>
+        <v>46354</v>
       </c>
       <c r="B126" s="33" t="n">
         <v>190</v>
@@ -6219,20 +6219,20 @@
       </c>
       <c r="F126" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Chosen 1s”</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
     <row r="127" ht="15" customHeight="1">
       <c r="A127" s="36" t="n">
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="B127" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C127" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C127" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D127" s="42" t="inlineStr">
@@ -6247,18 +6247,20 @@
       </c>
       <c r="F127" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Black/White”</t>
+          <t>Nike LeBron 24 “Chosen 1s”</t>
         </is>
       </c>
     </row>
     <row r="128" ht="15" customHeight="1">
       <c r="A128" s="31" t="n">
-        <v>46361</v>
-      </c>
-      <c r="B128" s="33" t="inlineStr"/>
-      <c r="C128" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>46359</v>
+      </c>
+      <c r="B128" s="33" t="n">
+        <v>170</v>
+      </c>
+      <c r="C128" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D128" s="43" t="inlineStr">
@@ -6268,12 +6270,12 @@
       </c>
       <c r="E128" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F128" s="30" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Nike Air Bakin “Black/White”</t>
         </is>
       </c>
     </row>
@@ -6281,9 +6283,7 @@
       <c r="A129" s="36" t="n">
         <v>46361</v>
       </c>
-      <c r="B129" s="41" t="n">
-        <v>215</v>
-      </c>
+      <c r="B129" s="41" t="inlineStr"/>
       <c r="C129" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="F129" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
@@ -6310,11 +6310,11 @@
         <v>46361</v>
       </c>
       <c r="B130" s="33" t="n">
-        <v>300</v>
-      </c>
-      <c r="C130" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C130" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D130" s="43" t="inlineStr">
@@ -6324,12 +6324,12 @@
       </c>
       <c r="E130" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F130" s="30" t="inlineStr">
         <is>
-          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
@@ -6340,14 +6340,14 @@
       <c r="B131" s="41" t="n">
         <v>300</v>
       </c>
-      <c r="C131" s="53" t="inlineStr">
+      <c r="C131" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D131" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+      <c r="D131" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E131" s="35" t="inlineStr">
@@ -6357,7 +6357,7 @@
       </c>
       <c r="F131" s="35" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
+          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
         </is>
       </c>
     </row>
@@ -6373,9 +6373,9 @@
           <t>MED</t>
         </is>
       </c>
-      <c r="D132" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D132" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E132" s="30" t="inlineStr">
@@ -6385,20 +6385,20 @@
       </c>
       <c r="F132" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish</t>
+          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
         </is>
       </c>
     </row>
     <row r="133" ht="15" customHeight="1">
       <c r="A133" s="36" t="n">
-        <v>46367</v>
+        <v>46361</v>
       </c>
       <c r="B133" s="41" t="n">
-        <v>240</v>
-      </c>
-      <c r="C133" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>300</v>
+      </c>
+      <c r="C133" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D133" s="42" t="inlineStr">
@@ -6408,12 +6408,12 @@
       </c>
       <c r="E133" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F133" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>Pharrell x adidas Adistar Jellyfish</t>
         </is>
       </c>
     </row>
@@ -6421,25 +6421,27 @@
       <c r="A134" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B134" s="33" t="inlineStr"/>
+      <c r="B134" s="33" t="n">
+        <v>240</v>
+      </c>
       <c r="C134" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D134" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D134" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E134" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F134" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -6447,9 +6449,7 @@
       <c r="A135" s="36" t="n">
         <v>46367</v>
       </c>
-      <c r="B135" s="41" t="n">
-        <v>150</v>
-      </c>
+      <c r="B135" s="41" t="inlineStr"/>
       <c r="C135" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6467,7 +6467,7 @@
       </c>
       <c r="F135" s="35" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -6476,35 +6476,35 @@
         <v>46367</v>
       </c>
       <c r="B136" s="33" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C136" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D136" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D136" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E136" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F136" s="30" t="inlineStr">
         <is>
-          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="137" ht="15" customHeight="1">
       <c r="A137" s="36" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="B137" s="41" t="n">
-        <v>235</v>
+        <v>190</v>
       </c>
       <c r="C137" s="40" t="inlineStr">
         <is>
@@ -6518,21 +6518,21 @@
       </c>
       <c r="E137" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F137" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
         </is>
       </c>
     </row>
     <row r="138" ht="15" customHeight="1">
       <c r="A138" s="31" t="n">
-        <v>46375</v>
+        <v>46368</v>
       </c>
       <c r="B138" s="33" t="n">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C138" s="39" t="inlineStr">
         <is>
@@ -6551,7 +6551,7 @@
       </c>
       <c r="F138" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       <c r="B141" s="41" t="n">
         <v>210</v>
       </c>
-      <c r="C141" s="53" t="inlineStr">
+      <c r="C141" s="54" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -6639,8 +6639,64 @@
         </is>
       </c>
     </row>
+    <row r="142" ht="15" customHeight="1">
+      <c r="A142" s="31" t="n">
+        <v>46375</v>
+      </c>
+      <c r="B142" s="33" t="n">
+        <v>220</v>
+      </c>
+      <c r="C142" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D142" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E142" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F142" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Pink Thunder”</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="15" customHeight="1">
+      <c r="A143" s="36" t="n">
+        <v>46377</v>
+      </c>
+      <c r="B143" s="41" t="n">
+        <v>140</v>
+      </c>
+      <c r="C143" s="54" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D143" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E143" s="35" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F143" s="35" t="inlineStr">
+        <is>
+          <t>Nike Caitlin 1 “Chiefs”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F141"/>
+  <autoFilter ref="A3:F143"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -6681,7 +6737,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 21, 2026  ·  12:15 UTC</t>
+          <t>Generated September 22, 2026  ·  11:09 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -8318,9 +8374,7 @@
       <c r="A61" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B61" s="41" t="n">
-        <v>190</v>
-      </c>
+      <c r="B61" s="41" t="inlineStr"/>
       <c r="C61" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8338,7 +8392,7 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -8346,15 +8400,17 @@
       <c r="A62" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B62" s="33" t="inlineStr"/>
+      <c r="B62" s="33" t="n">
+        <v>120</v>
+      </c>
       <c r="C62" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D62" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D62" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E62" s="30" t="inlineStr">
@@ -8364,7 +8420,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Instant Skateboards x Nike SB Air Force 1</t>
         </is>
       </c>
     </row>
@@ -8373,7 +8429,7 @@
         <v>46354</v>
       </c>
       <c r="B63" s="41" t="n">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="C63" s="40" t="inlineStr">
         <is>
@@ -8392,7 +8448,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -8400,12 +8456,10 @@
       <c r="A64" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B64" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C64" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B64" s="33" t="inlineStr"/>
+      <c r="C64" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D64" s="34" t="inlineStr">
@@ -8415,12 +8469,12 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -8428,25 +8482,27 @@
       <c r="A65" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B65" s="41" t="inlineStr"/>
-      <c r="C65" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D65" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B65" s="41" t="n">
+        <v>190</v>
+      </c>
+      <c r="C65" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D65" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -8675,26 +8731,26 @@
         <v>46375</v>
       </c>
       <c r="B74" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C74" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D74" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D74" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E74" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
         </is>
       </c>
     </row>
@@ -8703,26 +8759,26 @@
         <v>46375</v>
       </c>
       <c r="B75" s="41" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C75" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D75" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D75" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E75" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F75" s="35" t="inlineStr">
         <is>
-          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
+          <t>Air Jordan 4 “Pink Thunder”</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-09-28 13:11 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated September 27, 2026  ·  11:37 UTC</t>
+          <t>Generated September 28, 2026  ·  13:11 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1634,7 +1634,7 @@
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$181</t>
+          <t>$180</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46297</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         <v>46354</v>
       </c>
       <c r="D11" s="35" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E11" s="37" t="inlineStr">
         <is>
@@ -1803,7 +1803,7 @@
         <v>46295</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
@@ -1837,7 +1837,7 @@
         <v>46382</v>
       </c>
       <c r="D13" s="35" t="n">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E13" s="40" t="inlineStr">
         <is>
@@ -1859,19 +1859,19 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C14" s="31" t="n">
         <v>46295</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1882,7 +1882,7 @@
         <v>7</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>155</v>
+        <v>210</v>
       </c>
       <c r="H14" s="42" t="inlineStr">
         <is>
@@ -1893,19 +1893,19 @@
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
+          <t>Nike Air Force 1 Low “Leopard”</t>
         </is>
       </c>
       <c r="B15" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C15" s="36" t="n">
         <v>46295</v>
       </c>
       <c r="D15" s="35" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="40" t="inlineStr">
         <is>
@@ -1916,7 +1916,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="41" t="n">
-        <v>210</v>
+        <v>125</v>
       </c>
       <c r="H15" s="43" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Leopard”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>46295</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
         <v>7</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="H16" s="42" t="inlineStr">
         <is>
@@ -2191,7 +2191,7 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>9/27 – 10/3</t>
+          <t>9/28 – 10/4</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="B32" s="35" t="inlineStr">
         <is>
-          <t>10/4 – 10/10</t>
+          <t>10/5 – 10/11</t>
         </is>
       </c>
       <c r="C32" s="35" t="n">
@@ -2233,7 +2233,7 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>10/11 – 10/17</t>
+          <t>10/12 – 10/18</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
@@ -2254,17 +2254,17 @@
       </c>
       <c r="B34" s="35" t="inlineStr">
         <is>
-          <t>10/18 – 10/24</t>
+          <t>10/19 – 10/25</t>
         </is>
       </c>
       <c r="C34" s="35" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D34" s="40" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E34" s="35" t="n">
-        <v>5.1</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>10/25 – 10/31</t>
+          <t>10/26 – 11/1</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D35" s="39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>5.2</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B36" s="35" t="inlineStr">
         <is>
-          <t>11/1 – 11/7</t>
+          <t>11/2 – 11/8</t>
         </is>
       </c>
       <c r="C36" s="35" t="n">
@@ -2317,11 +2317,11 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>11/8 – 11/14</t>
+          <t>11/9 – 11/15</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D37" s="39" t="n">
         <v>5</v>
@@ -2338,17 +2338,17 @@
       </c>
       <c r="B38" s="35" t="inlineStr">
         <is>
-          <t>11/15 – 11/21</t>
+          <t>11/16 – 11/22</t>
         </is>
       </c>
       <c r="C38" s="35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D38" s="40" t="n">
         <v>9</v>
       </c>
       <c r="E38" s="35" t="n">
-        <v>5.6</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>11/22 – 11/28</t>
+          <t>11/23 – 11/29</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
@@ -2380,7 +2380,7 @@
       </c>
       <c r="B40" s="35" t="inlineStr">
         <is>
-          <t>11/29 – 12/5</t>
+          <t>11/30 – 12/6</t>
         </is>
       </c>
       <c r="C40" s="35" t="n">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>12/6 – 12/12</t>
+          <t>12/7 – 12/13</t>
         </is>
       </c>
       <c r="C41" s="30" t="n">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B42" s="35" t="inlineStr">
         <is>
-          <t>12/13 – 12/19</t>
+          <t>12/14 – 12/20</t>
         </is>
       </c>
       <c r="C42" s="35" t="n">
@@ -2443,7 +2443,7 @@
       </c>
       <c r="B43" s="30" t="inlineStr">
         <is>
-          <t>12/20 – 12/26</t>
+          <t>12/21 – 12/27</t>
         </is>
       </c>
       <c r="C43" s="30" t="n">
@@ -2758,7 +2758,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 27, 2026  ·  11:37 UTC</t>
+          <t>Generated September 28, 2026  ·  13:11 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2830,7 +2830,7 @@
         <v>46294</v>
       </c>
       <c r="B5" s="41" t="n">
-        <v>249</v>
+        <v>170</v>
       </c>
       <c r="C5" s="53" t="inlineStr">
         <is>
@@ -2849,7 +2849,7 @@
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Hyperice x Nike Air Zoom Hyperslide</t>
+          <t>Nike Air Bakin OG “Varsity Red” 2026</t>
         </is>
       </c>
     </row>
@@ -2858,7 +2858,7 @@
         <v>46294</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>170</v>
+        <v>249</v>
       </c>
       <c r="C6" s="48" t="inlineStr">
         <is>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Bakin OG “Varsity Red” 2026</t>
+          <t>Hyperice x Nike Air Zoom Hyperslide</t>
         </is>
       </c>
     </row>
@@ -2914,11 +2914,11 @@
         <v>46295</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C8" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>135</v>
+      </c>
+      <c r="C8" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D8" s="34" t="inlineStr">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>MoMA x Nike Air Rift 2 Pack</t>
+          <t>Union LA x Nike Dunk Low “Bamboo”</t>
         </is>
       </c>
     </row>
@@ -2942,11 +2942,11 @@
         <v>46295</v>
       </c>
       <c r="B9" s="41" t="n">
-        <v>200</v>
-      </c>
-      <c r="C9" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>210</v>
+      </c>
+      <c r="C9" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D9" s="43" t="inlineStr">
@@ -2956,12 +2956,12 @@
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Huarache 2K4 “UCLA”</t>
+          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -2970,7 +2970,7 @@
         <v>46295</v>
       </c>
       <c r="B10" s="33" t="n">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
@@ -2989,7 +2989,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Nike Air Force 1 Low “Leopard”</t>
         </is>
       </c>
     </row>
@@ -2998,11 +2998,11 @@
         <v>46295</v>
       </c>
       <c r="B11" s="41" t="n">
-        <v>135</v>
-      </c>
-      <c r="C11" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C11" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D11" s="38" t="inlineStr">
@@ -3017,7 +3017,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Union LA x Nike Dunk Low “Bamboo”</t>
+          <t>MoMA x Nike Air Rift 2 Pack</t>
         </is>
       </c>
     </row>
@@ -3026,7 +3026,7 @@
         <v>46295</v>
       </c>
       <c r="B12" s="33" t="n">
-        <v>210</v>
+        <v>155</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
@@ -3040,12 +3040,12 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -3054,11 +3054,11 @@
         <v>46295</v>
       </c>
       <c r="B13" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C13" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>200</v>
+      </c>
+      <c r="C13" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D13" s="43" t="inlineStr">
@@ -3073,7 +3073,7 @@
       </c>
       <c r="F13" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Leopard”</t>
+          <t>Nike Zoom Huarache 2K4 “UCLA”</t>
         </is>
       </c>
     </row>
@@ -3110,11 +3110,11 @@
         <v>46296</v>
       </c>
       <c r="B15" s="41" t="n">
-        <v>120</v>
-      </c>
-      <c r="C15" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>90</v>
+      </c>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D15" s="43" t="inlineStr">
@@ -3129,7 +3129,7 @@
       </c>
       <c r="F15" s="35" t="inlineStr">
         <is>
-          <t>Nike Dunk Low “Campfire Orange”</t>
+          <t>Nike Twelve Time “White”</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
         <v>46296</v>
       </c>
       <c r="B16" s="33" t="n">
-        <v>90</v>
+        <v>145</v>
       </c>
       <c r="C16" s="48" t="inlineStr">
         <is>
@@ -3157,7 +3157,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Twelve Time “White”</t>
+          <t>Nike A’Two “White Pink Spell”</t>
         </is>
       </c>
     </row>
@@ -3166,26 +3166,26 @@
         <v>46296</v>
       </c>
       <c r="B17" s="41" t="n">
-        <v>145</v>
-      </c>
-      <c r="C17" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D17" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>155</v>
+      </c>
+      <c r="C17" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E17" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="35" t="inlineStr">
         <is>
-          <t>Nike A’Two “White Pink Spell”</t>
+          <t>Air Jordan 1 Low OG “Howard” 2026</t>
         </is>
       </c>
     </row>
@@ -3194,26 +3194,26 @@
         <v>46296</v>
       </c>
       <c r="B18" s="33" t="n">
-        <v>155</v>
-      </c>
-      <c r="C18" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D18" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="C18" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D18" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Howard” 2026</t>
+          <t>Nike Caitlin 1 “Racer Blue”</t>
         </is>
       </c>
     </row>
@@ -3221,12 +3221,10 @@
       <c r="A19" s="36" t="n">
         <v>46296</v>
       </c>
-      <c r="B19" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C19" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B19" s="41" t="inlineStr"/>
+      <c r="C19" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D19" s="43" t="inlineStr">
@@ -3241,7 +3239,7 @@
       </c>
       <c r="F19" s="35" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Racer Blue”</t>
+          <t>Nike Air Max 95 “Liverpool”</t>
         </is>
       </c>
     </row>
@@ -3249,7 +3247,9 @@
       <c r="A20" s="31" t="n">
         <v>46296</v>
       </c>
-      <c r="B20" s="33" t="inlineStr"/>
+      <c r="B20" s="33" t="n">
+        <v>125</v>
+      </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -3267,7 +3267,7 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Liverpool”</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “Black Purple Stardust”</t>
         </is>
       </c>
     </row>
@@ -3276,7 +3276,7 @@
         <v>46296</v>
       </c>
       <c r="B21" s="41" t="n">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="C21" s="40" t="inlineStr">
         <is>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="F21" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Black Purple Stardust”</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “5 Rings”</t>
         </is>
       </c>
     </row>
@@ -3866,24 +3866,24 @@
       <c r="B42" s="33" t="n">
         <v>125</v>
       </c>
-      <c r="C42" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D42" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C42" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Jordan Tatum 5 “Sunrise”</t>
         </is>
       </c>
     </row>
@@ -3894,24 +3894,24 @@
       <c r="B43" s="41" t="n">
         <v>125</v>
       </c>
-      <c r="C43" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D43" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C43" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D43" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E43" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F43" s="35" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunrise”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
@@ -4114,11 +4114,11 @@
         <v>46318</v>
       </c>
       <c r="B51" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C51" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C51" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="43" t="inlineStr">
@@ -4133,7 +4133,7 @@
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “NYC Rat”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4161,7 +4161,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Nike Sabrina 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4170,11 +4170,11 @@
         <v>46318</v>
       </c>
       <c r="B53" s="41" t="n">
-        <v>145</v>
-      </c>
-      <c r="C53" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>140</v>
+      </c>
+      <c r="C53" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D53" s="43" t="inlineStr">
@@ -4189,7 +4189,7 @@
       </c>
       <c r="F53" s="35" t="inlineStr">
         <is>
-          <t>Nike Sabrina 4 “Halloween”</t>
+          <t>Nike Air Force 1 Low “NYC Rat”</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4226,7 @@
         <v>46319</v>
       </c>
       <c r="B55" s="41" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C55" s="40" t="inlineStr">
         <is>
@@ -4240,12 +4240,12 @@
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4254,11 +4254,11 @@
         <v>46319</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>125</v>
-      </c>
-      <c r="C56" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C56" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D56" s="42" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Nike Ja 4 “Radar”</t>
         </is>
       </c>
     </row>
@@ -4282,11 +4282,11 @@
         <v>46319</v>
       </c>
       <c r="B57" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C57" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C57" s="50" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D57" s="43" t="inlineStr">
@@ -4296,12 +4296,12 @@
       </c>
       <c r="E57" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Vans Old Skool 36 Pearlized “Red”</t>
         </is>
       </c>
     </row>
@@ -4310,16 +4310,16 @@
         <v>46319</v>
       </c>
       <c r="B58" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C58" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D58" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C58" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
@@ -4329,7 +4329,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Radar”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -4338,26 +4338,26 @@
         <v>46319</v>
       </c>
       <c r="B59" s="41" t="n">
-        <v>130</v>
-      </c>
-      <c r="C59" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D59" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C59" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D59" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Red”</t>
+          <t>Nike Air Force 1 Low “Ghostface Black”</t>
         </is>
       </c>
     </row>
@@ -4366,26 +4366,26 @@
         <v>46319</v>
       </c>
       <c r="B60" s="33" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C60" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D60" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
         </is>
       </c>
     </row>
@@ -4394,11 +4394,11 @@
         <v>46319</v>
       </c>
       <c r="B61" s="41" t="n">
-        <v>125</v>
-      </c>
-      <c r="C61" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D61" s="38" t="inlineStr">
@@ -4413,7 +4413,7 @@
       </c>
       <c r="F61" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface Black”</t>
+          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
         </is>
       </c>
     </row>
@@ -4422,11 +4422,11 @@
         <v>46319</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C62" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C62" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D62" s="42" t="inlineStr">
@@ -4436,12 +4436,12 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
+          <t>Nike Air Diamond Turf 2 “White Black”</t>
         </is>
       </c>
     </row>
@@ -4450,16 +4450,16 @@
         <v>46319</v>
       </c>
       <c r="B63" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C63" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D63" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>125</v>
+      </c>
+      <c r="C63" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D63" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E63" s="35" t="inlineStr">
@@ -4469,7 +4469,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -4478,11 +4478,11 @@
         <v>46319</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>170</v>
-      </c>
-      <c r="C64" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C64" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D64" s="42" t="inlineStr">
@@ -4497,7 +4497,7 @@
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “White Black”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -4870,7 +4870,7 @@
         <v>46337</v>
       </c>
       <c r="B78" s="33" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C78" s="39" t="inlineStr">
         <is>
@@ -4884,12 +4884,12 @@
       </c>
       <c r="E78" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -4898,7 +4898,7 @@
         <v>46337</v>
       </c>
       <c r="B79" s="41" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C79" s="40" t="inlineStr">
         <is>
@@ -4912,12 +4912,12 @@
       </c>
       <c r="E79" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F79" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Light British Tan”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -5122,11 +5122,11 @@
         <v>46340</v>
       </c>
       <c r="B87" s="41" t="n">
-        <v>255</v>
-      </c>
-      <c r="C87" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>240</v>
+      </c>
+      <c r="C87" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D87" s="38" t="inlineStr">
@@ -5141,7 +5141,7 @@
       </c>
       <c r="F87" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
         </is>
       </c>
     </row>
@@ -5150,26 +5150,26 @@
         <v>46340</v>
       </c>
       <c r="B88" s="33" t="n">
-        <v>240</v>
+        <v>140</v>
       </c>
       <c r="C88" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D88" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D88" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
+          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
         </is>
       </c>
     </row>
@@ -5178,16 +5178,16 @@
         <v>46340</v>
       </c>
       <c r="B89" s="41" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C89" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D89" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E89" s="35" t="inlineStr">
@@ -5197,7 +5197,7 @@
       </c>
       <c r="F89" s="35" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
+          <t>CPFM x Nike Flea 1 “Barely”</t>
         </is>
       </c>
     </row>
@@ -5206,16 +5206,16 @@
         <v>46340</v>
       </c>
       <c r="B90" s="33" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C90" s="48" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D90" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5225,7 +5225,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>CPFM x Nike Flea 1 “Barely”</t>
+          <t>Nike Zoom Hyperflight “Green Apple”</t>
         </is>
       </c>
     </row>
@@ -5234,26 +5234,26 @@
         <v>46340</v>
       </c>
       <c r="B91" s="41" t="n">
-        <v>170</v>
-      </c>
-      <c r="C91" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D91" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>255</v>
+      </c>
+      <c r="C91" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E91" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F91" s="35" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Green Apple”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -5402,11 +5402,11 @@
         <v>46346</v>
       </c>
       <c r="B97" s="41" t="n">
-        <v>190</v>
-      </c>
-      <c r="C97" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C97" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D97" s="43" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="F97" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “ACG”</t>
+          <t>Nike Book 2 “Be Legendary”</t>
         </is>
       </c>
     </row>
@@ -5430,11 +5430,11 @@
         <v>46346</v>
       </c>
       <c r="B98" s="33" t="n">
-        <v>145</v>
-      </c>
-      <c r="C98" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C98" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D98" s="42" t="inlineStr">
@@ -5449,7 +5449,7 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Be Legendary”</t>
+          <t>Nike Air Max 95 “ACG”</t>
         </is>
       </c>
     </row>
@@ -5486,7 +5486,7 @@
         <v>46347</v>
       </c>
       <c r="B100" s="33" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="C100" s="39" t="inlineStr">
         <is>
@@ -5500,12 +5500,12 @@
       </c>
       <c r="E100" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -5513,10 +5513,12 @@
       <c r="A101" s="36" t="n">
         <v>46347</v>
       </c>
-      <c r="B101" s="41" t="inlineStr"/>
-      <c r="C101" s="50" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B101" s="41" t="n">
+        <v>125</v>
+      </c>
+      <c r="C101" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D101" s="43" t="inlineStr">
@@ -5526,12 +5528,12 @@
       </c>
       <c r="E101" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F101" s="35" t="inlineStr">
         <is>
-          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5540,11 +5542,11 @@
         <v>46347</v>
       </c>
       <c r="B102" s="33" t="n">
-        <v>165</v>
-      </c>
-      <c r="C102" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C102" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D102" s="42" t="inlineStr">
@@ -5554,12 +5556,12 @@
       </c>
       <c r="E102" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -5568,16 +5570,16 @@
         <v>46347</v>
       </c>
       <c r="B103" s="41" t="n">
-        <v>125</v>
+        <v>230</v>
       </c>
       <c r="C103" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D103" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D103" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E103" s="35" t="inlineStr">
@@ -5587,7 +5589,7 @@
       </c>
       <c r="F103" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -5596,11 +5598,11 @@
         <v>46347</v>
       </c>
       <c r="B104" s="33" t="n">
-        <v>140</v>
-      </c>
-      <c r="C104" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C104" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D104" s="42" t="inlineStr">
@@ -5610,12 +5612,12 @@
       </c>
       <c r="E104" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -5624,16 +5626,16 @@
         <v>46347</v>
       </c>
       <c r="B105" s="41" t="n">
-        <v>230</v>
+        <v>140</v>
       </c>
       <c r="C105" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D105" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D105" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E105" s="35" t="inlineStr">
@@ -5643,7 +5645,7 @@
       </c>
       <c r="F105" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -5651,12 +5653,10 @@
       <c r="A106" s="31" t="n">
         <v>46347</v>
       </c>
-      <c r="B106" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C106" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B106" s="33" t="inlineStr"/>
+      <c r="C106" s="54" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D106" s="42" t="inlineStr">
@@ -5666,12 +5666,12 @@
       </c>
       <c r="E106" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
         </is>
       </c>
     </row>
@@ -5763,25 +5763,27 @@
       <c r="A110" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B110" s="33" t="inlineStr"/>
-      <c r="C110" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D110" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B110" s="33" t="n">
+        <v>140</v>
+      </c>
+      <c r="C110" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D110" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E110" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Caitlin 1 “Warning Code”</t>
         </is>
       </c>
     </row>
@@ -5790,11 +5792,11 @@
         <v>46354</v>
       </c>
       <c r="B111" s="41" t="n">
-        <v>140</v>
-      </c>
-      <c r="C111" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C111" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D111" s="43" t="inlineStr">
@@ -5809,7 +5811,7 @@
       </c>
       <c r="F111" s="35" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Warning Code”</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -5818,16 +5820,16 @@
         <v>46354</v>
       </c>
       <c r="B112" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C112" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D112" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D112" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E112" s="30" t="inlineStr">
@@ -5837,7 +5839,7 @@
       </c>
       <c r="F112" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro “FSU”</t>
         </is>
       </c>
     </row>
@@ -5846,7 +5848,7 @@
         <v>46354</v>
       </c>
       <c r="B113" s="41" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C113" s="40" t="inlineStr">
         <is>
@@ -5865,7 +5867,7 @@
       </c>
       <c r="F113" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “FSU”</t>
+          <t>Instant Skateboards x Nike SB Air Force 1</t>
         </is>
       </c>
     </row>
@@ -5873,17 +5875,15 @@
       <c r="A114" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B114" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B114" s="33" t="inlineStr"/>
       <c r="C114" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D114" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D114" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E114" s="30" t="inlineStr">
@@ -5893,7 +5893,7 @@
       </c>
       <c r="F114" s="30" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -5901,15 +5901,17 @@
       <c r="A115" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B115" s="41" t="inlineStr"/>
+      <c r="B115" s="41" t="n">
+        <v>130</v>
+      </c>
       <c r="C115" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D115" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D115" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E115" s="35" t="inlineStr">
@@ -5919,7 +5921,7 @@
       </c>
       <c r="F115" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -5927,17 +5929,15 @@
       <c r="A116" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B116" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C116" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D116" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B116" s="33" t="inlineStr"/>
+      <c r="C116" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D116" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E116" s="30" t="inlineStr">
@@ -5947,7 +5947,7 @@
       </c>
       <c r="F116" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Nike KD 6 “Aunt Pearl” 2026</t>
         </is>
       </c>
     </row>
@@ -5956,24 +5956,24 @@
         <v>46354</v>
       </c>
       <c r="B117" s="41" t="inlineStr"/>
-      <c r="C117" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D117" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C117" s="37" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D117" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E117" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F117" s="35" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Aunt Pearl” 2026</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6038,26 +6038,26 @@
         <v>46361</v>
       </c>
       <c r="B120" s="33" t="n">
-        <v>300</v>
-      </c>
-      <c r="C120" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D120" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>215</v>
+      </c>
+      <c r="C120" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D120" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E120" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F120" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
@@ -6066,11 +6066,11 @@
         <v>46361</v>
       </c>
       <c r="B121" s="41" t="n">
-        <v>225</v>
-      </c>
-      <c r="C121" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>300</v>
+      </c>
+      <c r="C121" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D121" s="43" t="inlineStr">
@@ -6080,12 +6080,12 @@
       </c>
       <c r="E121" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F121" s="35" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
         </is>
       </c>
     </row>
@@ -6094,26 +6094,26 @@
         <v>46361</v>
       </c>
       <c r="B122" s="33" t="n">
-        <v>215</v>
-      </c>
-      <c r="C122" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D122" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>300</v>
+      </c>
+      <c r="C122" s="48" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D122" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E122" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F122" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
         </is>
       </c>
     </row>
@@ -6122,11 +6122,11 @@
         <v>46361</v>
       </c>
       <c r="B123" s="41" t="n">
-        <v>300</v>
-      </c>
-      <c r="C123" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>225</v>
+      </c>
+      <c r="C123" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D123" s="43" t="inlineStr">
@@ -6136,12 +6136,12 @@
       </c>
       <c r="E123" s="35" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F123" s="35" t="inlineStr">
         <is>
-          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
@@ -6178,26 +6178,26 @@
         <v>46367</v>
       </c>
       <c r="B125" s="41" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C125" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D125" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D125" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E125" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F125" s="35" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -6205,27 +6205,25 @@
       <c r="A126" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B126" s="33" t="n">
-        <v>240</v>
-      </c>
+      <c r="B126" s="33" t="inlineStr"/>
       <c r="C126" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D126" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D126" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E126" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F126" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -6233,7 +6231,9 @@
       <c r="A127" s="36" t="n">
         <v>46367</v>
       </c>
-      <c r="B127" s="41" t="inlineStr"/>
+      <c r="B127" s="41" t="n">
+        <v>150</v>
+      </c>
       <c r="C127" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="F127" s="35" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6288,26 +6288,26 @@
         <v>46368</v>
       </c>
       <c r="B129" s="41" t="n">
-        <v>235</v>
-      </c>
-      <c r="C129" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D129" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>135</v>
+      </c>
+      <c r="C129" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D129" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E129" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F129" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>PaisaBoys x Nike SB P-Rod 1</t>
         </is>
       </c>
     </row>
@@ -6316,26 +6316,26 @@
         <v>46368</v>
       </c>
       <c r="B130" s="33" t="n">
-        <v>135</v>
-      </c>
-      <c r="C130" s="48" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D130" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C130" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D130" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E130" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F130" s="30" t="inlineStr">
         <is>
-          <t>PaisaBoys x Nike SB P-Rod 1</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
@@ -6344,11 +6344,11 @@
         <v>46375</v>
       </c>
       <c r="B131" s="41" t="n">
-        <v>210</v>
-      </c>
-      <c r="C131" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>220</v>
+      </c>
+      <c r="C131" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D131" s="43" t="inlineStr">
@@ -6358,12 +6358,12 @@
       </c>
       <c r="E131" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F131" s="35" t="inlineStr">
         <is>
-          <t>Nike GT Future “Triple Black”</t>
+          <t>Air Jordan 4 “Pink Thunder”</t>
         </is>
       </c>
     </row>
@@ -6372,26 +6372,26 @@
         <v>46375</v>
       </c>
       <c r="B132" s="33" t="n">
-        <v>220</v>
+        <v>120</v>
       </c>
       <c r="C132" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D132" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D132" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E132" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F132" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
         </is>
       </c>
     </row>
@@ -6400,16 +6400,16 @@
         <v>46375</v>
       </c>
       <c r="B133" s="41" t="n">
-        <v>120</v>
-      </c>
-      <c r="C133" s="40" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D133" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C133" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D133" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E133" s="35" t="inlineStr">
@@ -6419,7 +6419,7 @@
       </c>
       <c r="F133" s="35" t="inlineStr">
         <is>
-          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
+          <t>Nike Air Zoom Flight The Glove “Royal Blue”</t>
         </is>
       </c>
     </row>
@@ -6428,7 +6428,7 @@
         <v>46375</v>
       </c>
       <c r="B134" s="33" t="n">
-        <v>170</v>
+        <v>210</v>
       </c>
       <c r="C134" s="48" t="inlineStr">
         <is>
@@ -6447,7 +6447,7 @@
       </c>
       <c r="F134" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Flight The Glove “Royal Blue”</t>
+          <t>Nike GT Future “Triple Black”</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6661,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="52" t="inlineStr">
         <is>
-          <t>Generated September 27, 2026  ·  11:37 UTC</t>
+          <t>Generated September 28, 2026  ·  13:11 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6707,16 +6707,16 @@
         <v>46295</v>
       </c>
       <c r="B4" s="33" t="n">
-        <v>155</v>
+        <v>135</v>
       </c>
       <c r="C4" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D4" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D4" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E4" s="30" t="inlineStr">
@@ -6726,7 +6726,7 @@
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Union LA x Nike Dunk Low “Bamboo”</t>
         </is>
       </c>
     </row>
@@ -6735,26 +6735,26 @@
         <v>46295</v>
       </c>
       <c r="B5" s="41" t="n">
-        <v>135</v>
+        <v>210</v>
       </c>
       <c r="C5" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D5" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D5" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E5" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F5" s="35" t="inlineStr">
         <is>
-          <t>Union LA x Nike Dunk Low “Bamboo”</t>
+          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
         </is>
       </c>
     </row>
@@ -6763,7 +6763,7 @@
         <v>46295</v>
       </c>
       <c r="B6" s="33" t="n">
-        <v>210</v>
+        <v>125</v>
       </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
@@ -6777,12 +6777,12 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 MCS “Black Metallic Gold”</t>
+          <t>Nike Air Force 1 Low “Leopard”</t>
         </is>
       </c>
     </row>
@@ -6791,7 +6791,7 @@
         <v>46295</v>
       </c>
       <c r="B7" s="41" t="n">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="C7" s="40" t="inlineStr">
         <is>
@@ -6810,7 +6810,7 @@
       </c>
       <c r="F7" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Leopard”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -6819,26 +6819,26 @@
         <v>46296</v>
       </c>
       <c r="B8" s="33" t="n">
-        <v>120</v>
+        <v>155</v>
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D8" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D8" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Dunk Low “Campfire Orange”</t>
+          <t>Air Jordan 1 Low OG “Howard” 2026</t>
         </is>
       </c>
     </row>
@@ -6846,27 +6846,25 @@
       <c r="A9" s="36" t="n">
         <v>46296</v>
       </c>
-      <c r="B9" s="41" t="n">
-        <v>155</v>
-      </c>
+      <c r="B9" s="41" t="inlineStr"/>
       <c r="C9" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D9" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D9" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E9" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low OG “Howard” 2026</t>
+          <t>Nike Air Max 95 “Liverpool”</t>
         </is>
       </c>
     </row>
@@ -6874,7 +6872,9 @@
       <c r="A10" s="31" t="n">
         <v>46296</v>
       </c>
-      <c r="B10" s="33" t="inlineStr"/>
+      <c r="B10" s="33" t="n">
+        <v>125</v>
+      </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -6892,7 +6892,7 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Liverpool”</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “Black Purple Stardust”</t>
         </is>
       </c>
     </row>
@@ -6901,7 +6901,7 @@
         <v>46296</v>
       </c>
       <c r="B11" s="41" t="n">
-        <v>125</v>
+        <v>105</v>
       </c>
       <c r="C11" s="40" t="inlineStr">
         <is>
@@ -6920,7 +6920,7 @@
       </c>
       <c r="F11" s="35" t="inlineStr">
         <is>
-          <t>Kobe Bryant x Nike Air Force 1 Low “Black Purple Stardust”</t>
+          <t>Kobe Bryant x Nike Air Force 1 Low “5 Rings”</t>
         </is>
       </c>
     </row>
@@ -7377,7 +7377,7 @@
         <v>46319</v>
       </c>
       <c r="B28" s="33" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C28" s="39" t="inlineStr">
         <is>
@@ -7391,12 +7391,12 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -7405,16 +7405,16 @@
         <v>46319</v>
       </c>
       <c r="B29" s="41" t="n">
-        <v>125</v>
+        <v>150</v>
       </c>
       <c r="C29" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D29" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="35" t="inlineStr">
@@ -7424,7 +7424,7 @@
       </c>
       <c r="F29" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
@@ -7440,19 +7440,19 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D30" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D30" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Nike Air Force 1 Low “Ghostface Black”</t>
         </is>
       </c>
     </row>
@@ -7461,26 +7461,26 @@
         <v>46319</v>
       </c>
       <c r="B31" s="41" t="n">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C31" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D31" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D31" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F31" s="35" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
         </is>
       </c>
     </row>
@@ -7496,9 +7496,9 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D32" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D32" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E32" s="30" t="inlineStr">
@@ -7508,7 +7508,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface Black”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -7517,7 +7517,7 @@
         <v>46319</v>
       </c>
       <c r="B33" s="41" t="n">
-        <v>145</v>
+        <v>190</v>
       </c>
       <c r="C33" s="40" t="inlineStr">
         <is>
@@ -7531,12 +7531,12 @@
       </c>
       <c r="E33" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F33" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -7685,7 +7685,7 @@
         <v>46337</v>
       </c>
       <c r="B39" s="41" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C39" s="40" t="inlineStr">
         <is>
@@ -7699,12 +7699,12 @@
       </c>
       <c r="E39" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F39" s="35" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 11 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -7713,7 +7713,7 @@
         <v>46337</v>
       </c>
       <c r="B40" s="33" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C40" s="39" t="inlineStr">
         <is>
@@ -7727,12 +7727,12 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Light British Tan”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
@@ -7937,7 +7937,7 @@
         <v>46347</v>
       </c>
       <c r="B48" s="33" t="n">
-        <v>140</v>
+        <v>165</v>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
@@ -7951,12 +7951,12 @@
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -7965,7 +7965,7 @@
         <v>46347</v>
       </c>
       <c r="B49" s="41" t="n">
-        <v>165</v>
+        <v>125</v>
       </c>
       <c r="C49" s="40" t="inlineStr">
         <is>
@@ -7979,12 +7979,12 @@
       </c>
       <c r="E49" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F49" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -7993,16 +7993,16 @@
         <v>46347</v>
       </c>
       <c r="B50" s="33" t="n">
-        <v>125</v>
+        <v>230</v>
       </c>
       <c r="C50" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D50" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
@@ -8012,7 +8012,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -8021,26 +8021,26 @@
         <v>46347</v>
       </c>
       <c r="B51" s="41" t="n">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C51" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D51" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E51" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F51" s="35" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -8049,7 +8049,7 @@
         <v>46347</v>
       </c>
       <c r="B52" s="33" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="C52" s="39" t="inlineStr">
         <is>
@@ -8063,12 +8063,12 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -8132,25 +8132,27 @@
       <c r="A55" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B55" s="41" t="inlineStr"/>
-      <c r="C55" s="37" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D55" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="B55" s="41" t="n">
+        <v>190</v>
+      </c>
+      <c r="C55" s="40" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D55" s="43" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="35" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F55" s="35" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
         </is>
       </c>
     </row>
@@ -8159,16 +8161,16 @@
         <v>46354</v>
       </c>
       <c r="B56" s="33" t="n">
-        <v>190</v>
+        <v>240</v>
       </c>
       <c r="C56" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D56" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D56" s="34" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
@@ -8178,7 +8180,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Dynamic Yellow”</t>
+          <t>Nike Air Foamposite Pro “FSU”</t>
         </is>
       </c>
     </row>
@@ -8187,7 +8189,7 @@
         <v>46354</v>
       </c>
       <c r="B57" s="41" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="C57" s="40" t="inlineStr">
         <is>
@@ -8206,7 +8208,7 @@
       </c>
       <c r="F57" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “FSU”</t>
+          <t>Instant Skateboards x Nike SB Air Force 1</t>
         </is>
       </c>
     </row>
@@ -8214,17 +8216,15 @@
       <c r="A58" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B58" s="33" t="n">
-        <v>120</v>
-      </c>
+      <c r="B58" s="33" t="inlineStr"/>
       <c r="C58" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D58" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D58" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
@@ -8234,7 +8234,7 @@
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -8242,15 +8242,17 @@
       <c r="A59" s="36" t="n">
         <v>46354</v>
       </c>
-      <c r="B59" s="41" t="inlineStr"/>
+      <c r="B59" s="41" t="n">
+        <v>130</v>
+      </c>
       <c r="C59" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D59" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="35" t="inlineStr">
@@ -8260,7 +8262,7 @@
       </c>
       <c r="F59" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -8268,12 +8270,10 @@
       <c r="A60" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B60" s="33" t="n">
-        <v>130</v>
-      </c>
-      <c r="C60" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B60" s="33" t="inlineStr"/>
+      <c r="C60" s="32" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
         </is>
       </c>
       <c r="D60" s="34" t="inlineStr">
@@ -8283,12 +8283,12 @@
       </c>
       <c r="E60" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -8325,7 +8325,7 @@
         <v>46361</v>
       </c>
       <c r="B62" s="33" t="n">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C62" s="39" t="inlineStr">
         <is>
@@ -8344,7 +8344,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
@@ -8353,7 +8353,7 @@
         <v>46361</v>
       </c>
       <c r="B63" s="41" t="n">
-        <v>215</v>
+        <v>225</v>
       </c>
       <c r="C63" s="40" t="inlineStr">
         <is>
@@ -8372,7 +8372,7 @@
       </c>
       <c r="F63" s="35" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
@@ -8381,26 +8381,26 @@
         <v>46367</v>
       </c>
       <c r="B64" s="33" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C64" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D64" s="34" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D64" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -8408,27 +8408,25 @@
       <c r="A65" s="36" t="n">
         <v>46367</v>
       </c>
-      <c r="B65" s="41" t="n">
-        <v>240</v>
-      </c>
+      <c r="B65" s="41" t="inlineStr"/>
       <c r="C65" s="40" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D65" s="43" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D65" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E65" s="35" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="35" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -8436,7 +8434,9 @@
       <c r="A66" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B66" s="33" t="inlineStr"/>
+      <c r="B66" s="33" t="n">
+        <v>150</v>
+      </c>
       <c r="C66" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8454,7 +8454,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-10-09 12:46 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$151</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$79</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -549,7 +549,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -683,6 +683,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1578,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated October 08, 2026  ·  13:00 UTC</t>
+          <t>Generated October 09, 2026  ·  12:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1622,16 +1625,16 @@
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$178</t>
+          <t>$177</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1734,7 +1737,7 @@
         <v>46354</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1766,7 +1769,7 @@
         <v>46382</v>
       </c>
       <c r="D11" s="34" t="n">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E11" s="36" t="inlineStr">
         <is>
@@ -1800,7 +1803,7 @@
         <v>46304</v>
       </c>
       <c r="D12" s="30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E12" s="39" t="inlineStr">
         <is>
@@ -1834,7 +1837,7 @@
         <v>46304</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E13" s="36" t="inlineStr">
         <is>
@@ -1868,7 +1871,7 @@
         <v>46305</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1902,7 +1905,7 @@
         <v>46306</v>
       </c>
       <c r="D15" s="34" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="36" t="inlineStr">
         <is>
@@ -1936,7 +1939,7 @@
         <v>46310</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -2009,7 +2012,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2035,7 +2038,7 @@
         </is>
       </c>
       <c r="B21" s="34" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
@@ -2043,7 +2046,7 @@
         </is>
       </c>
       <c r="E21" s="34" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G21" s="46" t="inlineStr">
         <is>
@@ -2061,7 +2064,7 @@
         </is>
       </c>
       <c r="B22" s="30" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D22" s="47" t="inlineStr">
         <is>
@@ -2087,7 +2090,7 @@
         </is>
       </c>
       <c r="B23" s="34" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D23" s="49" t="inlineStr">
         <is>
@@ -2095,7 +2098,7 @@
         </is>
       </c>
       <c r="E23" s="34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -2178,17 +2181,17 @@
       </c>
       <c r="B30" s="30" t="inlineStr">
         <is>
-          <t>10/8 – 10/14</t>
+          <t>10/9 – 10/15</t>
         </is>
       </c>
       <c r="C30" s="30" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D30" s="39" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E30" s="30" t="n">
-        <v>4.9</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2199,17 +2202,17 @@
       </c>
       <c r="B31" s="34" t="inlineStr">
         <is>
-          <t>10/15 – 10/21</t>
+          <t>10/16 – 10/22</t>
         </is>
       </c>
       <c r="C31" s="34" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D31" s="36" t="n">
         <v>5</v>
       </c>
       <c r="E31" s="34" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
@@ -2220,17 +2223,17 @@
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t>10/22 – 10/28</t>
+          <t>10/23 – 10/29</t>
         </is>
       </c>
       <c r="C32" s="30" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D32" s="39" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="E32" s="30" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2241,17 +2244,17 @@
       </c>
       <c r="B33" s="34" t="inlineStr">
         <is>
-          <t>10/29 – 11/4</t>
+          <t>10/30 – 11/5</t>
         </is>
       </c>
       <c r="C33" s="34" t="n">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="D33" s="36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E33" s="34" t="n">
-        <v>5.5</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2262,17 +2265,17 @@
       </c>
       <c r="B34" s="30" t="inlineStr">
         <is>
-          <t>11/5 – 11/11</t>
+          <t>11/6 – 11/12</t>
         </is>
       </c>
       <c r="C34" s="30" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="D34" s="39" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E34" s="30" t="n">
-        <v>5.7</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2283,17 +2286,17 @@
       </c>
       <c r="B35" s="34" t="inlineStr">
         <is>
-          <t>11/12 – 11/18</t>
+          <t>11/13 – 11/19</t>
         </is>
       </c>
       <c r="C35" s="34" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D35" s="36" t="n">
         <v>6</v>
       </c>
       <c r="E35" s="34" t="n">
-        <v>5.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2304,17 +2307,17 @@
       </c>
       <c r="B36" s="30" t="inlineStr">
         <is>
-          <t>11/19 – 11/25</t>
+          <t>11/20 – 11/26</t>
         </is>
       </c>
       <c r="C36" s="30" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="D36" s="39" t="n">
         <v>7</v>
       </c>
       <c r="E36" s="30" t="n">
-        <v>5.3</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2325,17 +2328,17 @@
       </c>
       <c r="B37" s="34" t="inlineStr">
         <is>
-          <t>11/26 – 12/2</t>
+          <t>11/27 – 12/3</t>
         </is>
       </c>
       <c r="C37" s="34" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D37" s="36" t="n">
         <v>8</v>
       </c>
       <c r="E37" s="34" t="n">
-        <v>6.2</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2346,17 +2349,17 @@
       </c>
       <c r="B38" s="30" t="inlineStr">
         <is>
-          <t>12/3 – 12/9</t>
+          <t>12/4 – 12/10</t>
         </is>
       </c>
       <c r="C38" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D38" s="39" t="n">
         <v>3</v>
       </c>
       <c r="E38" s="30" t="n">
-        <v>5.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2367,7 +2370,7 @@
       </c>
       <c r="B39" s="34" t="inlineStr">
         <is>
-          <t>12/10 – 12/16</t>
+          <t>12/11 – 12/17</t>
         </is>
       </c>
       <c r="C39" s="34" t="n">
@@ -2388,17 +2391,17 @@
       </c>
       <c r="B40" s="30" t="inlineStr">
         <is>
-          <t>12/17 – 12/23</t>
+          <t>12/18 – 12/24</t>
         </is>
       </c>
       <c r="C40" s="30" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D40" s="39" t="n">
         <v>4</v>
       </c>
       <c r="E40" s="30" t="n">
-        <v>5.7</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
@@ -2409,17 +2412,17 @@
       </c>
       <c r="B41" s="34" t="inlineStr">
         <is>
-          <t>12/24 – 12/30</t>
+          <t>12/25 – 12/31</t>
         </is>
       </c>
       <c r="C41" s="34" t="n">
+        <v>6</v>
+      </c>
+      <c r="D41" s="36" t="n">
         <v>5</v>
       </c>
-      <c r="D41" s="36" t="n">
-        <v>3</v>
-      </c>
       <c r="E41" s="34" t="n">
-        <v>6.6</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
@@ -2430,17 +2433,17 @@
       </c>
       <c r="B42" s="30" t="inlineStr">
         <is>
-          <t>12/31 – 1/6</t>
+          <t>1/1 – 1/7</t>
         </is>
       </c>
       <c r="C42" s="30" t="n">
-        <v>3</v>
-      </c>
-      <c r="D42" s="39" t="n">
-        <v>2</v>
+        <v>1</v>
+      </c>
+      <c r="D42" s="30" t="n">
+        <v>0</v>
       </c>
       <c r="E42" s="30" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>
@@ -2538,7 +2541,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2572,7 +2575,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2580,7 +2583,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2596,7 +2599,7 @@
         </is>
       </c>
       <c r="K3" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4">
@@ -2606,7 +2609,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -2640,7 +2643,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2648,7 +2651,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2656,7 +2659,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6">
@@ -2735,7 +2738,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="51" t="inlineStr">
         <is>
-          <t>Generated October 08, 2026  ·  13:00 UTC</t>
+          <t>Generated October 09, 2026  ·  12:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2778,14 +2781,14 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B4" s="40" t="n">
-        <v>250</v>
-      </c>
-      <c r="C4" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C4" s="52" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D4" s="42" t="inlineStr">
@@ -2795,40 +2798,40 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Brain Dead x adidas Samba Bowling "Snakeskin"</t>
+          <t>Street Fighter x PUMA Suede Pack</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="35" t="n">
-        <v>46303</v>
+        <v>46304</v>
       </c>
       <c r="B5" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C5" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D5" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>190</v>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D5" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E5" s="34" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Marshmallow”</t>
+          <t>Nike LeBron 24 “Greater China”</t>
         </is>
       </c>
     </row>
@@ -2837,11 +2840,11 @@
         <v>46304</v>
       </c>
       <c r="B6" s="40" t="n">
-        <v>120</v>
-      </c>
-      <c r="C6" s="52" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>180</v>
+      </c>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D6" s="42" t="inlineStr">
@@ -2851,12 +2854,12 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Street Fighter x PUMA Suede Pack</t>
+          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
         </is>
       </c>
     </row>
@@ -2865,26 +2868,26 @@
         <v>46304</v>
       </c>
       <c r="B7" s="37" t="n">
-        <v>190</v>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D7" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>130</v>
+      </c>
+      <c r="C7" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D7" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E7" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Greater China”</t>
+          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
         </is>
       </c>
     </row>
@@ -2893,11 +2896,11 @@
         <v>46304</v>
       </c>
       <c r="B8" s="40" t="n">
-        <v>180</v>
-      </c>
-      <c r="C8" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>120</v>
+      </c>
+      <c r="C8" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D8" s="42" t="inlineStr">
@@ -2912,7 +2915,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Griffey Max 1 “Cincinnati Reds”</t>
+          <t>Instant Skateboards x Nike SB Air Force 1 “City Pack”</t>
         </is>
       </c>
     </row>
@@ -2921,11 +2924,11 @@
         <v>46304</v>
       </c>
       <c r="B9" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C9" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>220</v>
+      </c>
+      <c r="C9" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D9" s="41" t="inlineStr">
@@ -2935,21 +2938,21 @@
       </c>
       <c r="E9" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>New Balance</t>
         </is>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
-          <t>adidas Anthony Edwards 3 “Snow Camo”</t>
+          <t>Aminé x New Balance 992 “Outdoor School”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B10" s="40" t="n">
-        <v>120</v>
+        <v>180</v>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
@@ -2963,21 +2966,21 @@
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Instant Skateboards x Nike SB Air Force 1 “City Pack”</t>
+          <t>Air Jordan 1 High OG “Royal” 2026</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="35" t="n">
-        <v>46304</v>
+        <v>46305</v>
       </c>
       <c r="B11" s="37" t="n">
-        <v>220</v>
+        <v>135</v>
       </c>
       <c r="C11" s="53" t="inlineStr">
         <is>
@@ -2991,12 +2994,12 @@
       </c>
       <c r="E11" s="34" t="inlineStr">
         <is>
-          <t>New Balance</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
-          <t>Aminé x New Balance 992 “Outdoor School”</t>
+          <t>Nike KD 6 “Texas”</t>
         </is>
       </c>
     </row>
@@ -3030,10 +3033,10 @@
     </row>
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="35" t="n">
-        <v>46305</v>
+        <v>46306</v>
       </c>
       <c r="B13" s="37" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
@@ -3047,30 +3050,30 @@
       </c>
       <c r="E13" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 1 High OG “Royal” 2026</t>
+          <t>Ben-G x Nike SB Air Force 1 “City Pack”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46305</v>
+        <v>46308</v>
       </c>
       <c r="B14" s="40" t="n">
-        <v>135</v>
+        <v>200</v>
       </c>
       <c r="C14" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D14" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D14" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -3080,25 +3083,25 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Texas”</t>
+          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="n">
-        <v>46306</v>
+        <v>46308</v>
       </c>
       <c r="B15" s="37" t="n">
-        <v>120</v>
-      </c>
-      <c r="C15" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D15" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C15" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E15" s="34" t="inlineStr">
@@ -3108,7 +3111,7 @@
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
-          <t>Ben-G x Nike SB Air Force 1 “City Pack”</t>
+          <t>Nike SB P-Rod 1 “Light British Tan”</t>
         </is>
       </c>
     </row>
@@ -3117,16 +3120,16 @@
         <v>46308</v>
       </c>
       <c r="B16" s="40" t="n">
-        <v>200</v>
+        <v>125</v>
       </c>
       <c r="C16" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D16" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D16" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
@@ -3136,25 +3139,25 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Cryoshot Mercurial Vapor 1 OG</t>
+          <t>Nike SB P-Rod 1 “Ale Brown”</t>
         </is>
       </c>
     </row>
     <row r="17" ht="15" customHeight="1">
       <c r="A17" s="35" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B17" s="37" t="n">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C17" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D17" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D17" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="34" t="inlineStr">
@@ -3164,25 +3167,25 @@
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 “Light British Tan”</t>
+          <t>Nike Caitlin 1 “Midnight Fever”</t>
         </is>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
       <c r="A18" s="31" t="n">
-        <v>46308</v>
+        <v>46310</v>
       </c>
       <c r="B18" s="40" t="n">
         <v>125</v>
       </c>
-      <c r="C18" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D18" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C18" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E18" s="30" t="inlineStr">
@@ -3192,16 +3195,16 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike SB P-Rod 1 “Ale Brown”</t>
+          <t>NCAA x Nike Air Force 1 Low Pack</t>
         </is>
       </c>
     </row>
     <row r="19" ht="15" customHeight="1">
       <c r="A19" s="35" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B19" s="37" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C19" s="53" t="inlineStr">
         <is>
@@ -3215,12 +3218,12 @@
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Midnight Fever”</t>
+          <t>Jordan Tatum 5 “Sunrise”</t>
         </is>
       </c>
     </row>
@@ -3229,16 +3232,16 @@
         <v>46310</v>
       </c>
       <c r="B20" s="40" t="n">
-        <v>125</v>
-      </c>
-      <c r="C20" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D20" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>175</v>
+      </c>
+      <c r="C20" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D20" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E20" s="30" t="inlineStr">
@@ -3248,20 +3251,20 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>NCAA x Nike Air Force 1 Low Pack</t>
+          <t>Nike Air Max Goadome Low “Black Croc”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="35" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B21" s="37" t="n">
-        <v>135</v>
-      </c>
-      <c r="C21" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C21" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D21" s="41" t="inlineStr">
@@ -3271,25 +3274,25 @@
       </c>
       <c r="E21" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F21" s="34" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunrise”</t>
+          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B22" s="40" t="n">
-        <v>175</v>
-      </c>
-      <c r="C22" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>250</v>
+      </c>
+      <c r="C22" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D22" s="42" t="inlineStr">
@@ -3304,16 +3307,16 @@
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Goadome Low “Black Croc”</t>
+          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15" customHeight="1">
       <c r="A23" s="35" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B23" s="37" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="C23" s="36" t="inlineStr">
         <is>
@@ -3332,16 +3335,16 @@
       </c>
       <c r="F23" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>Nocturnal x Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
       <c r="A24" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B24" s="40" t="n">
-        <v>250</v>
+        <v>220</v>
       </c>
       <c r="C24" s="39" t="inlineStr">
         <is>
@@ -3355,12 +3358,12 @@
       </c>
       <c r="E24" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3369,11 +3372,11 @@
         <v>46312</v>
       </c>
       <c r="B25" s="37" t="n">
-        <v>120</v>
-      </c>
-      <c r="C25" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C25" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D25" s="41" t="inlineStr">
@@ -3383,25 +3386,25 @@
       </c>
       <c r="E25" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F25" s="34" t="inlineStr">
         <is>
-          <t>Nocturnal x Nike SB Air Force 1 Low</t>
+          <t>Bad Bunny x adidas Gazelle Indoor “Solar Gold”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B26" s="40" t="n">
-        <v>220</v>
-      </c>
-      <c r="C26" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C26" s="52" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D26" s="42" t="inlineStr">
@@ -3411,25 +3414,25 @@
       </c>
       <c r="E26" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Reebok Angel Reese 1 “Reese’s”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="35" t="n">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B27" s="37" t="n">
-        <v>140</v>
-      </c>
-      <c r="C27" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>180</v>
+      </c>
+      <c r="C27" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D27" s="41" t="inlineStr">
@@ -3444,17 +3447,15 @@
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
-          <t>Bad Bunny x adidas Gazelle Indoor “Solar Gold”</t>
+          <t>MENACE x adidas Adistar Control 5 “Heat Signature”</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15" customHeight="1">
       <c r="A28" s="31" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B28" s="40" t="n">
-        <v>160</v>
-      </c>
+        <v>46317</v>
+      </c>
+      <c r="B28" s="40" t="inlineStr"/>
       <c r="C28" s="52" t="inlineStr">
         <is>
           <t>LOW</t>
@@ -3467,84 +3468,86 @@
       </c>
       <c r="E28" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F28" s="30" t="inlineStr">
         <is>
-          <t>Reebok Angel Reese 1 “Reese’s”</t>
+          <t>SZA x Vans VANSZA Collection</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15" customHeight="1">
       <c r="A29" s="35" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="B29" s="37" t="n">
-        <v>180</v>
-      </c>
-      <c r="C29" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D29" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C29" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D29" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
-          <t>MENACE x adidas Adistar Control 5 “Heat Signature”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
       <c r="A30" s="31" t="n">
-        <v>46317</v>
-      </c>
-      <c r="B30" s="40" t="inlineStr"/>
-      <c r="C30" s="52" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D30" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>46318</v>
+      </c>
+      <c r="B30" s="40" t="n">
+        <v>140</v>
+      </c>
+      <c r="C30" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D30" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>SZA x Vans VANSZA Collection</t>
+          <t>Nike Air Force 1 ’01 “Nightmare”</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
       <c r="A31" s="35" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B31" s="37" t="n">
-        <v>150</v>
-      </c>
-      <c r="C31" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D31" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>165</v>
+      </c>
+      <c r="C31" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D31" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E31" s="34" t="inlineStr">
@@ -3554,7 +3557,7 @@
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Nike KD 19 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3566,7 @@
         <v>46318</v>
       </c>
       <c r="B32" s="40" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="C32" s="39" t="inlineStr">
         <is>
@@ -3582,7 +3585,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Nightmare”</t>
+          <t>Nike Dunk Low “Shibuya Halloween”</t>
         </is>
       </c>
     </row>
@@ -3591,7 +3594,7 @@
         <v>46318</v>
       </c>
       <c r="B33" s="37" t="n">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="C33" s="53" t="inlineStr">
         <is>
@@ -3610,7 +3613,7 @@
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Halloween”</t>
+          <t>Nike Caitlin 1 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3619,16 +3622,16 @@
         <v>46318</v>
       </c>
       <c r="B34" s="40" t="n">
-        <v>130</v>
-      </c>
-      <c r="C34" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D34" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>145</v>
+      </c>
+      <c r="C34" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D34" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E34" s="30" t="inlineStr">
@@ -3638,7 +3641,7 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Nike Dunk Low “Shibuya Halloween”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3647,7 +3650,7 @@
         <v>46318</v>
       </c>
       <c r="B35" s="37" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C35" s="53" t="inlineStr">
         <is>
@@ -3666,7 +3669,7 @@
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Halloween”</t>
+          <t>Nike Giannis Freak 8 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3675,11 +3678,11 @@
         <v>46318</v>
       </c>
       <c r="B36" s="40" t="n">
-        <v>145</v>
-      </c>
-      <c r="C36" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>140</v>
+      </c>
+      <c r="C36" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D36" s="42" t="inlineStr">
@@ -3694,7 +3697,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Nike Air Force 1 Low “NYC Rat”</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3706,7 @@
         <v>46318</v>
       </c>
       <c r="B37" s="37" t="n">
-        <v>130</v>
+        <v>145</v>
       </c>
       <c r="C37" s="53" t="inlineStr">
         <is>
@@ -3722,7 +3725,7 @@
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
-          <t>Nike Giannis Freak 8 “Halloween”</t>
+          <t>Nike Sabrina 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3731,11 +3734,11 @@
         <v>46318</v>
       </c>
       <c r="B38" s="40" t="n">
-        <v>140</v>
-      </c>
-      <c r="C38" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C38" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D38" s="42" t="inlineStr">
@@ -3750,7 +3753,7 @@
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “NYC Rat”</t>
+          <t>Nike Air Max Plus “Spider Web”</t>
         </is>
       </c>
     </row>
@@ -3759,11 +3762,11 @@
         <v>46318</v>
       </c>
       <c r="B39" s="37" t="n">
-        <v>145</v>
-      </c>
-      <c r="C39" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C39" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D39" s="41" t="inlineStr">
@@ -3773,12 +3776,12 @@
       </c>
       <c r="E39" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
-          <t>Nike Sabrina 4 “Halloween”</t>
+          <t>PUMA Hali 1 “Pacers”</t>
         </is>
       </c>
     </row>
@@ -3787,7 +3790,7 @@
         <v>46318</v>
       </c>
       <c r="B40" s="40" t="n">
-        <v>170</v>
+        <v>145</v>
       </c>
       <c r="C40" s="47" t="inlineStr">
         <is>
@@ -3806,35 +3809,35 @@
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max Plus “Spider Web”</t>
+          <t>Cade Cunningham x Nike ST Charge “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15" customHeight="1">
       <c r="A41" s="35" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B41" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C41" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D41" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>170</v>
+      </c>
+      <c r="C41" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D41" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E41" s="34" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
-          <t>PUMA Hali 1 “Pacers”</t>
+          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
         </is>
       </c>
     </row>
@@ -3843,16 +3846,16 @@
         <v>46319</v>
       </c>
       <c r="B42" s="40" t="n">
-        <v>170</v>
-      </c>
-      <c r="C42" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D42" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>190</v>
+      </c>
+      <c r="C42" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
@@ -3862,7 +3865,7 @@
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Jason Williams x SLAM x Nike Zoom Hyperflight “Platinum”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
@@ -3871,11 +3874,11 @@
         <v>46319</v>
       </c>
       <c r="B43" s="37" t="n">
-        <v>190</v>
-      </c>
-      <c r="C43" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C43" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D43" s="41" t="inlineStr">
@@ -3890,7 +3893,7 @@
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Nike Air Diamond Turf 2 “White Black”</t>
         </is>
       </c>
     </row>
@@ -3899,11 +3902,11 @@
         <v>46319</v>
       </c>
       <c r="B44" s="40" t="n">
-        <v>170</v>
-      </c>
-      <c r="C44" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C44" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="42" t="inlineStr">
@@ -3913,12 +3916,12 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “White Black”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3927,11 +3930,11 @@
         <v>46319</v>
       </c>
       <c r="B45" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C45" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C45" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D45" s="41" t="inlineStr">
@@ -3941,12 +3944,12 @@
       </c>
       <c r="E45" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Nike Ja 4 “Radar”</t>
         </is>
       </c>
     </row>
@@ -3955,11 +3958,11 @@
         <v>46319</v>
       </c>
       <c r="B46" s="40" t="n">
-        <v>140</v>
-      </c>
-      <c r="C46" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C46" s="52" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D46" s="42" t="inlineStr">
@@ -3969,12 +3972,12 @@
       </c>
       <c r="E46" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Radar”</t>
+          <t>Vans Old Skool 36 Pearlized “Red”</t>
         </is>
       </c>
     </row>
@@ -3983,26 +3986,26 @@
         <v>46319</v>
       </c>
       <c r="B47" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C47" s="49" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D47" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>125</v>
+      </c>
+      <c r="C47" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D47" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E47" s="34" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="34" t="inlineStr">
         <is>
-          <t>Vans Old Skool 36 Pearlized “Red”</t>
+          <t>Nike Air Force 1 Low “Ghostface Black”</t>
         </is>
       </c>
     </row>
@@ -4011,26 +4014,26 @@
         <v>46319</v>
       </c>
       <c r="B48" s="40" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C48" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D48" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D48" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E48" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface Black”</t>
+          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
         </is>
       </c>
     </row>
@@ -4039,7 +4042,7 @@
         <v>46319</v>
       </c>
       <c r="B49" s="37" t="n">
-        <v>145</v>
+        <v>215</v>
       </c>
       <c r="C49" s="36" t="inlineStr">
         <is>
@@ -4058,7 +4061,7 @@
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
+          <t>Air Jordan 12 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4070,7 @@
         <v>46319</v>
       </c>
       <c r="B50" s="40" t="n">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C50" s="39" t="inlineStr">
         <is>
@@ -4081,12 +4084,12 @@
       </c>
       <c r="E50" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Fireside”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -4095,11 +4098,11 @@
         <v>46319</v>
       </c>
       <c r="B51" s="37" t="n">
-        <v>125</v>
-      </c>
-      <c r="C51" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>300</v>
+      </c>
+      <c r="C51" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D51" s="41" t="inlineStr">
@@ -4109,25 +4112,25 @@
       </c>
       <c r="E51" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Pharrell x adidas Adistar Jellyfish</t>
         </is>
       </c>
     </row>
     <row r="52" ht="15" customHeight="1">
       <c r="A52" s="31" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="B52" s="40" t="n">
-        <v>300</v>
-      </c>
-      <c r="C52" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="42" t="inlineStr">
@@ -4137,21 +4140,21 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="35" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="B53" s="37" t="n">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="C53" s="36" t="inlineStr">
         <is>
@@ -4165,12 +4168,12 @@
       </c>
       <c r="E53" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Force 1 Low “University Pack”</t>
         </is>
       </c>
     </row>
@@ -4198,7 +4201,7 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “University Pack”</t>
+          <t>Nike Air Force 1 Low “Texas”</t>
         </is>
       </c>
     </row>
@@ -4226,7 +4229,7 @@
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Texas”</t>
+          <t>Nike Air Force 1 Low “Georgia”</t>
         </is>
       </c>
     </row>
@@ -4254,7 +4257,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Georgia”</t>
+          <t>Nike Air Force 1 Low “Kentucky”</t>
         </is>
       </c>
     </row>
@@ -4282,16 +4285,16 @@
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Kentucky”</t>
+          <t>Nike Air Force 1 Low “Oregon”</t>
         </is>
       </c>
     </row>
     <row r="58" ht="15" customHeight="1">
       <c r="A58" s="31" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="B58" s="40" t="n">
-        <v>125</v>
+        <v>205</v>
       </c>
       <c r="C58" s="39" t="inlineStr">
         <is>
@@ -4305,12 +4308,12 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Oregon”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -4319,26 +4322,26 @@
         <v>46325</v>
       </c>
       <c r="B59" s="37" t="n">
-        <v>205</v>
-      </c>
-      <c r="C59" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D59" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>180</v>
+      </c>
+      <c r="C59" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D59" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Nike Ja 4 High “University Red”</t>
         </is>
       </c>
     </row>
@@ -4347,16 +4350,16 @@
         <v>46325</v>
       </c>
       <c r="B60" s="40" t="n">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="C60" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D60" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D60" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E60" s="30" t="inlineStr">
@@ -4366,7 +4369,7 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 High “University Red”</t>
+          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
         </is>
       </c>
     </row>
@@ -4394,20 +4397,20 @@
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
-          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
+          <t>Nike Book 2 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="62" ht="15" customHeight="1">
       <c r="A62" s="31" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B62" s="40" t="n">
-        <v>155</v>
-      </c>
-      <c r="C62" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>140</v>
+      </c>
+      <c r="C62" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D62" s="42" t="inlineStr">
@@ -4422,7 +4425,7 @@
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Halloween”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4434,7 @@
         <v>46326</v>
       </c>
       <c r="B63" s="37" t="n">
-        <v>140</v>
+        <v>215</v>
       </c>
       <c r="C63" s="36" t="inlineStr">
         <is>
@@ -4445,40 +4448,40 @@
       </c>
       <c r="E63" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Air Jordan 14 “Forest Green”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46326</v>
+        <v>46331</v>
       </c>
       <c r="B64" s="40" t="n">
-        <v>215</v>
-      </c>
-      <c r="C64" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D64" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>265</v>
+      </c>
+      <c r="C64" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D64" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Forest Green”</t>
+          <t>Nike Air Max Foamdome “Eggplant” 2026</t>
         </is>
       </c>
     </row>
@@ -4487,26 +4490,26 @@
         <v>46331</v>
       </c>
       <c r="B65" s="37" t="n">
-        <v>265</v>
-      </c>
-      <c r="C65" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D65" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>140</v>
+      </c>
+      <c r="C65" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D65" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E65" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Max Foamdome “Eggplant” 2026</t>
+          <t>Air Jordan 1 Mid “Space Jam Hare”</t>
         </is>
       </c>
     </row>
@@ -4795,16 +4798,16 @@
         <v>46333</v>
       </c>
       <c r="B76" s="40" t="n">
-        <v>215</v>
+        <v>240</v>
       </c>
       <c r="C76" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D76" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D76" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E76" s="30" t="inlineStr">
@@ -4814,7 +4817,7 @@
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -4823,16 +4826,16 @@
         <v>46333</v>
       </c>
       <c r="B77" s="37" t="n">
-        <v>245</v>
+        <v>215</v>
       </c>
       <c r="C77" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D77" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D77" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E77" s="34" t="inlineStr">
@@ -4842,7 +4845,7 @@
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 17 Low “Black Pack”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4854,7 @@
         <v>46333</v>
       </c>
       <c r="B78" s="40" t="n">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C78" s="39" t="inlineStr">
         <is>
@@ -4870,7 +4873,7 @@
       </c>
       <c r="F78" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 17 Low “Black Pack”</t>
         </is>
       </c>
     </row>
@@ -5131,26 +5134,26 @@
         <v>46340</v>
       </c>
       <c r="B88" s="40" t="n">
-        <v>170</v>
-      </c>
-      <c r="C88" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>255</v>
+      </c>
+      <c r="C88" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Green Apple”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -5159,11 +5162,11 @@
         <v>46340</v>
       </c>
       <c r="B89" s="37" t="n">
-        <v>255</v>
-      </c>
-      <c r="C89" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>240</v>
+      </c>
+      <c r="C89" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D89" s="38" t="inlineStr">
@@ -5178,7 +5181,7 @@
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
         </is>
       </c>
     </row>
@@ -5187,26 +5190,26 @@
         <v>46340</v>
       </c>
       <c r="B90" s="40" t="n">
-        <v>240</v>
+        <v>140</v>
       </c>
       <c r="C90" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D90" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 9 Boot NRG “Iridescent”</t>
+          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
         </is>
       </c>
     </row>
@@ -5215,16 +5218,16 @@
         <v>46340</v>
       </c>
       <c r="B91" s="37" t="n">
-        <v>140</v>
+        <v>180</v>
       </c>
       <c r="C91" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D91" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E91" s="34" t="inlineStr">
@@ -5234,7 +5237,7 @@
       </c>
       <c r="F91" s="34" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
+          <t>CPFM x Nike Flea 1 “Barely”</t>
         </is>
       </c>
     </row>
@@ -5243,16 +5246,16 @@
         <v>46340</v>
       </c>
       <c r="B92" s="40" t="n">
-        <v>180</v>
+        <v>170</v>
       </c>
       <c r="C92" s="47" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D92" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D92" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E92" s="30" t="inlineStr">
@@ -5262,7 +5265,7 @@
       </c>
       <c r="F92" s="30" t="inlineStr">
         <is>
-          <t>CPFM x Nike Flea 1 “Barely”</t>
+          <t>Nike Zoom Hyperflight “Green Apple”</t>
         </is>
       </c>
     </row>
@@ -5411,11 +5414,11 @@
         <v>46346</v>
       </c>
       <c r="B98" s="40" t="n">
-        <v>145</v>
-      </c>
-      <c r="C98" s="47" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C98" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D98" s="42" t="inlineStr">
@@ -5430,7 +5433,7 @@
       </c>
       <c r="F98" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Be Legendary”</t>
+          <t>Nike Air Max 95 “ACG”</t>
         </is>
       </c>
     </row>
@@ -5439,11 +5442,11 @@
         <v>46346</v>
       </c>
       <c r="B99" s="37" t="n">
-        <v>190</v>
-      </c>
-      <c r="C99" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>145</v>
+      </c>
+      <c r="C99" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D99" s="41" t="inlineStr">
@@ -5458,7 +5461,7 @@
       </c>
       <c r="F99" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “ACG”</t>
+          <t>Nike Book 2 “Be Legendary”</t>
         </is>
       </c>
     </row>
@@ -5495,7 +5498,7 @@
         <v>46347</v>
       </c>
       <c r="B101" s="37" t="n">
-        <v>215</v>
+        <v>125</v>
       </c>
       <c r="C101" s="36" t="inlineStr">
         <is>
@@ -5509,12 +5512,12 @@
       </c>
       <c r="E101" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5523,7 +5526,7 @@
         <v>46347</v>
       </c>
       <c r="B102" s="40" t="n">
-        <v>125</v>
+        <v>155</v>
       </c>
       <c r="C102" s="39" t="inlineStr">
         <is>
@@ -5542,7 +5545,7 @@
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -5550,17 +5553,15 @@
       <c r="A103" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B103" s="37" t="n">
-        <v>155</v>
-      </c>
+      <c r="B103" s="37" t="inlineStr"/>
       <c r="C103" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D103" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D103" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E103" s="34" t="inlineStr">
@@ -5570,7 +5571,7 @@
       </c>
       <c r="F103" s="34" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
         </is>
       </c>
     </row>
@@ -5578,25 +5579,27 @@
       <c r="A104" s="31" t="n">
         <v>46347</v>
       </c>
-      <c r="B104" s="40" t="inlineStr"/>
+      <c r="B104" s="40" t="n">
+        <v>165</v>
+      </c>
       <c r="C104" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D104" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D104" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E104" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -5605,26 +5608,26 @@
         <v>46347</v>
       </c>
       <c r="B105" s="37" t="n">
-        <v>165</v>
+        <v>230</v>
       </c>
       <c r="C105" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D105" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D105" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E105" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -5633,26 +5636,26 @@
         <v>46347</v>
       </c>
       <c r="B106" s="40" t="n">
-        <v>230</v>
-      </c>
-      <c r="C106" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D106" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>135</v>
+      </c>
+      <c r="C106" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D106" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E106" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Jordan Tatum 5 “Sunset”</t>
         </is>
       </c>
     </row>
@@ -5660,12 +5663,10 @@
       <c r="A107" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B107" s="37" t="n">
-        <v>135</v>
-      </c>
-      <c r="C107" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="B107" s="37" t="inlineStr"/>
+      <c r="C107" s="49" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D107" s="41" t="inlineStr">
@@ -5675,12 +5676,12 @@
       </c>
       <c r="E107" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F107" s="34" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunset”</t>
+          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
         </is>
       </c>
     </row>
@@ -5688,10 +5689,12 @@
       <c r="A108" s="31" t="n">
         <v>46347</v>
       </c>
-      <c r="B108" s="40" t="inlineStr"/>
-      <c r="C108" s="52" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B108" s="40" t="n">
+        <v>150</v>
+      </c>
+      <c r="C108" s="47" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D108" s="42" t="inlineStr">
@@ -5701,12 +5704,12 @@
       </c>
       <c r="E108" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F108" s="30" t="inlineStr">
         <is>
-          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
+          <t>Jordan Triangle “Paolo Banchero”</t>
         </is>
       </c>
     </row>
@@ -5715,7 +5718,7 @@
         <v>46347</v>
       </c>
       <c r="B109" s="37" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C109" s="53" t="inlineStr">
         <is>
@@ -5729,12 +5732,12 @@
       </c>
       <c r="E109" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F109" s="34" t="inlineStr">
         <is>
-          <t>Jordan Triangle “Paolo Banchero”</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -5743,7 +5746,7 @@
         <v>46347</v>
       </c>
       <c r="B110" s="40" t="n">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="C110" s="47" t="inlineStr">
         <is>
@@ -5762,7 +5765,7 @@
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Nike Zoom Hyperflight “Safari”</t>
         </is>
       </c>
     </row>
@@ -5771,11 +5774,11 @@
         <v>46347</v>
       </c>
       <c r="B111" s="37" t="n">
-        <v>190</v>
-      </c>
-      <c r="C111" s="53" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C111" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D111" s="41" t="inlineStr">
@@ -5785,12 +5788,12 @@
       </c>
       <c r="E111" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F111" s="34" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Safari”</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -6920,7 +6923,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F78"/>
+  <dimension ref="A1:F79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6946,7 +6949,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="51" t="inlineStr">
         <is>
-          <t>Generated October 08, 2026  ·  13:00 UTC</t>
+          <t>Generated October 09, 2026  ·  12:46 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -7776,7 +7779,7 @@
         <v>46331</v>
       </c>
       <c r="B32" s="40" t="n">
-        <v>165</v>
+        <v>140</v>
       </c>
       <c r="C32" s="39" t="inlineStr">
         <is>
@@ -7795,7 +7798,7 @@
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Mid “Space Jam”</t>
+          <t>Air Jordan 1 Mid “Space Jam Hare”</t>
         </is>
       </c>
     </row>
@@ -7804,7 +7807,7 @@
         <v>46331</v>
       </c>
       <c r="B33" s="37" t="n">
-        <v>155</v>
+        <v>165</v>
       </c>
       <c r="C33" s="36" t="inlineStr">
         <is>
@@ -7823,7 +7826,7 @@
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Lola Bunny”</t>
+          <t>Air Jordan 1 Mid “Space Jam”</t>
         </is>
       </c>
     </row>
@@ -7832,7 +7835,7 @@
         <v>46331</v>
       </c>
       <c r="B34" s="40" t="n">
-        <v>130</v>
+        <v>155</v>
       </c>
       <c r="C34" s="39" t="inlineStr">
         <is>
@@ -7851,16 +7854,16 @@
       </c>
       <c r="F34" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Magic Ball”</t>
+          <t>Air Jordan 3 “Lola Bunny”</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
       <c r="A35" s="35" t="n">
-        <v>46333</v>
+        <v>46331</v>
       </c>
       <c r="B35" s="37" t="n">
-        <v>215</v>
+        <v>130</v>
       </c>
       <c r="C35" s="36" t="inlineStr">
         <is>
@@ -7879,7 +7882,7 @@
       </c>
       <c r="F35" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 6 “White Infrared” 2026</t>
+          <t>Air Jordan 1 Low “Magic Ball”</t>
         </is>
       </c>
     </row>
@@ -7888,7 +7891,7 @@
         <v>46333</v>
       </c>
       <c r="B36" s="40" t="n">
-        <v>245</v>
+        <v>240</v>
       </c>
       <c r="C36" s="39" t="inlineStr">
         <is>
@@ -7907,7 +7910,7 @@
       </c>
       <c r="F36" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 17 Low “Black Pack”</t>
+          <t>Air Jordan 15 “Snakeskin”</t>
         </is>
       </c>
     </row>
@@ -7916,16 +7919,16 @@
         <v>46333</v>
       </c>
       <c r="B37" s="37" t="n">
-        <v>240</v>
+        <v>215</v>
       </c>
       <c r="C37" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D37" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E37" s="34" t="inlineStr">
@@ -7935,35 +7938,35 @@
       </c>
       <c r="F37" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 15 “Snakeskin”</t>
+          <t>Air Jordan 6 “White Infrared” 2026</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
       <c r="A38" s="31" t="n">
-        <v>46337</v>
+        <v>46333</v>
       </c>
       <c r="B38" s="40" t="n">
-        <v>200</v>
+        <v>245</v>
       </c>
       <c r="C38" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D38" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D38" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E38" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F38" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
+          <t>Air Jordan 17 Low “Black Pack”</t>
         </is>
       </c>
     </row>
@@ -7972,7 +7975,7 @@
         <v>46337</v>
       </c>
       <c r="B39" s="37" t="n">
-        <v>235</v>
+        <v>200</v>
       </c>
       <c r="C39" s="36" t="inlineStr">
         <is>
@@ -7986,21 +7989,21 @@
       </c>
       <c r="E39" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F39" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Magic Ball”</t>
+          <t>Nike Kobe 8 Protro “Shanghai Fireworks”</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
       <c r="A40" s="31" t="n">
-        <v>46339</v>
+        <v>46337</v>
       </c>
       <c r="B40" s="40" t="n">
-        <v>240</v>
+        <v>235</v>
       </c>
       <c r="C40" s="39" t="inlineStr">
         <is>
@@ -8014,12 +8017,12 @@
       </c>
       <c r="E40" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F40" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Mummy”</t>
+          <t>Air Jordan 11 “Magic Ball”</t>
         </is>
       </c>
     </row>
@@ -8047,41 +8050,41 @@
       </c>
       <c r="F41" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Phantom”</t>
+          <t>Nike Air Foamposite One “Mummy”</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15" customHeight="1">
       <c r="A42" s="31" t="n">
-        <v>46340</v>
+        <v>46339</v>
       </c>
       <c r="B42" s="40" t="n">
-        <v>255</v>
+        <v>240</v>
       </c>
       <c r="C42" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D42" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D42" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Nike Air Foamposite One “Phantom”</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="35" t="n">
-        <v>46342</v>
+        <v>46340</v>
       </c>
       <c r="B43" s="37" t="n">
         <v>255</v>
@@ -8103,7 +8106,7 @@
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam Galaxy”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -8112,7 +8115,7 @@
         <v>46342</v>
       </c>
       <c r="B44" s="40" t="n">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C44" s="39" t="inlineStr">
         <is>
@@ -8126,30 +8129,30 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
+          <t>Air Jordan 11 “Space Jam Galaxy”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="35" t="n">
-        <v>46343</v>
+        <v>46342</v>
       </c>
       <c r="B45" s="37" t="n">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="C45" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D45" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D45" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E45" s="34" t="inlineStr">
@@ -8159,16 +8162,16 @@
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Stars”</t>
+          <t>Nike Air Foamposite Pro “Mummy Duck”</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15" customHeight="1">
       <c r="A46" s="31" t="n">
-        <v>46346</v>
+        <v>46343</v>
       </c>
       <c r="B46" s="40" t="n">
-        <v>190</v>
+        <v>200</v>
       </c>
       <c r="C46" s="39" t="inlineStr">
         <is>
@@ -8187,16 +8190,16 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “ACG”</t>
+          <t>Nike LeBron 24 “Stars”</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15" customHeight="1">
       <c r="A47" s="35" t="n">
-        <v>46347</v>
+        <v>46346</v>
       </c>
       <c r="B47" s="37" t="n">
-        <v>215</v>
+        <v>190</v>
       </c>
       <c r="C47" s="36" t="inlineStr">
         <is>
@@ -8210,12 +8213,12 @@
       </c>
       <c r="E47" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F47" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Nike Air Max 95 “ACG”</t>
         </is>
       </c>
     </row>
@@ -8359,10 +8362,10 @@
     </row>
     <row r="53" ht="15" customHeight="1">
       <c r="A53" s="35" t="n">
-        <v>46353</v>
+        <v>46347</v>
       </c>
       <c r="B53" s="37" t="n">
-        <v>230</v>
+        <v>215</v>
       </c>
       <c r="C53" s="36" t="inlineStr">
         <is>
@@ -8381,7 +8384,7 @@
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -8390,7 +8393,7 @@
         <v>46353</v>
       </c>
       <c r="B54" s="40" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C54" s="39" t="inlineStr">
         <is>
@@ -8404,30 +8407,30 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="35" t="n">
-        <v>46354</v>
+        <v>46353</v>
       </c>
       <c r="B55" s="37" t="n">
-        <v>130</v>
+        <v>240</v>
       </c>
       <c r="C55" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="34" t="inlineStr">
@@ -8437,7 +8440,7 @@
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -8446,7 +8449,7 @@
         <v>46354</v>
       </c>
       <c r="B56" s="40" t="n">
-        <v>240</v>
+        <v>130</v>
       </c>
       <c r="C56" s="39" t="inlineStr">
         <is>
@@ -8465,7 +8468,7 @@
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “FSU”</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -8473,15 +8476,17 @@
       <c r="A57" s="35" t="n">
         <v>46354</v>
       </c>
-      <c r="B57" s="37" t="inlineStr"/>
+      <c r="B57" s="37" t="n">
+        <v>240</v>
+      </c>
       <c r="C57" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D57" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D57" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E57" s="34" t="inlineStr">
@@ -8491,7 +8496,7 @@
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike Air Foamposite Pro “FSU”</t>
         </is>
       </c>
     </row>
@@ -8500,24 +8505,24 @@
         <v>46354</v>
       </c>
       <c r="B58" s="40" t="inlineStr"/>
-      <c r="C58" s="32" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D58" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C58" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D58" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -8526,34 +8531,32 @@
         <v>46354</v>
       </c>
       <c r="B59" s="37" t="inlineStr"/>
-      <c r="C59" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D59" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C59" s="55" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D59" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E59" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F59" s="34" t="inlineStr">
         <is>
-          <t>Slam Jam x Nike Air Max 97</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
     <row r="60" ht="15" customHeight="1">
       <c r="A60" s="31" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B60" s="40" t="n">
-        <v>190</v>
-      </c>
+        <v>46354</v>
+      </c>
+      <c r="B60" s="40" t="inlineStr"/>
       <c r="C60" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8571,16 +8574,16 @@
       </c>
       <c r="F60" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Chosen 1s”</t>
+          <t>Slam Jam x Nike Air Max 97</t>
         </is>
       </c>
     </row>
     <row r="61" ht="15" customHeight="1">
       <c r="A61" s="35" t="n">
-        <v>46361</v>
+        <v>46357</v>
       </c>
       <c r="B61" s="37" t="n">
-        <v>155</v>
+        <v>190</v>
       </c>
       <c r="C61" s="36" t="inlineStr">
         <is>
@@ -8599,7 +8602,7 @@
       </c>
       <c r="F61" s="34" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Laser Orange”</t>
+          <t>Nike LeBron 24 “Chosen 1s”</t>
         </is>
       </c>
     </row>
@@ -8608,7 +8611,7 @@
         <v>46361</v>
       </c>
       <c r="B62" s="40" t="n">
-        <v>215</v>
+        <v>155</v>
       </c>
       <c r="C62" s="39" t="inlineStr">
         <is>
@@ -8622,12 +8625,12 @@
       </c>
       <c r="E62" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F62" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>Nike Kobe AD Protro “Laser Orange”</t>
         </is>
       </c>
     </row>
@@ -8636,7 +8639,7 @@
         <v>46361</v>
       </c>
       <c r="B63" s="37" t="n">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C63" s="36" t="inlineStr">
         <is>
@@ -8655,16 +8658,16 @@
       </c>
       <c r="F63" s="34" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
     <row r="64" ht="15" customHeight="1">
       <c r="A64" s="31" t="n">
-        <v>46367</v>
+        <v>46361</v>
       </c>
       <c r="B64" s="40" t="n">
-        <v>240</v>
+        <v>225</v>
       </c>
       <c r="C64" s="39" t="inlineStr">
         <is>
@@ -8678,12 +8681,12 @@
       </c>
       <c r="E64" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F64" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
@@ -8692,26 +8695,26 @@
         <v>46367</v>
       </c>
       <c r="B65" s="37" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C65" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D65" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D65" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E65" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F65" s="34" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -8719,7 +8722,9 @@
       <c r="A66" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B66" s="40" t="inlineStr"/>
+      <c r="B66" s="40" t="n">
+        <v>150</v>
+      </c>
       <c r="C66" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8737,7 +8742,7 @@
       </c>
       <c r="F66" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -8745,45 +8750,43 @@
       <c r="A67" s="35" t="n">
         <v>46367</v>
       </c>
-      <c r="B67" s="37" t="n">
-        <v>190</v>
-      </c>
+      <c r="B67" s="37" t="inlineStr"/>
       <c r="C67" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D67" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D67" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E67" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F67" s="34" t="inlineStr">
         <is>
-          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
     <row r="68" ht="15" customHeight="1">
       <c r="A68" s="31" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="B68" s="40" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="C68" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D68" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D68" s="42" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E68" s="30" t="inlineStr">
@@ -8793,7 +8796,7 @@
       </c>
       <c r="F68" s="30" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low “Midnight Navy”</t>
+          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
         </is>
       </c>
     </row>
@@ -8802,35 +8805,35 @@
         <v>46368</v>
       </c>
       <c r="B69" s="37" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C69" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D69" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D69" s="38" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E69" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>APB x Nike Dunk Low “Midnight Navy”</t>
         </is>
       </c>
     </row>
     <row r="70" ht="15" customHeight="1">
       <c r="A70" s="31" t="n">
-        <v>46374</v>
+        <v>46368</v>
       </c>
       <c r="B70" s="40" t="n">
-        <v>200</v>
+        <v>235</v>
       </c>
       <c r="C70" s="39" t="inlineStr">
         <is>
@@ -8849,35 +8852,35 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>APB x Air Jordan 11 Low</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
     <row r="71" ht="15" customHeight="1">
       <c r="A71" s="35" t="n">
-        <v>46375</v>
+        <v>46374</v>
       </c>
       <c r="B71" s="37" t="n">
-        <v>350</v>
+        <v>200</v>
       </c>
       <c r="C71" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D71" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D71" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E71" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
-          <t>Victor Solomon x Nike Air Foamposite One “Trophies Red”</t>
+          <t>APB x Air Jordan 11 Low</t>
         </is>
       </c>
     </row>
@@ -8886,26 +8889,26 @@
         <v>46375</v>
       </c>
       <c r="B72" s="40" t="n">
-        <v>220</v>
+        <v>350</v>
       </c>
       <c r="C72" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D72" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D72" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E72" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F72" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Victor Solomon x Nike Air Foamposite One “Trophies Red”</t>
         </is>
       </c>
     </row>
@@ -8914,44 +8917,44 @@
         <v>46375</v>
       </c>
       <c r="B73" s="37" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C73" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D73" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D73" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E73" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F73" s="34" t="inlineStr">
         <is>
-          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
+          <t>Air Jordan 4 “Pink Thunder”</t>
         </is>
       </c>
     </row>
     <row r="74" ht="15" customHeight="1">
       <c r="A74" s="31" t="n">
-        <v>46381</v>
+        <v>46375</v>
       </c>
       <c r="B74" s="40" t="n">
-        <v>190</v>
+        <v>120</v>
       </c>
       <c r="C74" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D74" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D74" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E74" s="30" t="inlineStr">
@@ -8961,35 +8964,35 @@
       </c>
       <c r="F74" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 6 Protro “Coals”</t>
+          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
         </is>
       </c>
     </row>
     <row r="75" ht="15" customHeight="1">
       <c r="A75" s="35" t="n">
-        <v>46382</v>
+        <v>46381</v>
       </c>
       <c r="B75" s="37" t="n">
-        <v>355</v>
+        <v>190</v>
       </c>
       <c r="C75" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D75" s="38" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D75" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E75" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F75" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “BIN 23”</t>
+          <t>Nike Kobe 6 Protro “Coals”</t>
         </is>
       </c>
     </row>
@@ -8998,7 +9001,7 @@
         <v>46382</v>
       </c>
       <c r="B76" s="40" t="n">
-        <v>150</v>
+        <v>355</v>
       </c>
       <c r="C76" s="39" t="inlineStr">
         <is>
@@ -9012,21 +9015,21 @@
       </c>
       <c r="E76" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F76" s="30" t="inlineStr">
         <is>
-          <t>Supreme x Martine Rose x Nike Dunk Low</t>
+          <t>Air Jordan 4 “BIN 23”</t>
         </is>
       </c>
     </row>
     <row r="77" ht="15" customHeight="1">
       <c r="A77" s="35" t="n">
-        <v>46387</v>
+        <v>46382</v>
       </c>
       <c r="B77" s="37" t="n">
-        <v>215</v>
+        <v>150</v>
       </c>
       <c r="C77" s="36" t="inlineStr">
         <is>
@@ -9040,12 +9043,12 @@
       </c>
       <c r="E77" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F77" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Middle East”</t>
+          <t>Supreme x Martine Rose x Nike Dunk Low</t>
         </is>
       </c>
     </row>
@@ -9054,31 +9057,59 @@
         <v>46387</v>
       </c>
       <c r="B78" s="40" t="n">
+        <v>215</v>
+      </c>
+      <c r="C78" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D78" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
+        </is>
+      </c>
+      <c r="E78" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F78" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 3 “Middle East”</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="15" customHeight="1">
+      <c r="A79" s="35" t="n">
+        <v>46387</v>
+      </c>
+      <c r="B79" s="37" t="n">
         <v>190</v>
       </c>
-      <c r="C78" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D78" s="42" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E78" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F78" s="30" t="inlineStr">
+      <c r="C79" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D79" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E79" s="34" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F79" s="34" t="inlineStr">
         <is>
           <t>Nike Kobe 9 EM Low Protro “Philippines”</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:F78"/>
+  <autoFilter ref="A3:F79"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>

<commit_message>
chore: sneaker release update [2026-10-17 10:19 UTC]
</commit_message>
<xml_diff>
--- a/docs/data/sneaker_releases.xlsx
+++ b/docs/data/sneaker_releases.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="High Hype Alerts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$150</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All Releases'!$A$3:$F$152</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'High Hype Alerts'!$A$3:$F$82</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -673,19 +673,19 @@
     <xf numFmtId="0" fontId="18" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="17" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="15" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="3" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="25" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1581,7 +1581,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Generated October 16, 2026  ·  10:56 UTC</t>
+          <t>Generated October 17, 2026  ·  10:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -1621,20 +1621,20 @@
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="12" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="B5" s="13" t="n"/>
       <c r="C5" s="14" t="n">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="D5" s="15" t="n"/>
       <c r="E5" s="16" t="n">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="F5" s="17" t="n"/>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>$178</t>
+          <t>$177</t>
         </is>
       </c>
       <c r="H5" s="19" t="n"/>
@@ -1737,7 +1737,7 @@
         <v>46354</v>
       </c>
       <c r="D10" s="30" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="E10" s="32" t="inlineStr">
         <is>
@@ -1757,16 +1757,16 @@
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="C11" s="35" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="D11" s="34" t="n">
         <v>0</v>
@@ -1780,7 +1780,7 @@
         <v>7</v>
       </c>
       <c r="G11" s="37" t="n">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="H11" s="38" t="inlineStr">
         <is>
@@ -1791,7 +1791,7 @@
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Nocturnal x Nike SB Air Force 1 Low</t>
         </is>
       </c>
       <c r="B12" s="30" t="inlineStr">
@@ -1800,7 +1800,7 @@
         </is>
       </c>
       <c r="C12" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="D12" s="30" t="n">
         <v>0</v>
@@ -1814,7 +1814,7 @@
         <v>7</v>
       </c>
       <c r="G12" s="40" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="H12" s="41" t="inlineStr">
         <is>
@@ -1825,19 +1825,19 @@
     <row r="13" ht="15" customHeight="1">
       <c r="A13" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="C13" s="35" t="n">
-        <v>46312</v>
+        <v>46316</v>
       </c>
       <c r="D13" s="34" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E13" s="36" t="inlineStr">
         <is>
@@ -1848,7 +1848,7 @@
         <v>7</v>
       </c>
       <c r="G13" s="37" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="H13" s="38" t="inlineStr">
         <is>
@@ -1859,7 +1859,7 @@
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="30" t="inlineStr">
         <is>
-          <t>Nocturnal x Nike SB Air Force 1 Low</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
       <c r="B14" s="30" t="inlineStr">
@@ -1868,10 +1868,10 @@
         </is>
       </c>
       <c r="C14" s="31" t="n">
-        <v>46312</v>
+        <v>46317</v>
       </c>
       <c r="D14" s="30" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E14" s="39" t="inlineStr">
         <is>
@@ -1882,18 +1882,18 @@
         <v>7</v>
       </c>
       <c r="G14" s="40" t="n">
-        <v>120</v>
-      </c>
-      <c r="H14" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="H14" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Nike Air Force 1 “What The LA”</t>
         </is>
       </c>
       <c r="B15" s="34" t="inlineStr">
@@ -1902,7 +1902,7 @@
         </is>
       </c>
       <c r="C15" s="35" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="D15" s="34" t="n">
         <v>5</v>
@@ -1916,7 +1916,7 @@
         <v>7</v>
       </c>
       <c r="G15" s="37" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="H15" s="38" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 “What The LA”</t>
+          <t>Nike Air Force 1 Low “What The LA”</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
@@ -1939,7 +1939,7 @@
         <v>46317</v>
       </c>
       <c r="D16" s="30" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E16" s="39" t="inlineStr">
         <is>
@@ -2012,7 +2012,7 @@
         </is>
       </c>
       <c r="B20" s="30" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D20" s="32" t="inlineStr">
         <is>
@@ -2038,7 +2038,7 @@
         </is>
       </c>
       <c r="B21" s="34" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D21" s="36" t="inlineStr">
         <is>
@@ -2046,7 +2046,7 @@
         </is>
       </c>
       <c r="E21" s="34" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G21" s="45" t="inlineStr">
         <is>
@@ -2054,7 +2054,7 @@
         </is>
       </c>
       <c r="H21" s="34" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
@@ -2072,7 +2072,7 @@
         </is>
       </c>
       <c r="E22" s="30" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G22" s="47" t="inlineStr">
         <is>
@@ -2090,7 +2090,7 @@
         </is>
       </c>
       <c r="B23" s="34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D23" s="48" t="inlineStr">
         <is>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="E23" s="34" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" ht="15" customHeight="1">
@@ -2171,17 +2171,17 @@
       </c>
       <c r="B29" s="30" t="inlineStr">
         <is>
-          <t>10/16 – 10/22</t>
+          <t>10/17 – 10/23</t>
         </is>
       </c>
       <c r="C29" s="30" t="n">
-        <v>13</v>
+        <v>28</v>
       </c>
       <c r="D29" s="39" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="E29" s="30" t="n">
-        <v>5.6</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
@@ -2192,17 +2192,17 @@
       </c>
       <c r="B30" s="34" t="inlineStr">
         <is>
-          <t>10/23 – 10/29</t>
+          <t>10/24 – 10/30</t>
         </is>
       </c>
       <c r="C30" s="34" t="n">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D30" s="36" t="n">
         <v>16</v>
       </c>
       <c r="E30" s="34" t="n">
-        <v>5.4</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="31" ht="15" customHeight="1">
@@ -2213,14 +2213,14 @@
       </c>
       <c r="B31" s="30" t="inlineStr">
         <is>
-          <t>10/30 – 11/5</t>
+          <t>10/31 – 11/6</t>
         </is>
       </c>
       <c r="C31" s="30" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D31" s="39" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="E31" s="30" t="n">
         <v>5.5</v>
@@ -2234,17 +2234,17 @@
       </c>
       <c r="B32" s="34" t="inlineStr">
         <is>
-          <t>11/6 – 11/12</t>
+          <t>11/7 – 11/13</t>
         </is>
       </c>
       <c r="C32" s="34" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D32" s="36" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E32" s="34" t="n">
-        <v>5.5</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
@@ -2255,17 +2255,17 @@
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t>11/13 – 11/19</t>
+          <t>11/14 – 11/20</t>
         </is>
       </c>
       <c r="C33" s="30" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D33" s="39" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E33" s="30" t="n">
-        <v>5.3</v>
+        <v>5.1</v>
       </c>
     </row>
     <row r="34" ht="15" customHeight="1">
@@ -2276,17 +2276,17 @@
       </c>
       <c r="B34" s="34" t="inlineStr">
         <is>
-          <t>11/20 – 11/26</t>
+          <t>11/21 – 11/27</t>
         </is>
       </c>
       <c r="C34" s="34" t="n">
         <v>14</v>
       </c>
       <c r="D34" s="36" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E34" s="34" t="n">
-        <v>5.5</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="35" ht="15" customHeight="1">
@@ -2297,17 +2297,17 @@
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t>11/27 – 12/3</t>
+          <t>11/28 – 12/4</t>
         </is>
       </c>
       <c r="C35" s="30" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D35" s="39" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E35" s="30" t="n">
-        <v>6.1</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36" ht="15" customHeight="1">
@@ -2318,17 +2318,17 @@
       </c>
       <c r="B36" s="34" t="inlineStr">
         <is>
-          <t>12/4 – 12/10</t>
+          <t>12/5 – 12/11</t>
         </is>
       </c>
       <c r="C36" s="34" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="D36" s="36" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E36" s="34" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="37" ht="15" customHeight="1">
@@ -2339,17 +2339,17 @@
       </c>
       <c r="B37" s="30" t="inlineStr">
         <is>
-          <t>12/11 – 12/17</t>
+          <t>12/12 – 12/18</t>
         </is>
       </c>
       <c r="C37" s="30" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="D37" s="39" t="n">
+        <v>2</v>
+      </c>
+      <c r="E37" s="30" t="n">
         <v>6</v>
-      </c>
-      <c r="E37" s="30" t="n">
-        <v>6.6</v>
       </c>
     </row>
     <row r="38" ht="15" customHeight="1">
@@ -2360,17 +2360,17 @@
       </c>
       <c r="B38" s="34" t="inlineStr">
         <is>
-          <t>12/18 – 12/24</t>
+          <t>12/19 – 12/25</t>
         </is>
       </c>
       <c r="C38" s="34" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="D38" s="36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E38" s="34" t="n">
-        <v>5.6</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="39" ht="15" customHeight="1">
@@ -2381,17 +2381,17 @@
       </c>
       <c r="B39" s="30" t="inlineStr">
         <is>
-          <t>12/25 – 12/31</t>
+          <t>12/26 – 1/1</t>
         </is>
       </c>
       <c r="C39" s="30" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D39" s="39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E39" s="30" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="40" ht="15" customHeight="1">
@@ -2402,7 +2402,7 @@
       </c>
       <c r="B40" s="34" t="inlineStr">
         <is>
-          <t>1/1 – 1/7</t>
+          <t>1/2 – 1/8</t>
         </is>
       </c>
       <c r="C40" s="34" t="n">
@@ -2423,16 +2423,18 @@
       </c>
       <c r="B41" s="30" t="inlineStr">
         <is>
-          <t>1/8 – 1/14</t>
+          <t>1/9 – 1/15</t>
         </is>
       </c>
       <c r="C41" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="D41" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" s="30" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D41" s="39" t="n">
+        <v>1</v>
+      </c>
+      <c r="E41" s="30" t="n">
+        <v>7</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="17">
@@ -2529,7 +2531,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -2563,7 +2565,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -2571,7 +2573,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -2579,7 +2581,7 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -2605,7 +2607,7 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -2621,7 +2623,7 @@
         </is>
       </c>
       <c r="K4" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="5">
@@ -2631,7 +2633,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -2639,7 +2641,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2647,7 +2649,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -2690,7 +2692,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F150"/>
+  <dimension ref="A1:F152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2716,7 +2718,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Generated October 16, 2026  ·  10:56 UTC</t>
+          <t>Generated October 17, 2026  ·  10:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -2759,10 +2761,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B4" s="40" t="n">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="C4" s="39" t="inlineStr">
         <is>
@@ -2776,25 +2778,25 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="35" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B5" s="37" t="n">
-        <v>195</v>
-      </c>
-      <c r="C5" s="48" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>120</v>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D5" s="38" t="inlineStr">
@@ -2804,25 +2806,25 @@
       </c>
       <c r="E5" s="34" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
-          <t>Satoshi Nakamoto x Vans Era “Gems”</t>
+          <t>Nocturnal x Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B6" s="40" t="n">
-        <v>250</v>
-      </c>
-      <c r="C6" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>140</v>
+      </c>
+      <c r="C6" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D6" s="41" t="inlineStr">
@@ -2832,25 +2834,25 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Bad Bunny x adidas Gazelle Indoor “Solar Gold”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="35" t="n">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B7" s="37" t="n">
-        <v>215</v>
-      </c>
-      <c r="C7" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>160</v>
+      </c>
+      <c r="C7" s="48" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D7" s="38" t="inlineStr">
@@ -2860,25 +2862,25 @@
       </c>
       <c r="E7" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Reebok Angel Reese 1 “Reese’s”</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46312</v>
+        <v>46315</v>
       </c>
       <c r="B8" s="40" t="n">
-        <v>120</v>
-      </c>
-      <c r="C8" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>180</v>
+      </c>
+      <c r="C8" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D8" s="41" t="inlineStr">
@@ -2888,25 +2890,25 @@
       </c>
       <c r="E8" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nocturnal x Nike SB Air Force 1 Low</t>
+          <t>MENACE x adidas Adistar Control 5 “Heat Signature”</t>
         </is>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
       <c r="A9" s="35" t="n">
-        <v>46312</v>
+        <v>46316</v>
       </c>
       <c r="B9" s="37" t="n">
         <v>140</v>
       </c>
-      <c r="C9" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+      <c r="C9" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D9" s="38" t="inlineStr">
@@ -2916,50 +2918,48 @@
       </c>
       <c r="E9" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
-          <t>Bad Bunny x adidas Gazelle Indoor “Solar Gold”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46315</v>
+        <v>46317</v>
       </c>
       <c r="B10" s="40" t="n">
-        <v>160</v>
-      </c>
-      <c r="C10" s="52" t="inlineStr">
-        <is>
-          <t>LOW</t>
-        </is>
-      </c>
-      <c r="D10" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>150</v>
+      </c>
+      <c r="C10" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D10" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E10" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>Reebok Angel Reese 1 “Reese’s”</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="35" t="n">
-        <v>46315</v>
-      </c>
-      <c r="B11" s="37" t="n">
-        <v>180</v>
-      </c>
+        <v>46317</v>
+      </c>
+      <c r="B11" s="37" t="inlineStr"/>
       <c r="C11" s="48" t="inlineStr">
         <is>
           <t>LOW</t>
@@ -2972,21 +2972,21 @@
       </c>
       <c r="E11" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Vans</t>
         </is>
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
-          <t>MENACE x adidas Adistar Control 5 “Heat Signature”</t>
+          <t>SZA x Vans VANSZA Collection</t>
         </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1">
       <c r="A12" s="31" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B12" s="40" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Nike Air Force 1 “What The LA”</t>
         </is>
       </c>
     </row>
@@ -3013,10 +3013,12 @@
       <c r="A13" s="35" t="n">
         <v>46317</v>
       </c>
-      <c r="B13" s="37" t="inlineStr"/>
-      <c r="C13" s="48" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B13" s="37" t="n">
+        <v>125</v>
+      </c>
+      <c r="C13" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D13" s="38" t="inlineStr">
@@ -3026,25 +3028,25 @@
       </c>
       <c r="E13" s="34" t="inlineStr">
         <is>
-          <t>Vans</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
-          <t>SZA x Vans VANSZA Collection</t>
+          <t>Nike Air Force 1 Low “What The LA”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B14" s="40" t="n">
-        <v>125</v>
-      </c>
-      <c r="C14" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>165</v>
+      </c>
+      <c r="C14" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D14" s="41" t="inlineStr">
@@ -3059,23 +3061,23 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 “What The LA”</t>
+          <t>Nike KD 19 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B15" s="37" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C15" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="53" t="inlineStr">
+      <c r="D15" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3087,20 +3089,20 @@
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Nike Dunk Low “Shibuya Halloween”</t>
         </is>
       </c>
     </row>
     <row r="16" ht="15" customHeight="1">
       <c r="A16" s="31" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B16" s="40" t="n">
-        <v>125</v>
-      </c>
-      <c r="C16" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>150</v>
+      </c>
+      <c r="C16" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D16" s="41" t="inlineStr">
@@ -3115,7 +3117,7 @@
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “What The LA”</t>
+          <t>Nike Caitlin 1 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3124,9 +3126,9 @@
         <v>46318</v>
       </c>
       <c r="B17" s="37" t="n">
-        <v>150</v>
-      </c>
-      <c r="C17" s="51" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C17" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3143,7 +3145,7 @@
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Halloween”</t>
+          <t>Nike Ja 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3152,7 +3154,7 @@
         <v>46318</v>
       </c>
       <c r="B18" s="40" t="n">
-        <v>140</v>
+        <v>210</v>
       </c>
       <c r="C18" s="46" t="inlineStr">
         <is>
@@ -3171,7 +3173,7 @@
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Nike Ja 4 “Halloween”</t>
+          <t>Victor Wembanyama x Nike GT Cut 4 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -3210,7 +3212,7 @@
       <c r="B20" s="40" t="n">
         <v>150</v>
       </c>
-      <c r="C20" s="52" t="inlineStr">
+      <c r="C20" s="51" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -3294,7 +3296,7 @@
       <c r="B23" s="37" t="n">
         <v>145</v>
       </c>
-      <c r="C23" s="51" t="inlineStr">
+      <c r="C23" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3350,7 +3352,7 @@
       <c r="B25" s="37" t="n">
         <v>170</v>
       </c>
-      <c r="C25" s="51" t="inlineStr">
+      <c r="C25" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3406,7 +3408,7 @@
       <c r="B27" s="37" t="n">
         <v>145</v>
       </c>
-      <c r="C27" s="51" t="inlineStr">
+      <c r="C27" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3460,11 +3462,11 @@
         <v>46318</v>
       </c>
       <c r="B29" s="37" t="n">
-        <v>165</v>
-      </c>
-      <c r="C29" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>130</v>
+      </c>
+      <c r="C29" s="48" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D29" s="38" t="inlineStr">
@@ -3474,12 +3476,12 @@
       </c>
       <c r="E29" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Puma</t>
         </is>
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
-          <t>Nike KD 19 “Halloween”</t>
+          <t>PUMA Hali 1 “Pacers”</t>
         </is>
       </c>
     </row>
@@ -3488,26 +3490,26 @@
         <v>46318</v>
       </c>
       <c r="B30" s="40" t="n">
-        <v>130</v>
-      </c>
-      <c r="C30" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D30" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>150</v>
+      </c>
+      <c r="C30" s="51" t="inlineStr">
+        <is>
+          <t>LOW</t>
+        </is>
+      </c>
+      <c r="D30" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E30" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Reebok</t>
         </is>
       </c>
       <c r="F30" s="30" t="inlineStr">
         <is>
-          <t>Nike Dunk Low “Shibuya Halloween”</t>
+          <t>BBC x Reebok Board Flip “Pumpkin”</t>
         </is>
       </c>
     </row>
@@ -3518,9 +3520,9 @@
       <c r="B31" s="37" t="n">
         <v>130</v>
       </c>
-      <c r="C31" s="48" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="C31" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D31" s="38" t="inlineStr">
@@ -3530,25 +3532,25 @@
       </c>
       <c r="E31" s="34" t="inlineStr">
         <is>
-          <t>Puma</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F31" s="34" t="inlineStr">
         <is>
-          <t>PUMA Hali 1 “Pacers”</t>
+          <t>Nike Giannis Freak 8 “Trick Question”</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15" customHeight="1">
       <c r="A32" s="31" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B32" s="40" t="n">
-        <v>150</v>
-      </c>
-      <c r="C32" s="52" t="inlineStr">
-        <is>
-          <t>LOW</t>
+        <v>190</v>
+      </c>
+      <c r="C32" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D32" s="41" t="inlineStr">
@@ -3558,23 +3560,23 @@
       </c>
       <c r="E32" s="30" t="inlineStr">
         <is>
-          <t>Reebok</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F32" s="30" t="inlineStr">
         <is>
-          <t>BBC x Reebok Board Flip “Pumpkin”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15" customHeight="1">
       <c r="A33" s="35" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B33" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C33" s="51" t="inlineStr">
+        <v>170</v>
+      </c>
+      <c r="C33" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -3591,7 +3593,7 @@
       </c>
       <c r="F33" s="34" t="inlineStr">
         <is>
-          <t>Nike Giannis Freak 8 “Trick Question”</t>
+          <t>Nike Air Diamond Turf 2 “White Black”</t>
         </is>
       </c>
     </row>
@@ -3691,7 +3693,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D37" s="53" t="inlineStr">
+      <c r="D37" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3798,12 +3800,12 @@
       <c r="B41" s="37" t="n">
         <v>170</v>
       </c>
-      <c r="C41" s="51" t="inlineStr">
+      <c r="C41" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D41" s="53" t="inlineStr">
+      <c r="D41" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -3824,11 +3826,11 @@
         <v>46319</v>
       </c>
       <c r="B42" s="40" t="n">
-        <v>190</v>
-      </c>
-      <c r="C42" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>300</v>
+      </c>
+      <c r="C42" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D42" s="41" t="inlineStr">
@@ -3838,25 +3840,25 @@
       </c>
       <c r="E42" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F42" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Pharrell x adidas Adistar Jellyfish</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15" customHeight="1">
       <c r="A43" s="35" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="B43" s="37" t="n">
-        <v>170</v>
-      </c>
-      <c r="C43" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C43" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D43" s="38" t="inlineStr">
@@ -3866,25 +3868,25 @@
       </c>
       <c r="E43" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F43" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Diamond Turf 2 “White Black”</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15" customHeight="1">
       <c r="A44" s="31" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="B44" s="40" t="n">
-        <v>300</v>
-      </c>
-      <c r="C44" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>125</v>
+      </c>
+      <c r="C44" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D44" s="41" t="inlineStr">
@@ -3894,21 +3896,21 @@
       </c>
       <c r="E44" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F44" s="30" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish</t>
+          <t>Nike Air Force 1 Low “University Pack”</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15" customHeight="1">
       <c r="A45" s="35" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="B45" s="37" t="n">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="C45" s="36" t="inlineStr">
         <is>
@@ -3922,12 +3924,12 @@
       </c>
       <c r="E45" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F45" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Force 1 Low “Texas”</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3957,7 @@
       </c>
       <c r="F46" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “University Pack”</t>
+          <t>Nike Air Force 1 Low “Georgia”</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3985,7 @@
       </c>
       <c r="F47" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Texas”</t>
+          <t>Nike Air Force 1 Low “Kentucky”</t>
         </is>
       </c>
     </row>
@@ -4011,16 +4013,16 @@
       </c>
       <c r="F48" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Georgia”</t>
+          <t>Nike Air Force 1 Low “Oregon”</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15" customHeight="1">
       <c r="A49" s="35" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="B49" s="37" t="n">
-        <v>125</v>
+        <v>190</v>
       </c>
       <c r="C49" s="36" t="inlineStr">
         <is>
@@ -4039,25 +4041,25 @@
       </c>
       <c r="F49" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Kentucky”</t>
+          <t>Nike Kobe 3 Low Protro “Mamba Eterno”</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15" customHeight="1">
       <c r="A50" s="31" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="B50" s="40" t="n">
-        <v>125</v>
+        <v>200</v>
       </c>
       <c r="C50" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D50" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D50" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E50" s="30" t="inlineStr">
@@ -4067,7 +4069,7 @@
       </c>
       <c r="F50" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Oregon”</t>
+          <t>Nike LeBron 24 “Storm Drain”</t>
         </is>
       </c>
     </row>
@@ -4076,16 +4078,16 @@
         <v>46325</v>
       </c>
       <c r="B51" s="37" t="n">
-        <v>180</v>
-      </c>
-      <c r="C51" s="51" t="inlineStr">
+        <v>155</v>
+      </c>
+      <c r="C51" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D51" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D51" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E51" s="34" t="inlineStr">
@@ -4095,7 +4097,7 @@
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
-          <t>Nike Ja 4 High “University Red”</t>
+          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
         </is>
       </c>
     </row>
@@ -4104,11 +4106,11 @@
         <v>46325</v>
       </c>
       <c r="B52" s="40" t="n">
-        <v>155</v>
-      </c>
-      <c r="C52" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>205</v>
+      </c>
+      <c r="C52" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D52" s="41" t="inlineStr">
@@ -4118,12 +4120,12 @@
       </c>
       <c r="E52" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Nike Book 2 Halloween “Oogie Boogie”</t>
+          <t>Air Jordan 3 “Fireside”</t>
         </is>
       </c>
     </row>
@@ -4132,11 +4134,11 @@
         <v>46325</v>
       </c>
       <c r="B53" s="37" t="n">
-        <v>205</v>
-      </c>
-      <c r="C53" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>155</v>
+      </c>
+      <c r="C53" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D53" s="38" t="inlineStr">
@@ -4146,12 +4148,12 @@
       </c>
       <c r="E53" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Fireside”</t>
+          <t>Nike Book 2 “Halloween”</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4162,7 @@
         <v>46325</v>
       </c>
       <c r="B54" s="40" t="n">
-        <v>190</v>
+        <v>155</v>
       </c>
       <c r="C54" s="39" t="inlineStr">
         <is>
@@ -4179,20 +4181,20 @@
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Mamba Eterno”</t>
+          <t>Nike Kobe AD Protro “Mamba Eterno”</t>
         </is>
       </c>
     </row>
     <row r="55" ht="15" customHeight="1">
       <c r="A55" s="35" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
       <c r="B55" s="37" t="n">
-        <v>155</v>
-      </c>
-      <c r="C55" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>215</v>
+      </c>
+      <c r="C55" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D55" s="38" t="inlineStr">
@@ -4202,12 +4204,12 @@
       </c>
       <c r="E55" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
-          <t>Nike Book 2 “Halloween”</t>
+          <t>Air Jordan 14 “Forest Green”</t>
         </is>
       </c>
     </row>
@@ -4216,26 +4218,26 @@
         <v>46326</v>
       </c>
       <c r="B56" s="40" t="n">
-        <v>215</v>
-      </c>
-      <c r="C56" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D56" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>180</v>
+      </c>
+      <c r="C56" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D56" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 14 “Forest Green”</t>
+          <t>Nike Ja 4 High “Zombie”</t>
         </is>
       </c>
     </row>
@@ -4246,7 +4248,7 @@
       <c r="B57" s="37" t="n">
         <v>140</v>
       </c>
-      <c r="C57" s="51" t="inlineStr">
+      <c r="C57" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4302,7 +4304,7 @@
       <c r="B59" s="37" t="n">
         <v>165</v>
       </c>
-      <c r="C59" s="51" t="inlineStr">
+      <c r="C59" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4358,7 +4360,7 @@
       <c r="B61" s="37" t="n">
         <v>210</v>
       </c>
-      <c r="C61" s="51" t="inlineStr">
+      <c r="C61" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4470,7 +4472,7 @@
       <c r="B65" s="37" t="n">
         <v>130</v>
       </c>
-      <c r="C65" s="51" t="inlineStr">
+      <c r="C65" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4582,12 +4584,12 @@
       <c r="B69" s="37" t="n">
         <v>265</v>
       </c>
-      <c r="C69" s="51" t="inlineStr">
+      <c r="C69" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D69" s="53" t="inlineStr">
+      <c r="D69" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -4638,7 +4640,7 @@
       <c r="B71" s="37" t="n">
         <v>210</v>
       </c>
-      <c r="C71" s="51" t="inlineStr">
+      <c r="C71" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4694,7 +4696,7 @@
       <c r="B73" s="37" t="n">
         <v>145</v>
       </c>
-      <c r="C73" s="51" t="inlineStr">
+      <c r="C73" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -4753,7 +4755,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D75" s="53" t="inlineStr">
+      <c r="D75" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -4809,7 +4811,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D77" s="53" t="inlineStr">
+      <c r="D77" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -4944,7 +4946,7 @@
       <c r="B82" s="40" t="n">
         <v>130</v>
       </c>
-      <c r="C82" s="52" t="inlineStr">
+      <c r="C82" s="51" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -4972,7 +4974,7 @@
       <c r="B83" s="37" t="n">
         <v>170</v>
       </c>
-      <c r="C83" s="51" t="inlineStr">
+      <c r="C83" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5028,7 +5030,7 @@
       <c r="B85" s="37" t="n">
         <v>170</v>
       </c>
-      <c r="C85" s="51" t="inlineStr">
+      <c r="C85" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -5110,26 +5112,26 @@
         <v>46340</v>
       </c>
       <c r="B88" s="40" t="n">
-        <v>140</v>
-      </c>
-      <c r="C88" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D88" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>255</v>
+      </c>
+      <c r="C88" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D88" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E88" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F88" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
+          <t>Air Jordan 11 “Green Screen”</t>
         </is>
       </c>
     </row>
@@ -5138,16 +5140,16 @@
         <v>46340</v>
       </c>
       <c r="B89" s="37" t="n">
-        <v>180</v>
-      </c>
-      <c r="C89" s="51" t="inlineStr">
+        <v>140</v>
+      </c>
+      <c r="C89" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D89" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D89" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E89" s="34" t="inlineStr">
@@ -5157,7 +5159,7 @@
       </c>
       <c r="F89" s="34" t="inlineStr">
         <is>
-          <t>CPFM x Nike Flea 1 “Barely”</t>
+          <t>Nike Caitlin 1 “Racer Blue Pink”</t>
         </is>
       </c>
     </row>
@@ -5166,16 +5168,16 @@
         <v>46340</v>
       </c>
       <c r="B90" s="40" t="n">
-        <v>170</v>
+        <v>180</v>
       </c>
       <c r="C90" s="46" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D90" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D90" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E90" s="30" t="inlineStr">
@@ -5185,7 +5187,7 @@
       </c>
       <c r="F90" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Green Apple”</t>
+          <t>CPFM x Nike Flea 1 “Barely”</t>
         </is>
       </c>
     </row>
@@ -5194,26 +5196,26 @@
         <v>46340</v>
       </c>
       <c r="B91" s="37" t="n">
-        <v>255</v>
-      </c>
-      <c r="C91" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D91" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>170</v>
+      </c>
+      <c r="C91" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D91" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E91" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F91" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Green Screen”</t>
+          <t>Nike Zoom Hyperflight “Green Apple”</t>
         </is>
       </c>
     </row>
@@ -5257,7 +5259,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D93" s="53" t="inlineStr">
+      <c r="D93" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5336,7 +5338,7 @@
       <c r="B96" s="40" t="n">
         <v>130</v>
       </c>
-      <c r="C96" s="52" t="inlineStr">
+      <c r="C96" s="51" t="inlineStr">
         <is>
           <t>LOW</t>
         </is>
@@ -5445,9 +5447,7 @@
       <c r="A100" s="31" t="n">
         <v>46347</v>
       </c>
-      <c r="B100" s="40" t="n">
-        <v>230</v>
-      </c>
+      <c r="B100" s="40" t="inlineStr"/>
       <c r="C100" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -5465,7 +5465,7 @@
       </c>
       <c r="F100" s="30" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
         </is>
       </c>
     </row>
@@ -5474,11 +5474,11 @@
         <v>46347</v>
       </c>
       <c r="B101" s="37" t="n">
-        <v>135</v>
-      </c>
-      <c r="C101" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>155</v>
+      </c>
+      <c r="C101" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D101" s="38" t="inlineStr">
@@ -5493,7 +5493,7 @@
       </c>
       <c r="F101" s="34" t="inlineStr">
         <is>
-          <t>Jordan Tatum 5 “Sunset”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -5502,16 +5502,16 @@
         <v>46347</v>
       </c>
       <c r="B102" s="40" t="n">
-        <v>140</v>
-      </c>
-      <c r="C102" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D102" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>230</v>
+      </c>
+      <c r="C102" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D102" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E102" s="30" t="inlineStr">
@@ -5521,7 +5521,7 @@
       </c>
       <c r="F102" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Snow White”</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -5529,10 +5529,12 @@
       <c r="A103" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B103" s="37" t="inlineStr"/>
-      <c r="C103" s="48" t="inlineStr">
-        <is>
-          <t>LOW</t>
+      <c r="B103" s="37" t="n">
+        <v>135</v>
+      </c>
+      <c r="C103" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D103" s="38" t="inlineStr">
@@ -5542,12 +5544,12 @@
       </c>
       <c r="E103" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F103" s="34" t="inlineStr">
         <is>
-          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
+          <t>Jordan Tatum 5 “Sunset”</t>
         </is>
       </c>
     </row>
@@ -5556,7 +5558,7 @@
         <v>46347</v>
       </c>
       <c r="B104" s="40" t="n">
-        <v>150</v>
+        <v>140</v>
       </c>
       <c r="C104" s="46" t="inlineStr">
         <is>
@@ -5570,12 +5572,12 @@
       </c>
       <c r="E104" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F104" s="30" t="inlineStr">
         <is>
-          <t>Jordan Triangle “Paolo Banchero”</t>
+          <t>Nike Caitlin 1 “Snow White”</t>
         </is>
       </c>
     </row>
@@ -5583,12 +5585,10 @@
       <c r="A105" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B105" s="37" t="n">
-        <v>215</v>
-      </c>
-      <c r="C105" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+      <c r="B105" s="37" t="inlineStr"/>
+      <c r="C105" s="48" t="inlineStr">
+        <is>
+          <t>LOW</t>
         </is>
       </c>
       <c r="D105" s="38" t="inlineStr">
@@ -5598,12 +5598,12 @@
       </c>
       <c r="E105" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F105" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>UNheardof x adidas Adistar Control 5 “Doggy Runner”</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5612,7 @@
         <v>46347</v>
       </c>
       <c r="B106" s="40" t="n">
-        <v>190</v>
+        <v>150</v>
       </c>
       <c r="C106" s="46" t="inlineStr">
         <is>
@@ -5626,12 +5626,12 @@
       </c>
       <c r="E106" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F106" s="30" t="inlineStr">
         <is>
-          <t>Nike Zoom Hyperflight “Safari”</t>
+          <t>Jordan Triangle “Paolo Banchero”</t>
         </is>
       </c>
     </row>
@@ -5640,7 +5640,7 @@
         <v>46347</v>
       </c>
       <c r="B107" s="37" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="C107" s="36" t="inlineStr">
         <is>
@@ -5654,12 +5654,12 @@
       </c>
       <c r="E107" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F107" s="34" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -5668,11 +5668,11 @@
         <v>46347</v>
       </c>
       <c r="B108" s="40" t="n">
-        <v>155</v>
-      </c>
-      <c r="C108" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>190</v>
+      </c>
+      <c r="C108" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D108" s="41" t="inlineStr">
@@ -5687,7 +5687,7 @@
       </c>
       <c r="F108" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Nike Zoom Hyperflight “Safari”</t>
         </is>
       </c>
     </row>
@@ -5695,15 +5695,17 @@
       <c r="A109" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B109" s="37" t="inlineStr"/>
+      <c r="B109" s="37" t="n">
+        <v>125</v>
+      </c>
       <c r="C109" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D109" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D109" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E109" s="34" t="inlineStr">
@@ -5713,7 +5715,7 @@
       </c>
       <c r="F109" s="34" t="inlineStr">
         <is>
-          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -5736,12 +5738,12 @@
       </c>
       <c r="E110" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F110" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -5750,7 +5752,7 @@
         <v>46353</v>
       </c>
       <c r="B111" s="37" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C111" s="36" t="inlineStr">
         <is>
@@ -5764,12 +5766,12 @@
       </c>
       <c r="E111" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F111" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5780,7 @@
         <v>46353</v>
       </c>
       <c r="B112" s="40" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C112" s="39" t="inlineStr">
         <is>
@@ -5792,12 +5794,12 @@
       </c>
       <c r="E112" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F112" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -5836,14 +5838,14 @@
       <c r="B114" s="40" t="n">
         <v>140</v>
       </c>
-      <c r="C114" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D114" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C114" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D114" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E114" s="30" t="inlineStr">
@@ -5853,7 +5855,7 @@
       </c>
       <c r="F114" s="30" t="inlineStr">
         <is>
-          <t>Victory Lap x Nike Air Force 1 Mid</t>
+          <t>Nike Caitlin 1 “Warning Code”</t>
         </is>
       </c>
     </row>
@@ -5862,14 +5864,14 @@
         <v>46354</v>
       </c>
       <c r="B115" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C115" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D115" s="53" t="inlineStr">
+        <v>190</v>
+      </c>
+      <c r="C115" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D115" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -5881,7 +5883,7 @@
       </c>
       <c r="F115" s="34" t="inlineStr">
         <is>
-          <t>Nike SB Dunk Low “Green Patent”</t>
+          <t>Carhartt WIP x Nike Air Max Goadome Low Pack</t>
         </is>
       </c>
     </row>
@@ -5890,26 +5892,26 @@
         <v>46354</v>
       </c>
       <c r="B116" s="40" t="n">
-        <v>200</v>
-      </c>
-      <c r="C116" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D116" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>140</v>
+      </c>
+      <c r="C116" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D116" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E116" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F116" s="30" t="inlineStr">
         <is>
-          <t>Jordan 6 Rings Winterized “Cobalt Blue”</t>
+          <t>Victory Lap x Nike Air Force 1 Mid</t>
         </is>
       </c>
     </row>
@@ -5917,15 +5919,17 @@
       <c r="A117" s="35" t="n">
         <v>46354</v>
       </c>
-      <c r="B117" s="37" t="inlineStr"/>
+      <c r="B117" s="37" t="n">
+        <v>130</v>
+      </c>
       <c r="C117" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D117" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D117" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E117" s="34" t="inlineStr">
@@ -5935,7 +5939,7 @@
       </c>
       <c r="F117" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro College Football Pack</t>
+          <t>Nike SB Dunk Low “Green Patent”</t>
         </is>
       </c>
     </row>
@@ -5944,26 +5948,26 @@
         <v>46354</v>
       </c>
       <c r="B118" s="40" t="n">
-        <v>240</v>
-      </c>
-      <c r="C118" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D118" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>200</v>
+      </c>
+      <c r="C118" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D118" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E118" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F118" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “FSU”</t>
+          <t>Jordan 6 Rings Winterized “Cobalt Blue”</t>
         </is>
       </c>
     </row>
@@ -5972,24 +5976,24 @@
         <v>46354</v>
       </c>
       <c r="B119" s="37" t="inlineStr"/>
-      <c r="C119" s="54" t="inlineStr">
-        <is>
-          <t>EXTREME</t>
-        </is>
-      </c>
-      <c r="D119" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="C119" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D119" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E119" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F119" s="34" t="inlineStr">
         <is>
-          <t>Social Status x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite Pro College Football Pack</t>
         </is>
       </c>
     </row>
@@ -5997,15 +6001,17 @@
       <c r="A120" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B120" s="40" t="inlineStr"/>
-      <c r="C120" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D120" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="B120" s="40" t="n">
+        <v>240</v>
+      </c>
+      <c r="C120" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D120" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E120" s="30" t="inlineStr">
@@ -6015,7 +6021,7 @@
       </c>
       <c r="F120" s="30" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Aunt Pearl” 2026</t>
+          <t>Nike Air Foamposite Pro “FSU”</t>
         </is>
       </c>
     </row>
@@ -6024,24 +6030,24 @@
         <v>46354</v>
       </c>
       <c r="B121" s="37" t="inlineStr"/>
-      <c r="C121" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D121" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="C121" s="54" t="inlineStr">
+        <is>
+          <t>EXTREME</t>
+        </is>
+      </c>
+      <c r="D121" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E121" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F121" s="34" t="inlineStr">
         <is>
-          <t>Slam Jam x Nike Air Max 97</t>
+          <t>Social Status x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6049,9 +6055,7 @@
       <c r="A122" s="31" t="n">
         <v>46354</v>
       </c>
-      <c r="B122" s="40" t="n">
-        <v>140</v>
-      </c>
+      <c r="B122" s="40" t="inlineStr"/>
       <c r="C122" s="46" t="inlineStr">
         <is>
           <t>MED</t>
@@ -6069,20 +6073,18 @@
       </c>
       <c r="F122" s="30" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Warning Code”</t>
+          <t>Nike KD 6 “Aunt Pearl” 2026</t>
         </is>
       </c>
     </row>
     <row r="123" ht="15" customHeight="1">
       <c r="A123" s="35" t="n">
-        <v>46357</v>
-      </c>
-      <c r="B123" s="37" t="n">
-        <v>130</v>
-      </c>
-      <c r="C123" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>46354</v>
+      </c>
+      <c r="B123" s="37" t="inlineStr"/>
+      <c r="C123" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D123" s="38" t="inlineStr">
@@ -6097,7 +6099,7 @@
       </c>
       <c r="F123" s="34" t="inlineStr">
         <is>
-          <t>Nike KD 6 “Texas”</t>
+          <t>Slam Jam x Nike Air Max 97</t>
         </is>
       </c>
     </row>
@@ -6106,11 +6108,11 @@
         <v>46357</v>
       </c>
       <c r="B124" s="40" t="n">
-        <v>190</v>
-      </c>
-      <c r="C124" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>130</v>
+      </c>
+      <c r="C124" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D124" s="41" t="inlineStr">
@@ -6125,20 +6127,20 @@
       </c>
       <c r="F124" s="30" t="inlineStr">
         <is>
-          <t>Nike LeBron 24 “Chosen 1s”</t>
+          <t>Nike KD 6 “Texas”</t>
         </is>
       </c>
     </row>
     <row r="125" ht="15" customHeight="1">
       <c r="A125" s="35" t="n">
-        <v>46359</v>
+        <v>46357</v>
       </c>
       <c r="B125" s="37" t="n">
-        <v>170</v>
-      </c>
-      <c r="C125" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>190</v>
+      </c>
+      <c r="C125" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D125" s="38" t="inlineStr">
@@ -6153,20 +6155,20 @@
       </c>
       <c r="F125" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Bakin “Black White”</t>
+          <t>Nike LeBron 24 “Chosen 1s”</t>
         </is>
       </c>
     </row>
     <row r="126" ht="15" customHeight="1">
       <c r="A126" s="31" t="n">
-        <v>46361</v>
+        <v>46359</v>
       </c>
       <c r="B126" s="40" t="n">
-        <v>155</v>
-      </c>
-      <c r="C126" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C126" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D126" s="41" t="inlineStr">
@@ -6181,7 +6183,7 @@
       </c>
       <c r="F126" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Laser Orange”</t>
+          <t>Nike Air Bakin “Black White”</t>
         </is>
       </c>
     </row>
@@ -6190,26 +6192,26 @@
         <v>46361</v>
       </c>
       <c r="B127" s="37" t="n">
-        <v>300</v>
-      </c>
-      <c r="C127" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D127" s="55" t="inlineStr">
-        <is>
-          <t>Confirmed App</t>
+        <v>155</v>
+      </c>
+      <c r="C127" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D127" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E127" s="34" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F127" s="34" t="inlineStr">
         <is>
-          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
+          <t>Nike Kobe AD Protro “Laser Orange”</t>
         </is>
       </c>
     </row>
@@ -6218,26 +6220,26 @@
         <v>46361</v>
       </c>
       <c r="B128" s="40" t="n">
-        <v>215</v>
-      </c>
-      <c r="C128" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D128" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>300</v>
+      </c>
+      <c r="C128" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D128" s="55" t="inlineStr">
+        <is>
+          <t>Confirmed App</t>
         </is>
       </c>
       <c r="E128" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F128" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 10 “Sacramento”</t>
+          <t>Pharrell x adidas Adistar Jellyfish “Auburn Timber”</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6248,7 @@
         <v>46361</v>
       </c>
       <c r="B129" s="37" t="n">
-        <v>225</v>
+        <v>215</v>
       </c>
       <c r="C129" s="36" t="inlineStr">
         <is>
@@ -6265,7 +6267,7 @@
       </c>
       <c r="F129" s="34" t="inlineStr">
         <is>
-          <t>SoleFly x Air Jordan 5</t>
+          <t>Air Jordan 10 “Sacramento”</t>
         </is>
       </c>
     </row>
@@ -6274,11 +6276,11 @@
         <v>46361</v>
       </c>
       <c r="B130" s="40" t="n">
-        <v>300</v>
-      </c>
-      <c r="C130" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
+        <v>225</v>
+      </c>
+      <c r="C130" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
         </is>
       </c>
       <c r="D130" s="41" t="inlineStr">
@@ -6288,40 +6290,40 @@
       </c>
       <c r="E130" s="30" t="inlineStr">
         <is>
-          <t>Adidas</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F130" s="30" t="inlineStr">
         <is>
-          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
+          <t>SoleFly x Air Jordan 5</t>
         </is>
       </c>
     </row>
     <row r="131" ht="15" customHeight="1">
       <c r="A131" s="35" t="n">
-        <v>46367</v>
+        <v>46361</v>
       </c>
       <c r="B131" s="37" t="n">
-        <v>150</v>
-      </c>
-      <c r="C131" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D131" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>300</v>
+      </c>
+      <c r="C131" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D131" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E131" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Adidas</t>
         </is>
       </c>
       <c r="F131" s="34" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Pharrell Williams x adidas Adistar Jellyfish “Dark Brown Frozen Green”</t>
         </is>
       </c>
     </row>
@@ -6329,25 +6331,27 @@
       <c r="A132" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B132" s="40" t="inlineStr"/>
+      <c r="B132" s="40" t="n">
+        <v>240</v>
+      </c>
       <c r="C132" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D132" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D132" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E132" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F132" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -6356,26 +6360,26 @@
         <v>46367</v>
       </c>
       <c r="B133" s="37" t="n">
-        <v>240</v>
+        <v>150</v>
       </c>
       <c r="C133" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D133" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D133" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E133" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F133" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -6383,45 +6387,43 @@
       <c r="A134" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B134" s="40" t="n">
-        <v>190</v>
-      </c>
+      <c r="B134" s="40" t="inlineStr"/>
       <c r="C134" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D134" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D134" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E134" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F134" s="30" t="inlineStr">
         <is>
-          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
     <row r="135" ht="15" customHeight="1">
       <c r="A135" s="35" t="n">
-        <v>46368</v>
+        <v>46367</v>
       </c>
       <c r="B135" s="37" t="n">
-        <v>130</v>
+        <v>190</v>
       </c>
       <c r="C135" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D135" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D135" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E135" s="34" t="inlineStr">
@@ -6431,7 +6433,7 @@
       </c>
       <c r="F135" s="34" t="inlineStr">
         <is>
-          <t>APB x Nike Dunk Low “Midnight Navy”</t>
+          <t>Jalen Brunson x Nike Kobe 3 Low Protro “Arancia”</t>
         </is>
       </c>
     </row>
@@ -6440,26 +6442,26 @@
         <v>46368</v>
       </c>
       <c r="B136" s="40" t="n">
-        <v>235</v>
+        <v>130</v>
       </c>
       <c r="C136" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D136" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D136" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E136" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F136" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 11 “Space Jam” 2026</t>
+          <t>APB x Nike Dunk Low “Midnight Navy”</t>
         </is>
       </c>
     </row>
@@ -6468,44 +6470,44 @@
         <v>46368</v>
       </c>
       <c r="B137" s="37" t="n">
-        <v>135</v>
-      </c>
-      <c r="C137" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D137" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>235</v>
+      </c>
+      <c r="C137" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D137" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E137" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F137" s="34" t="inlineStr">
         <is>
-          <t>PaisaBoys x Nike SB P-Rod 1</t>
+          <t>Air Jordan 11 “Space Jam” 2026</t>
         </is>
       </c>
     </row>
     <row r="138" ht="15" customHeight="1">
       <c r="A138" s="31" t="n">
-        <v>46375</v>
+        <v>46368</v>
       </c>
       <c r="B138" s="40" t="n">
-        <v>210</v>
+        <v>135</v>
       </c>
       <c r="C138" s="46" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D138" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D138" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E138" s="30" t="inlineStr">
@@ -6515,7 +6517,7 @@
       </c>
       <c r="F138" s="30" t="inlineStr">
         <is>
-          <t>Nike GT Future “Triple Black”</t>
+          <t>PaisaBoys x Nike SB P-Rod 1</t>
         </is>
       </c>
     </row>
@@ -6524,11 +6526,11 @@
         <v>46375</v>
       </c>
       <c r="B139" s="37" t="n">
-        <v>220</v>
-      </c>
-      <c r="C139" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>170</v>
+      </c>
+      <c r="C139" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D139" s="38" t="inlineStr">
@@ -6538,12 +6540,12 @@
       </c>
       <c r="E139" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F139" s="34" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Pink Thunder”</t>
+          <t>Nike Air Zoom Flight The Glove “Royal Blue”</t>
         </is>
       </c>
     </row>
@@ -6552,16 +6554,16 @@
         <v>46375</v>
       </c>
       <c r="B140" s="40" t="n">
-        <v>350</v>
-      </c>
-      <c r="C140" s="39" t="inlineStr">
-        <is>
-          <t>HIGH</t>
-        </is>
-      </c>
-      <c r="D140" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+        <v>210</v>
+      </c>
+      <c r="C140" s="46" t="inlineStr">
+        <is>
+          <t>MED</t>
+        </is>
+      </c>
+      <c r="D140" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E140" s="30" t="inlineStr">
@@ -6571,7 +6573,7 @@
       </c>
       <c r="F140" s="30" t="inlineStr">
         <is>
-          <t>Victor Solomon x Nike Air Foamposite One “Trophies Red”</t>
+          <t>Nike GT Future “Triple Black”</t>
         </is>
       </c>
     </row>
@@ -6580,26 +6582,26 @@
         <v>46375</v>
       </c>
       <c r="B141" s="37" t="n">
-        <v>120</v>
+        <v>220</v>
       </c>
       <c r="C141" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D141" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D141" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E141" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F141" s="34" t="inlineStr">
         <is>
-          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
+          <t>Air Jordan 4 “Pink Thunder”</t>
         </is>
       </c>
     </row>
@@ -6608,16 +6610,16 @@
         <v>46375</v>
       </c>
       <c r="B142" s="40" t="n">
-        <v>170</v>
-      </c>
-      <c r="C142" s="46" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D142" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>350</v>
+      </c>
+      <c r="C142" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D142" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E142" s="30" t="inlineStr">
@@ -6627,25 +6629,25 @@
       </c>
       <c r="F142" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Zoom Flight The Glove “Royal Blue”</t>
+          <t>Victor Solomon x Nike Air Foamposite One “Trophies Red”</t>
         </is>
       </c>
     </row>
     <row r="143" ht="15" customHeight="1">
       <c r="A143" s="35" t="n">
-        <v>46377</v>
+        <v>46375</v>
       </c>
       <c r="B143" s="37" t="n">
-        <v>140</v>
-      </c>
-      <c r="C143" s="51" t="inlineStr">
-        <is>
-          <t>MED</t>
-        </is>
-      </c>
-      <c r="D143" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+        <v>120</v>
+      </c>
+      <c r="C143" s="36" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D143" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E143" s="34" t="inlineStr">
@@ -6655,16 +6657,16 @@
       </c>
       <c r="F143" s="34" t="inlineStr">
         <is>
-          <t>Nike Caitlin 1 “Chiefs”</t>
+          <t>Fly Streetwear x Nike SB Air Force 1 Low “University Gold”</t>
         </is>
       </c>
     </row>
     <row r="144" ht="15" customHeight="1">
       <c r="A144" s="31" t="n">
-        <v>46380</v>
+        <v>46377</v>
       </c>
       <c r="B144" s="40" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="C144" s="46" t="inlineStr">
         <is>
@@ -6678,25 +6680,25 @@
       </c>
       <c r="E144" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F144" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 8 “Knicks”</t>
+          <t>Nike Caitlin 1 “Chiefs”</t>
         </is>
       </c>
     </row>
     <row r="145" ht="15" customHeight="1">
       <c r="A145" s="35" t="n">
-        <v>46381</v>
+        <v>46380</v>
       </c>
       <c r="B145" s="37" t="n">
-        <v>190</v>
-      </c>
-      <c r="C145" s="36" t="inlineStr">
-        <is>
-          <t>HIGH</t>
+        <v>215</v>
+      </c>
+      <c r="C145" s="53" t="inlineStr">
+        <is>
+          <t>MED</t>
         </is>
       </c>
       <c r="D145" s="38" t="inlineStr">
@@ -6706,40 +6708,40 @@
       </c>
       <c r="E145" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F145" s="34" t="inlineStr">
         <is>
-          <t>Nike Kobe 6 Protro “Coals”</t>
+          <t>Air Jordan 8 “Knicks”</t>
         </is>
       </c>
     </row>
     <row r="146" ht="15" customHeight="1">
       <c r="A146" s="31" t="n">
-        <v>46382</v>
+        <v>46381</v>
       </c>
       <c r="B146" s="40" t="n">
-        <v>355</v>
+        <v>190</v>
       </c>
       <c r="C146" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D146" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D146" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E146" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F146" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “BIN 23”</t>
+          <t>Nike Kobe 6 Protro “Coals”</t>
         </is>
       </c>
     </row>
@@ -6750,7 +6752,7 @@
       <c r="B147" s="37" t="n">
         <v>135</v>
       </c>
-      <c r="C147" s="51" t="inlineStr">
+      <c r="C147" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
@@ -6773,10 +6775,10 @@
     </row>
     <row r="148" ht="15" customHeight="1">
       <c r="A148" s="31" t="n">
-        <v>46387</v>
+        <v>46382</v>
       </c>
       <c r="B148" s="40" t="n">
-        <v>215</v>
+        <v>355</v>
       </c>
       <c r="C148" s="39" t="inlineStr">
         <is>
@@ -6795,7 +6797,7 @@
       </c>
       <c r="F148" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Middle East”</t>
+          <t>Air Jordan 4 “BIN 23”</t>
         </is>
       </c>
     </row>
@@ -6804,59 +6806,115 @@
         <v>46387</v>
       </c>
       <c r="B149" s="37" t="n">
-        <v>190</v>
+        <v>215</v>
       </c>
       <c r="C149" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D149" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D149" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E149" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F149" s="34" t="inlineStr">
         <is>
-          <t>Nike Kobe 9 EM Low Protro “Philippines”</t>
+          <t>Air Jordan 3 “Middle East”</t>
         </is>
       </c>
     </row>
     <row r="150" ht="15" customHeight="1">
       <c r="A150" s="31" t="n">
+        <v>46387</v>
+      </c>
+      <c r="B150" s="40" t="n">
+        <v>190</v>
+      </c>
+      <c r="C150" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D150" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E150" s="30" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F150" s="30" t="inlineStr">
+        <is>
+          <t>Nike Kobe 9 EM Low Protro “Philippines”</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="15" customHeight="1">
+      <c r="A151" s="35" t="n">
         <v>46392</v>
       </c>
-      <c r="B150" s="40" t="n">
+      <c r="B151" s="37" t="n">
         <v>140</v>
       </c>
-      <c r="C150" s="46" t="inlineStr">
+      <c r="C151" s="53" t="inlineStr">
         <is>
           <t>MED</t>
         </is>
       </c>
-      <c r="D150" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
-        </is>
-      </c>
-      <c r="E150" s="30" t="inlineStr">
-        <is>
-          <t>Nike</t>
-        </is>
-      </c>
-      <c r="F150" s="30" t="inlineStr">
+      <c r="D151" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E151" s="34" t="inlineStr">
+        <is>
+          <t>Nike</t>
+        </is>
+      </c>
+      <c r="F151" s="34" t="inlineStr">
         <is>
           <t>Nike Caitlin 1 “3x Black”</t>
         </is>
       </c>
     </row>
+    <row r="152" ht="15" customHeight="1">
+      <c r="A152" s="31" t="n">
+        <v>46402</v>
+      </c>
+      <c r="B152" s="40" t="n">
+        <v>220</v>
+      </c>
+      <c r="C152" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D152" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E152" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F152" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Spotlight”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F150"/>
+  <autoFilter ref="A3:F152"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -6871,7 +6929,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F81"/>
+  <dimension ref="A1:F82"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6897,7 +6955,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="50" t="inlineStr">
         <is>
-          <t>Generated October 16, 2026  ·  10:56 UTC</t>
+          <t>Generated October 17, 2026  ·  10:19 UTC</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -6940,10 +6998,10 @@
     </row>
     <row r="4" ht="15" customHeight="1">
       <c r="A4" s="31" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B4" s="40" t="n">
-        <v>250</v>
+        <v>215</v>
       </c>
       <c r="C4" s="39" t="inlineStr">
         <is>
@@ -6957,21 +7015,21 @@
       </c>
       <c r="E4" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F4" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Glow in the Dark”</t>
+          <t>Air Jordan 5 “Halloween”</t>
         </is>
       </c>
     </row>
     <row r="5" ht="15" customHeight="1">
       <c r="A5" s="35" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B5" s="37" t="n">
-        <v>250</v>
+        <v>120</v>
       </c>
       <c r="C5" s="36" t="inlineStr">
         <is>
@@ -6990,16 +7048,16 @@
       </c>
       <c r="F5" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro PRM “Glow in the Dark”</t>
+          <t>Nocturnal x Nike SB Air Force 1 Low</t>
         </is>
       </c>
     </row>
     <row r="6" ht="15" customHeight="1">
       <c r="A6" s="31" t="n">
-        <v>46312</v>
+        <v>46316</v>
       </c>
       <c r="B6" s="40" t="n">
-        <v>215</v>
+        <v>140</v>
       </c>
       <c r="C6" s="39" t="inlineStr">
         <is>
@@ -7013,30 +7071,30 @@
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F6" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 5 “Halloween”</t>
+          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
         </is>
       </c>
     </row>
     <row r="7" ht="15" customHeight="1">
       <c r="A7" s="35" t="n">
-        <v>46312</v>
+        <v>46317</v>
       </c>
       <c r="B7" s="37" t="n">
-        <v>120</v>
+        <v>150</v>
       </c>
       <c r="C7" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D7" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D7" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E7" s="34" t="inlineStr">
@@ -7046,16 +7104,16 @@
       </c>
       <c r="F7" s="34" t="inlineStr">
         <is>
-          <t>Nocturnal x Nike SB Air Force 1 Low</t>
+          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
         </is>
       </c>
     </row>
     <row r="8" ht="15" customHeight="1">
       <c r="A8" s="31" t="n">
-        <v>46316</v>
+        <v>46317</v>
       </c>
       <c r="B8" s="40" t="n">
-        <v>140</v>
+        <v>125</v>
       </c>
       <c r="C8" s="39" t="inlineStr">
         <is>
@@ -7074,7 +7132,7 @@
       </c>
       <c r="F8" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low Pony Hair “Team Red”</t>
+          <t>Nike Air Force 1 “What The LA”</t>
         </is>
       </c>
     </row>
@@ -7102,16 +7160,16 @@
       </c>
       <c r="F9" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 “What The LA”</t>
+          <t>Nike Air Force 1 Low “What The LA”</t>
         </is>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
       <c r="A10" s="31" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B10" s="40" t="n">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="C10" s="39" t="inlineStr">
         <is>
@@ -7130,16 +7188,16 @@
       </c>
       <c r="F10" s="30" t="inlineStr">
         <is>
-          <t>NIGO x J-Hope x Nike Air Force 1 ’01</t>
+          <t>Nike Dunk Low “Shibuya Halloween”</t>
         </is>
       </c>
     </row>
     <row r="11" ht="15" customHeight="1">
       <c r="A11" s="35" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
       <c r="B11" s="37" t="n">
-        <v>125</v>
+        <v>140</v>
       </c>
       <c r="C11" s="36" t="inlineStr">
         <is>
@@ -7158,7 +7216,7 @@
       </c>
       <c r="F11" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “What The LA”</t>
+          <t>Nike Air Force 1 Low “NYC Rat”</t>
         </is>
       </c>
     </row>
@@ -7167,7 +7225,7 @@
         <v>46318</v>
       </c>
       <c r="B12" s="40" t="n">
-        <v>140</v>
+        <v>200</v>
       </c>
       <c r="C12" s="39" t="inlineStr">
         <is>
@@ -7181,12 +7239,12 @@
       </c>
       <c r="E12" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F12" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “NYC Rat”</t>
+          <t>APB x Air Jordan 11 Low “Made for Locals”</t>
         </is>
       </c>
     </row>
@@ -7195,44 +7253,44 @@
         <v>46318</v>
       </c>
       <c r="B13" s="37" t="n">
-        <v>200</v>
+        <v>140</v>
       </c>
       <c r="C13" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D13" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D13" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E13" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F13" s="34" t="inlineStr">
         <is>
-          <t>APB x Air Jordan 11 Low “Made for Locals”</t>
+          <t>Nike Air Force 1 ’01 “Nightmare”</t>
         </is>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
       <c r="A14" s="31" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B14" s="40" t="n">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="C14" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D14" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E14" s="30" t="inlineStr">
@@ -7242,13 +7300,13 @@
       </c>
       <c r="F14" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 ’01 “Nightmare”</t>
+          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
         </is>
       </c>
     </row>
     <row r="15" ht="15" customHeight="1">
       <c r="A15" s="35" t="n">
-        <v>46318</v>
+        <v>46319</v>
       </c>
       <c r="B15" s="37" t="n">
         <v>130</v>
@@ -7258,19 +7316,19 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D15" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D15" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E15" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F15" s="34" t="inlineStr">
         <is>
-          <t>Nike Dunk Low “Shibuya Halloween”</t>
+          <t>Air Jordan 1 Low “Halloween”</t>
         </is>
       </c>
     </row>
@@ -7279,26 +7337,26 @@
         <v>46319</v>
       </c>
       <c r="B16" s="40" t="n">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="C16" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D16" s="41" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D16" s="33" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E16" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F16" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Low “Halloween”</t>
+          <t>Nike Air Force 1 Low “Ghostface Black”</t>
         </is>
       </c>
     </row>
@@ -7307,26 +7365,26 @@
         <v>46319</v>
       </c>
       <c r="B17" s="37" t="n">
-        <v>125</v>
+        <v>145</v>
       </c>
       <c r="C17" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D17" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D17" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E17" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F17" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface Black”</t>
+          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
         </is>
       </c>
     </row>
@@ -7335,7 +7393,7 @@
         <v>46319</v>
       </c>
       <c r="B18" s="40" t="n">
-        <v>145</v>
+        <v>125</v>
       </c>
       <c r="C18" s="39" t="inlineStr">
         <is>
@@ -7349,12 +7407,12 @@
       </c>
       <c r="E18" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F18" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 1 Mid “Dia de Los Muertos”</t>
+          <t>Nike Air Force 1 Low “Ghostface”</t>
         </is>
       </c>
     </row>
@@ -7363,7 +7421,7 @@
         <v>46319</v>
       </c>
       <c r="B19" s="37" t="n">
-        <v>125</v>
+        <v>215</v>
       </c>
       <c r="C19" s="36" t="inlineStr">
         <is>
@@ -7377,21 +7435,21 @@
       </c>
       <c r="E19" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F19" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Ghostface”</t>
+          <t>Air Jordan 12 “Fireside”</t>
         </is>
       </c>
     </row>
     <row r="20" ht="15" customHeight="1">
       <c r="A20" s="31" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
       <c r="B20" s="40" t="n">
-        <v>215</v>
+        <v>205</v>
       </c>
       <c r="C20" s="39" t="inlineStr">
         <is>
@@ -7410,16 +7468,16 @@
       </c>
       <c r="F20" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 12 “Fireside”</t>
+          <t>Air Jordan 41 “University Red”</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15" customHeight="1">
       <c r="A21" s="35" t="n">
-        <v>46319</v>
+        <v>46321</v>
       </c>
       <c r="B21" s="37" t="n">
-        <v>190</v>
+        <v>125</v>
       </c>
       <c r="C21" s="36" t="inlineStr">
         <is>
@@ -7438,16 +7496,16 @@
       </c>
       <c r="F21" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Max 95 “Reverse Blue Spark”</t>
+          <t>Nike Air Force 1 Low “University Pack”</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15" customHeight="1">
       <c r="A22" s="31" t="n">
-        <v>46320</v>
+        <v>46321</v>
       </c>
       <c r="B22" s="40" t="n">
-        <v>205</v>
+        <v>125</v>
       </c>
       <c r="C22" s="39" t="inlineStr">
         <is>
@@ -7461,12 +7519,12 @@
       </c>
       <c r="E22" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F22" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 41 “University Red”</t>
+          <t>Nike Air Force 1 Low “Texas”</t>
         </is>
       </c>
     </row>
@@ -7494,7 +7552,7 @@
       </c>
       <c r="F23" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “University Pack”</t>
+          <t>Nike Air Force 1 Low “Georgia”</t>
         </is>
       </c>
     </row>
@@ -7522,7 +7580,7 @@
       </c>
       <c r="F24" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Texas”</t>
+          <t>Nike Air Force 1 Low “Kentucky”</t>
         </is>
       </c>
     </row>
@@ -7550,16 +7608,16 @@
       </c>
       <c r="F25" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Georgia”</t>
+          <t>Nike Air Force 1 Low “Oregon”</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15" customHeight="1">
       <c r="A26" s="31" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="B26" s="40" t="n">
-        <v>125</v>
+        <v>190</v>
       </c>
       <c r="C26" s="39" t="inlineStr">
         <is>
@@ -7578,25 +7636,25 @@
       </c>
       <c r="F26" s="30" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Kentucky”</t>
+          <t>Nike Kobe 3 Low Protro “Mamba Eterno”</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15" customHeight="1">
       <c r="A27" s="35" t="n">
-        <v>46321</v>
+        <v>46325</v>
       </c>
       <c r="B27" s="37" t="n">
-        <v>125</v>
+        <v>200</v>
       </c>
       <c r="C27" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D27" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D27" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E27" s="34" t="inlineStr">
@@ -7606,7 +7664,7 @@
       </c>
       <c r="F27" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Force 1 Low “Oregon”</t>
+          <t>Nike LeBron 24 “Storm Drain”</t>
         </is>
       </c>
     </row>
@@ -7643,7 +7701,7 @@
         <v>46325</v>
       </c>
       <c r="B29" s="37" t="n">
-        <v>190</v>
+        <v>155</v>
       </c>
       <c r="C29" s="36" t="inlineStr">
         <is>
@@ -7662,7 +7720,7 @@
       </c>
       <c r="F29" s="34" t="inlineStr">
         <is>
-          <t>Nike Kobe 3 Low Protro “Mamba Eterno”</t>
+          <t>Nike Kobe AD Protro “Mamba Eterno”</t>
         </is>
       </c>
     </row>
@@ -7928,7 +7986,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D39" s="53" t="inlineStr">
+      <c r="D39" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -7984,7 +8042,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D41" s="53" t="inlineStr">
+      <c r="D41" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8152,7 +8210,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D47" s="53" t="inlineStr">
+      <c r="D47" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8256,15 +8314,13 @@
       <c r="A51" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B51" s="37" t="n">
-        <v>230</v>
-      </c>
+      <c r="B51" s="37" t="inlineStr"/>
       <c r="C51" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D51" s="53" t="inlineStr">
+      <c r="D51" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8276,7 +8332,7 @@
       </c>
       <c r="F51" s="34" t="inlineStr">
         <is>
-          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
+          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
         </is>
       </c>
     </row>
@@ -8285,7 +8341,7 @@
         <v>46347</v>
       </c>
       <c r="B52" s="40" t="n">
-        <v>215</v>
+        <v>155</v>
       </c>
       <c r="C52" s="39" t="inlineStr">
         <is>
@@ -8304,7 +8360,7 @@
       </c>
       <c r="F52" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Not Nice”</t>
+          <t>Air Jordan 3 “Santa”</t>
         </is>
       </c>
     </row>
@@ -8313,16 +8369,16 @@
         <v>46347</v>
       </c>
       <c r="B53" s="37" t="n">
-        <v>125</v>
+        <v>230</v>
       </c>
       <c r="C53" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D53" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D53" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E53" s="34" t="inlineStr">
@@ -8332,7 +8388,7 @@
       </c>
       <c r="F53" s="34" t="inlineStr">
         <is>
-          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
+          <t>Oregon Ducks x Nike Air Foamposite Pro “Mummy Duck” (Phantom)</t>
         </is>
       </c>
     </row>
@@ -8341,7 +8397,7 @@
         <v>46347</v>
       </c>
       <c r="B54" s="40" t="n">
-        <v>155</v>
+        <v>215</v>
       </c>
       <c r="C54" s="39" t="inlineStr">
         <is>
@@ -8355,12 +8411,12 @@
       </c>
       <c r="E54" s="30" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F54" s="30" t="inlineStr">
         <is>
-          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
+          <t>Air Jordan 3 “Not Nice”</t>
         </is>
       </c>
     </row>
@@ -8368,15 +8424,17 @@
       <c r="A55" s="35" t="n">
         <v>46347</v>
       </c>
-      <c r="B55" s="37" t="inlineStr"/>
+      <c r="B55" s="37" t="n">
+        <v>125</v>
+      </c>
       <c r="C55" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D55" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D55" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E55" s="34" t="inlineStr">
@@ -8386,7 +8444,7 @@
       </c>
       <c r="F55" s="34" t="inlineStr">
         <is>
-          <t>Victory Lap Radio x Nike Air Force 1 Low</t>
+          <t>Oregon Ducks Nike Air Force 1 Low 2026</t>
         </is>
       </c>
     </row>
@@ -8409,12 +8467,12 @@
       </c>
       <c r="E56" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F56" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 3 “Santa”</t>
+          <t>Nike Kobe AD Protro “Purple Stardust” 2026</t>
         </is>
       </c>
     </row>
@@ -8423,7 +8481,7 @@
         <v>46353</v>
       </c>
       <c r="B57" s="37" t="n">
-        <v>240</v>
+        <v>230</v>
       </c>
       <c r="C57" s="36" t="inlineStr">
         <is>
@@ -8437,12 +8495,12 @@
       </c>
       <c r="E57" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F57" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
+          <t>Air Jordan 4 “Bred” 2026</t>
         </is>
       </c>
     </row>
@@ -8451,7 +8509,7 @@
         <v>46353</v>
       </c>
       <c r="B58" s="40" t="n">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="C58" s="39" t="inlineStr">
         <is>
@@ -8465,12 +8523,12 @@
       </c>
       <c r="E58" s="30" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F58" s="30" t="inlineStr">
         <is>
-          <t>Air Jordan 4 “Bred” 2026</t>
+          <t>Nike Air Foamposite Pro “Dr. Doom”</t>
         </is>
       </c>
     </row>
@@ -8486,7 +8544,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D59" s="53" t="inlineStr">
+      <c r="D59" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8594,7 +8652,7 @@
           <t>EXTREME</t>
         </is>
       </c>
-      <c r="D63" s="53" t="inlineStr">
+      <c r="D63" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8753,26 +8811,26 @@
         <v>46367</v>
       </c>
       <c r="B69" s="37" t="n">
-        <v>150</v>
+        <v>240</v>
       </c>
       <c r="C69" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D69" s="53" t="inlineStr">
-        <is>
-          <t>SNKRS App</t>
+      <c r="D69" s="38" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
         </is>
       </c>
       <c r="E69" s="34" t="inlineStr">
         <is>
-          <t>Jordan</t>
+          <t>Nike</t>
         </is>
       </c>
       <c r="F69" s="34" t="inlineStr">
         <is>
-          <t>JAIDE x Air Jordan 1 Low OG</t>
+          <t>Nike Air Foamposite One “Floral” 2026</t>
         </is>
       </c>
     </row>
@@ -8780,7 +8838,9 @@
       <c r="A70" s="31" t="n">
         <v>46367</v>
       </c>
-      <c r="B70" s="40" t="inlineStr"/>
+      <c r="B70" s="40" t="n">
+        <v>150</v>
+      </c>
       <c r="C70" s="39" t="inlineStr">
         <is>
           <t>HIGH</t>
@@ -8798,7 +8858,7 @@
       </c>
       <c r="F70" s="30" t="inlineStr">
         <is>
-          <t>Free The Youth x Air Jordan 3</t>
+          <t>JAIDE x Air Jordan 1 Low OG</t>
         </is>
       </c>
     </row>
@@ -8806,27 +8866,25 @@
       <c r="A71" s="35" t="n">
         <v>46367</v>
       </c>
-      <c r="B71" s="37" t="n">
-        <v>240</v>
-      </c>
+      <c r="B71" s="37" t="inlineStr"/>
       <c r="C71" s="36" t="inlineStr">
         <is>
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D71" s="38" t="inlineStr">
-        <is>
-          <t>Online + Retail</t>
+      <c r="D71" s="52" t="inlineStr">
+        <is>
+          <t>SNKRS App</t>
         </is>
       </c>
       <c r="E71" s="34" t="inlineStr">
         <is>
-          <t>Nike</t>
+          <t>Jordan</t>
         </is>
       </c>
       <c r="F71" s="34" t="inlineStr">
         <is>
-          <t>Nike Air Foamposite One “Floral” 2026</t>
+          <t>Free The Youth x Air Jordan 3</t>
         </is>
       </c>
     </row>
@@ -8870,7 +8928,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D73" s="53" t="inlineStr">
+      <c r="D73" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -8982,7 +9040,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D77" s="53" t="inlineStr">
+      <c r="D77" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -9038,7 +9096,7 @@
           <t>HIGH</t>
         </is>
       </c>
-      <c r="D79" s="53" t="inlineStr">
+      <c r="D79" s="52" t="inlineStr">
         <is>
           <t>SNKRS App</t>
         </is>
@@ -9110,8 +9168,36 @@
         </is>
       </c>
     </row>
+    <row r="82" ht="15" customHeight="1">
+      <c r="A82" s="31" t="n">
+        <v>46402</v>
+      </c>
+      <c r="B82" s="40" t="n">
+        <v>220</v>
+      </c>
+      <c r="C82" s="39" t="inlineStr">
+        <is>
+          <t>HIGH</t>
+        </is>
+      </c>
+      <c r="D82" s="41" t="inlineStr">
+        <is>
+          <t>Online + Retail</t>
+        </is>
+      </c>
+      <c r="E82" s="30" t="inlineStr">
+        <is>
+          <t>Jordan</t>
+        </is>
+      </c>
+      <c r="F82" s="30" t="inlineStr">
+        <is>
+          <t>Air Jordan 4 “Spotlight”</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:F81"/>
+  <autoFilter ref="A3:F82"/>
   <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A1:F1"/>

</xml_diff>